<commit_message>
ingest: Canadian Standard cost basis confirmed, import unblocked
Albert confirmed the printed price is Titan's cost per unit - no MSRP, no
multiplier - so the file's existing values were already correct and no
reprice is needed. Replaced the COST BASIS UNCONFIRMED assumption note on
all 336 rows with the confirmed statement.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DXeoXeeCbDbxXN7V7sibfF
</commit_message>
<xml_diff>
--- a/ingest/2026-09-03/canadian_standard_airtable_upload_2026-09-03.xlsx
+++ b/ingest/2026-09-03/canadian_standard_airtable_upload_2026-09-03.xlsx
@@ -831,7 +831,7 @@
       </c>
       <c r="BC2" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANENG - Origins - Oak (Arlington) T&amp;G | #CAN.E.O.Arl.6 |  - 6½" x". PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). 'New Arrival'. Species printed only as 'Oak' (origin not stated) - stored verbatim. NOTE: the name 'Origins' is used by two different page-1/page-3 programmes with different specs; Collection kept as printed, distinguish by species/width/finish. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANENG - Origins - Oak (Arlington) T&amp;G | #CAN.E.O.Arl.6 |  - 6½" x". PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). 'New Arrival'. Species printed only as 'Oak' (origin not stated) - stored verbatim. NOTE: the name 'Origins' is used by two different page-1/page-3 programmes with different specs; Collection kept as printed, distinguish by species/width/finish. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF2" t="inlineStr">
@@ -959,7 +959,7 @@
       </c>
       <c r="BC3" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANENG - Origins - Oak (Mckinney) T&amp;G | #CAN.E.O.Mck.6 |  - 6½" x ". PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). 'New Arrival'. Species printed only as 'Oak' (origin not stated) - stored verbatim. NOTE: the name 'Origins' is used by two different page-1/page-3 programmes with different specs; Collection kept as printed, distinguish by species/width/finish. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANENG - Origins - Oak (Mckinney) T&amp;G | #CAN.E.O.Mck.6 |  - 6½" x ". PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). 'New Arrival'. Species printed only as 'Oak' (origin not stated) - stored verbatim. NOTE: the name 'Origins' is used by two different page-1/page-3 programmes with different specs; Collection kept as printed, distinguish by species/width/finish. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF3" t="inlineStr">
@@ -1087,7 +1087,7 @@
       </c>
       <c r="BC4" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANENG - Origins - Oak (Nashville) T&amp;G | #CAN.E.O.Nas.6 |  - 6½" x". PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). 'New Arrival'. Species printed only as 'Oak' (origin not stated) - stored verbatim. NOTE: the name 'Origins' is used by two different page-1/page-3 programmes with different specs; Collection kept as printed, distinguish by species/width/finish. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANENG - Origins - Oak (Nashville) T&amp;G | #CAN.E.O.Nas.6 |  - 6½" x". PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). 'New Arrival'. Species printed only as 'Oak' (origin not stated) - stored verbatim. NOTE: the name 'Origins' is used by two different page-1/page-3 programmes with different specs; Collection kept as printed, distinguish by species/width/finish. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF4" t="inlineStr">
@@ -1215,7 +1215,7 @@
       </c>
       <c r="BC5" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANENG - Origins - Oak (Quincy) T&amp;G | #CAN.E.O.Qui.6 |  - 6½" x ¾"". PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). 'New Arrival'. Species printed only as 'Oak' (origin not stated) - stored verbatim. NOTE: the name 'Origins' is used by two different page-1/page-3 programmes with different specs; Collection kept as printed, distinguish by species/width/finish. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANENG - Origins - Oak (Quincy) T&amp;G | #CAN.E.O.Qui.6 |  - 6½" x ¾"". PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). 'New Arrival'. Species printed only as 'Oak' (origin not stated) - stored verbatim. NOTE: the name 'Origins' is used by two different page-1/page-3 programmes with different specs; Collection kept as printed, distinguish by species/width/finish. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF5" t="inlineStr">
@@ -1343,7 +1343,7 @@
       </c>
       <c r="BC6" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANENG - Origins - Oak (Wrenwood) T&amp;G | #CAN.E.O.Wre.6 |  - 6½" x ". PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). 'New Arrival'. Species printed only as 'Oak' (origin not stated) - stored verbatim. NOTE: the name 'Origins' is used by two different page-1/page-3 programmes with different specs; Collection kept as printed, distinguish by species/width/finish. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANENG - Origins - Oak (Wrenwood) T&amp;G | #CAN.E.O.Wre.6 |  - 6½" x ". PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). 'New Arrival'. Species printed only as 'Oak' (origin not stated) - stored verbatim. NOTE: the name 'Origins' is used by two different page-1/page-3 programmes with different specs; Collection kept as printed, distinguish by species/width/finish. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF6" t="inlineStr">
@@ -1451,7 +1451,7 @@
       </c>
       <c r="BC7" t="inlineStr">
         <is>
-          <t>PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). 'New Arrival'. 9"w x 60"l (228mm x 1520mm) x 9mm. ASSUMPTION: core printed only as '9mm Vinyl' - Material type set to SPC core as the schema's default for unlabelled rigid vinyl; WPC not named anywhere. Confirm with supplier. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). 'New Arrival'. 9"w x 60"l (228mm x 1520mm) x 9mm. ASSUMPTION: core printed only as '9mm Vinyl' - Material type set to SPC core as the schema's default for unlabelled rigid vinyl; WPC not named anywhere. Confirm with supplier. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF7" t="inlineStr">
@@ -1559,7 +1559,7 @@
       </c>
       <c r="BC8" t="inlineStr">
         <is>
-          <t>PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). 'New Arrival'. 9"w x 60"l (228mm x 1520mm) x 9mm. ASSUMPTION: core printed only as '9mm Vinyl' - Material type set to SPC core as the schema's default for unlabelled rigid vinyl; WPC not named anywhere. Confirm with supplier. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). 'New Arrival'. 9"w x 60"l (228mm x 1520mm) x 9mm. ASSUMPTION: core printed only as '9mm Vinyl' - Material type set to SPC core as the schema's default for unlabelled rigid vinyl; WPC not named anywhere. Confirm with supplier. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF8" t="inlineStr">
@@ -1667,7 +1667,7 @@
       </c>
       <c r="BC9" t="inlineStr">
         <is>
-          <t>PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). 'New Arrival'. 9"w x 60"l (228mm x 1520mm) x 9mm. ASSUMPTION: core printed only as '9mm Vinyl' - Material type set to SPC core as the schema's default for unlabelled rigid vinyl; WPC not named anywhere. Confirm with supplier. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). 'New Arrival'. 9"w x 60"l (228mm x 1520mm) x 9mm. ASSUMPTION: core printed only as '9mm Vinyl' - Material type set to SPC core as the schema's default for unlabelled rigid vinyl; WPC not named anywhere. Confirm with supplier. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF9" t="inlineStr">
@@ -1775,7 +1775,7 @@
       </c>
       <c r="BC10" t="inlineStr">
         <is>
-          <t>PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). 'New Arrival'. 9"w x 60"l (228mm x 1520mm) x 9mm. ASSUMPTION: core printed only as '9mm Vinyl' - Material type set to SPC core as the schema's default for unlabelled rigid vinyl; WPC not named anywhere. Confirm with supplier. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). 'New Arrival'. 9"w x 60"l (228mm x 1520mm) x 9mm. ASSUMPTION: core printed only as '9mm Vinyl' - Material type set to SPC core as the schema's default for unlabelled rigid vinyl; WPC not named anywhere. Confirm with supplier. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF10" t="inlineStr">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="BC11" t="inlineStr">
         <is>
-          <t>PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). 'New Arrival'. 9"w x 60"l (228mm x 1520mm) x 9mm. ASSUMPTION: core printed only as '9mm Vinyl' - Material type set to SPC core as the schema's default for unlabelled rigid vinyl; WPC not named anywhere. Confirm with supplier. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). 'New Arrival'. 9"w x 60"l (228mm x 1520mm) x 9mm. ASSUMPTION: core printed only as '9mm Vinyl' - Material type set to SPC core as the schema's default for unlabelled rigid vinyl; WPC not named anywhere. Confirm with supplier. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF11" t="inlineStr">
@@ -1991,7 +1991,7 @@
       </c>
       <c r="BC12" t="inlineStr">
         <is>
-          <t>PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). 'New Arrival'. 9"w x 60"l (228mm x 1520mm) x 9mm. ASSUMPTION: core printed only as '9mm Vinyl' - Material type set to SPC core as the schema's default for unlabelled rigid vinyl; WPC not named anywhere. Confirm with supplier. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). 'New Arrival'. 9"w x 60"l (228mm x 1520mm) x 9mm. ASSUMPTION: core printed only as '9mm Vinyl' - Material type set to SPC core as the schema's default for unlabelled rigid vinyl; WPC not named anywhere. Confirm with supplier. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF12" t="inlineStr">
@@ -2099,7 +2099,7 @@
       </c>
       <c r="BC13" t="inlineStr">
         <is>
-          <t>PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). 'New Arrival'. 9"w x 60"l (228mm x 1520mm) x 9mm. ASSUMPTION: core printed only as '9mm Vinyl' - Material type set to SPC core as the schema's default for unlabelled rigid vinyl; WPC not named anywhere. Confirm with supplier. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). 'New Arrival'. 9"w x 60"l (228mm x 1520mm) x 9mm. ASSUMPTION: core printed only as '9mm Vinyl' - Material type set to SPC core as the schema's default for unlabelled rigid vinyl; WPC not named anywhere. Confirm with supplier. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF13" t="inlineStr">
@@ -2207,7 +2207,7 @@
       </c>
       <c r="BC14" t="inlineStr">
         <is>
-          <t>PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). 'New Arrival'. 9"w x 60"l (228mm x 1520mm) x 9mm. ASSUMPTION: core printed only as '9mm Vinyl' - Material type set to SPC core as the schema's default for unlabelled rigid vinyl; WPC not named anywhere. Confirm with supplier. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). 'New Arrival'. 9"w x 60"l (228mm x 1520mm) x 9mm. ASSUMPTION: core printed only as '9mm Vinyl' - Material type set to SPC core as the schema's default for unlabelled rigid vinyl; WPC not named anywhere. Confirm with supplier. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF14" t="inlineStr">
@@ -2285,7 +2285,7 @@
       </c>
       <c r="BC15" t="inlineStr">
         <is>
-          <t>Per-piece trim, 2400mm x 45mm x 10mm. Cross-supplier accessory markup applied (T-Moulding/Reducer +$10, Stair Nose +$15) -&gt; Retail $28.00/pc. Supplier: 'Due to the fragile nature of this product, all sales are final. No Returns or Exchanges.' Sheet groups 'T Moulding / Reducer' under one $18.00 price and 'Stair Nose' at $22.00. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>Per-piece trim, 2400mm x 45mm x 10mm. Cross-supplier accessory markup applied (T-Moulding/Reducer +$10, Stair Nose +$15) -&gt; Retail $28.00/pc. Supplier: 'Due to the fragile nature of this product, all sales are final. No Returns or Exchanges.' Sheet groups 'T Moulding / Reducer' under one $18.00 price and 'Stair Nose' at $22.00. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF15" t="inlineStr">
@@ -2363,7 +2363,7 @@
       </c>
       <c r="BC16" t="inlineStr">
         <is>
-          <t>Per-piece trim, 2400mm x 45mm x 12mm. Cross-supplier accessory markup applied (T-Moulding/Reducer +$10, Stair Nose +$15) -&gt; Retail $28.00/pc. Supplier: 'Due to the fragile nature of this product, all sales are final. No Returns or Exchanges.' Sheet groups 'T Moulding / Reducer' under one $18.00 price and 'Stair Nose' at $22.00. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>Per-piece trim, 2400mm x 45mm x 12mm. Cross-supplier accessory markup applied (T-Moulding/Reducer +$10, Stair Nose +$15) -&gt; Retail $28.00/pc. Supplier: 'Due to the fragile nature of this product, all sales are final. No Returns or Exchanges.' Sheet groups 'T Moulding / Reducer' under one $18.00 price and 'Stair Nose' at $22.00. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF16" t="inlineStr">
@@ -2441,7 +2441,7 @@
       </c>
       <c r="BC17" t="inlineStr">
         <is>
-          <t>Per-piece trim, 2400mm x 115mm x 24mm. Cross-supplier accessory markup applied (T-Moulding/Reducer +$10, Stair Nose +$15) -&gt; Retail $37.00/pc. Supplier: 'Due to the fragile nature of this product, all sales are final. No Returns or Exchanges.' Sheet groups 'T Moulding / Reducer' under one $18.00 price and 'Stair Nose' at $22.00. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>Per-piece trim, 2400mm x 115mm x 24mm. Cross-supplier accessory markup applied (T-Moulding/Reducer +$10, Stair Nose +$15) -&gt; Retail $37.00/pc. Supplier: 'Due to the fragile nature of this product, all sales are final. No Returns or Exchanges.' Sheet groups 'T Moulding / Reducer' under one $18.00 price and 'Stair Nose' at $22.00. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF17" t="inlineStr">
@@ -2549,7 +2549,7 @@
       </c>
       <c r="BC18" t="inlineStr">
         <is>
-          <t>PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). 'New Arrival'. 9.29" x 59.76" (236mm x 1518mm). Supplier calls the line 'Waterproof Collection - 12mm Laminate' -&gt; Material type = Water-Resistant Core, Waterproof = TRUE. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). 'New Arrival'. 9.29" x 59.76" (236mm x 1518mm). Supplier calls the line 'Waterproof Collection - 12mm Laminate' -&gt; Material type = Water-Resistant Core, Waterproof = TRUE. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF18" t="inlineStr">
@@ -2657,7 +2657,7 @@
       </c>
       <c r="BC19" t="inlineStr">
         <is>
-          <t>PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). 'New Arrival'. 9.29" x 59.76" (236mm x 1518mm). Supplier calls the line 'Waterproof Collection - 12mm Laminate' -&gt; Material type = Water-Resistant Core, Waterproof = TRUE. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). 'New Arrival'. 9.29" x 59.76" (236mm x 1518mm). Supplier calls the line 'Waterproof Collection - 12mm Laminate' -&gt; Material type = Water-Resistant Core, Waterproof = TRUE. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF19" t="inlineStr">
@@ -2765,7 +2765,7 @@
       </c>
       <c r="BC20" t="inlineStr">
         <is>
-          <t>PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). 'New Arrival'. 9.29" x 59.76" (236mm x 1518mm). Supplier calls the line 'Waterproof Collection - 12mm Laminate' -&gt; Material type = Water-Resistant Core, Waterproof = TRUE. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). 'New Arrival'. 9.29" x 59.76" (236mm x 1518mm). Supplier calls the line 'Waterproof Collection - 12mm Laminate' -&gt; Material type = Water-Resistant Core, Waterproof = TRUE. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF20" t="inlineStr">
@@ -2873,7 +2873,7 @@
       </c>
       <c r="BC21" t="inlineStr">
         <is>
-          <t>PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). 'New Arrival'. 9.29" x 59.76" (236mm x 1518mm). Supplier calls the line 'Waterproof Collection - 12mm Laminate' -&gt; Material type = Water-Resistant Core, Waterproof = TRUE. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). 'New Arrival'. 9.29" x 59.76" (236mm x 1518mm). Supplier calls the line 'Waterproof Collection - 12mm Laminate' -&gt; Material type = Water-Resistant Core, Waterproof = TRUE. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF21" t="inlineStr">
@@ -2981,7 +2981,7 @@
       </c>
       <c r="BC22" t="inlineStr">
         <is>
-          <t>PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). 'New Arrival'. 9.29" x 59.76" (236mm x 1518mm). Supplier calls the line 'Waterproof Collection - 12mm Laminate' -&gt; Material type = Water-Resistant Core, Waterproof = TRUE. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). 'New Arrival'. 9.29" x 59.76" (236mm x 1518mm). Supplier calls the line 'Waterproof Collection - 12mm Laminate' -&gt; Material type = Water-Resistant Core, Waterproof = TRUE. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF22" t="inlineStr">
@@ -3089,7 +3089,7 @@
       </c>
       <c r="BC23" t="inlineStr">
         <is>
-          <t>PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). 'New Arrival'. 9.29" x 59.76" (236mm x 1518mm). Supplier calls the line 'Waterproof Collection - 12mm Laminate' -&gt; Material type = Water-Resistant Core, Waterproof = TRUE. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). 'New Arrival'. 9.29" x 59.76" (236mm x 1518mm). Supplier calls the line 'Waterproof Collection - 12mm Laminate' -&gt; Material type = Water-Resistant Core, Waterproof = TRUE. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF23" t="inlineStr">
@@ -3197,7 +3197,7 @@
       </c>
       <c r="BC24" t="inlineStr">
         <is>
-          <t>PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). 'New Arrival'. 9.29" x 59.76" (236mm x 1518mm). Supplier calls the line 'Waterproof Collection - 12mm Laminate' -&gt; Material type = Water-Resistant Core, Waterproof = TRUE. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). 'New Arrival'. 9.29" x 59.76" (236mm x 1518mm). Supplier calls the line 'Waterproof Collection - 12mm Laminate' -&gt; Material type = Water-Resistant Core, Waterproof = TRUE. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF24" t="inlineStr">
@@ -3310,7 +3310,7 @@
       </c>
       <c r="BC25" t="inlineStr">
         <is>
-          <t>PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). 'New Arrival'. 165mm x 800mm herringbone block; Width (in) 6.5 converted from 165mm. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). 'New Arrival'. 165mm x 800mm herringbone block; Width (in) 6.5 converted from 165mm. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF25" t="inlineStr">
@@ -3388,7 +3388,7 @@
       </c>
       <c r="BC26" t="inlineStr">
         <is>
-          <t>Per-piece trim, 2400mm x 45mm x 10mm. Cross-supplier accessory markup applied (T-Moulding/Reducer +$10, Stair Nose +$15) -&gt; Retail $28.00/pc. Supplier: 'Due to the fragile nature of this product, all sales are final. No Returns or Exchanges.' Sheet groups 'T Moulding / Reducer' under one $18.00 price and 'Stair Nose' at $22.00. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>Per-piece trim, 2400mm x 45mm x 10mm. Cross-supplier accessory markup applied (T-Moulding/Reducer +$10, Stair Nose +$15) -&gt; Retail $28.00/pc. Supplier: 'Due to the fragile nature of this product, all sales are final. No Returns or Exchanges.' Sheet groups 'T Moulding / Reducer' under one $18.00 price and 'Stair Nose' at $22.00. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF26" t="inlineStr">
@@ -3466,7 +3466,7 @@
       </c>
       <c r="BC27" t="inlineStr">
         <is>
-          <t>Per-piece trim, 2400mm x 45mm x 12mm. Cross-supplier accessory markup applied (T-Moulding/Reducer +$10, Stair Nose +$15) -&gt; Retail $28.00/pc. Supplier: 'Due to the fragile nature of this product, all sales are final. No Returns or Exchanges.' Sheet groups 'T Moulding / Reducer' under one $18.00 price and 'Stair Nose' at $22.00. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>Per-piece trim, 2400mm x 45mm x 12mm. Cross-supplier accessory markup applied (T-Moulding/Reducer +$10, Stair Nose +$15) -&gt; Retail $28.00/pc. Supplier: 'Due to the fragile nature of this product, all sales are final. No Returns or Exchanges.' Sheet groups 'T Moulding / Reducer' under one $18.00 price and 'Stair Nose' at $22.00. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF27" t="inlineStr">
@@ -3544,7 +3544,7 @@
       </c>
       <c r="BC28" t="inlineStr">
         <is>
-          <t>Per-piece trim, 2400mm x 115mm x 24mm. Cross-supplier accessory markup applied (T-Moulding/Reducer +$10, Stair Nose +$15) -&gt; Retail $37.00/pc. Supplier: 'Due to the fragile nature of this product, all sales are final. No Returns or Exchanges.' Sheet groups 'T Moulding / Reducer' under one $18.00 price and 'Stair Nose' at $22.00. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>Per-piece trim, 2400mm x 115mm x 24mm. Cross-supplier accessory markup applied (T-Moulding/Reducer +$10, Stair Nose +$15) -&gt; Retail $37.00/pc. Supplier: 'Due to the fragile nature of this product, all sales are final. No Returns or Exchanges.' Sheet groups 'T Moulding / Reducer' under one $18.00 price and 'Stair Nose' at $22.00. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF28" t="inlineStr">
@@ -3659,7 +3659,7 @@
       </c>
       <c r="BC29" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANENG - LUCID 6" PLANKS - Oak (Calm)  | #CAN.E.O.Cal.6 |  - 6½" x". PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). 'New Arrival'. 6.5" x 3/4" x RL. Sheet prints 'Amercian Oak' (supplier typo) -&gt; Species stored as American Oak. Install profile not stated on this page - left blank. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANENG - LUCID 6" PLANKS - Oak (Calm)  | #CAN.E.O.Cal.6 |  - 6½" x". PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). 'New Arrival'. 6.5" x 3/4" x RL. Sheet prints 'Amercian Oak' (supplier typo) -&gt; Species stored as American Oak. Install profile not stated on this page - left blank. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF29" t="inlineStr">
@@ -3774,7 +3774,7 @@
       </c>
       <c r="BC30" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANENG - LUCID 6" PLANKS - Oak (Enhance)  | #CAN.E.O.Enh.6 |  - 6½". PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). 'New Arrival'. 6.5" x 3/4" x RL. Sheet prints 'Amercian Oak' (supplier typo) -&gt; Species stored as American Oak. Install profile not stated on this page - left blank. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANENG - LUCID 6" PLANKS - Oak (Enhance)  | #CAN.E.O.Enh.6 |  - 6½". PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). 'New Arrival'. 6.5" x 3/4" x RL. Sheet prints 'Amercian Oak' (supplier typo) -&gt; Species stored as American Oak. Install profile not stated on this page - left blank. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF30" t="inlineStr">
@@ -3889,7 +3889,7 @@
       </c>
       <c r="BC31" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANENG - LUCID 6" PLANKS - Oak (Senses)  | #CAN.E.O.Sen.6 |  - 6½"". PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). 'New Arrival'. 6.5" x 3/4" x RL. Sheet prints 'Amercian Oak' (supplier typo) -&gt; Species stored as American Oak. Install profile not stated on this page - left blank. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANENG - LUCID 6" PLANKS - Oak (Senses)  | #CAN.E.O.Sen.6 |  - 6½"". PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). 'New Arrival'. 6.5" x 3/4" x RL. Sheet prints 'Amercian Oak' (supplier typo) -&gt; Species stored as American Oak. Install profile not stated on this page - left blank. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF31" t="inlineStr">
@@ -4009,7 +4009,7 @@
       </c>
       <c r="BC32" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANENG - LUCID 6" HERRINGBONE - Oak (Soothe)  | #CAN.E.O.Soo.5 |  ". PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). 'New Arrival'. 5" x 3/4" x 24". Sheet prints 'Amercian Oak' (supplier typo) -&gt; Species stored as American Oak. Install profile not stated on this page - left blank. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANENG - LUCID 6" HERRINGBONE - Oak (Soothe)  | #CAN.E.O.Soo.5 |  ". PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). 'New Arrival'. 5" x 3/4" x 24". Sheet prints 'Amercian Oak' (supplier typo) -&gt; Species stored as American Oak. Install profile not stated on this page - left blank. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF32" t="inlineStr">
@@ -4129,7 +4129,7 @@
       </c>
       <c r="BC33" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANENG - LUCID 6" HERRINGBONE - Oak (Tranquil)  | #CAN.E.O.Tra.5 |". PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). 'New Arrival'. 5" x 3/4" x 24". Sheet prints 'Amercian Oak' (supplier typo) -&gt; Species stored as American Oak. Install profile not stated on this page - left blank. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANENG - LUCID 6" HERRINGBONE - Oak (Tranquil)  | #CAN.E.O.Tra.5 |". PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). 'New Arrival'. 5" x 3/4" x 24". Sheet prints 'Amercian Oak' (supplier typo) -&gt; Species stored as American Oak. Install profile not stated on this page - left blank. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF33" t="inlineStr">
@@ -4244,7 +4244,7 @@
       </c>
       <c r="BC34" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANENG - LUCID 7" PLANKS - Oak (Bare)  | #CAN.E.O.Bar.7 |  - 7½" x". PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). 'New Arrival'. 7.5" x 3/4" x RL. Sheet prints 'Amercian Oak' (supplier typo) -&gt; Species stored as American Oak. Install profile not stated on this page - left blank. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANENG - LUCID 7" PLANKS - Oak (Bare)  | #CAN.E.O.Bar.7 |  - 7½" x". PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). 'New Arrival'. 7.5" x 3/4" x RL. Sheet prints 'Amercian Oak' (supplier typo) -&gt; Species stored as American Oak. Install profile not stated on this page - left blank. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF34" t="inlineStr">
@@ -4359,7 +4359,7 @@
       </c>
       <c r="BC35" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANENG - LUCID 7" PLANKS - Oak (Essence)  | #CAN.E.O.Ess.7 |  - 7½". PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). 'New Arrival'. 7.5" x 3/4" x RL. Sheet prints 'Amercian Oak' (supplier typo) -&gt; Species stored as American Oak. Install profile not stated on this page - left blank. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANENG - LUCID 7" PLANKS - Oak (Essence)  | #CAN.E.O.Ess.7 |  - 7½". PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). 'New Arrival'. 7.5" x 3/4" x RL. Sheet prints 'Amercian Oak' (supplier typo) -&gt; Species stored as American Oak. Install profile not stated on this page - left blank. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF35" t="inlineStr">
@@ -4474,7 +4474,7 @@
       </c>
       <c r="BC36" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANENG - LUCID 7" PLANKS - Oak (Nature)  | #CAN.E.O.Nat.7 |  - 7½"". PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). 'New Arrival'. 7.5" x 3/4" x RL. Sheet prints 'Amercian Oak' (supplier typo) -&gt; Species stored as American Oak. Install profile not stated on this page - left blank. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANENG - LUCID 7" PLANKS - Oak (Nature)  | #CAN.E.O.Nat.7 |  - 7½"". PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). 'New Arrival'. 7.5" x 3/4" x RL. Sheet prints 'Amercian Oak' (supplier typo) -&gt; Species stored as American Oak. Install profile not stated on this page - left blank. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF36" t="inlineStr">
@@ -4594,7 +4594,7 @@
       </c>
       <c r="BC37" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANENG - LUCID 7" HERRINGBONE - Oak (Pristine)  | #CAN.E.O.Pri.6 |". PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). 'New Arrival'. 6" x 3/4" x 36". Sheet prints 'Amercian Oak' (supplier typo) -&gt; Species stored as American Oak. Install profile not stated on this page - left blank. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANENG - LUCID 7" HERRINGBONE - Oak (Pristine)  | #CAN.E.O.Pri.6 |". PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). 'New Arrival'. 6" x 3/4" x 36". Sheet prints 'Amercian Oak' (supplier typo) -&gt; Species stored as American Oak. Install profile not stated on this page - left blank. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF37" t="inlineStr">
@@ -4714,7 +4714,7 @@
       </c>
       <c r="BC38" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANENG - LUCID 7" HERRINGBONE - Oak (Pure)  | #CAN.E.O.Pur.6 |  - ". PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). 'New Arrival'. 6" x 3/4" x 36". Sheet prints 'Amercian Oak' (supplier typo) -&gt; Species stored as American Oak. Install profile not stated on this page - left blank. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANENG - LUCID 7" HERRINGBONE - Oak (Pure)  | #CAN.E.O.Pur.6 |  - ". PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). 'New Arrival'. 6" x 3/4" x 36". Sheet prints 'Amercian Oak' (supplier typo) -&gt; Species stored as American Oak. Install profile not stated on this page - left blank. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF38" t="inlineStr">
@@ -4821,7 +4821,7 @@
       </c>
       <c r="BC39" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - NOVELLA - Hickory (Lewis)  | #CAN.E.H.Lew.7 |  - 7½" x ¾" x R". 'New Arrival'. 7.5" x 3/4" x RL (16"-83"). Sheet prints 'Amercian Hickory' (supplier typo). COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - NOVELLA - Hickory (Lewis)  | #CAN.E.H.Lew.7 |  - 7½" x ¾" x R". 'New Arrival'. 7.5" x 3/4" x RL (16"-83"). Sheet prints 'Amercian Hickory' (supplier typo). COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF39" t="inlineStr">
@@ -4928,7 +4928,7 @@
       </c>
       <c r="BC40" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - NOVELLA - Hickory (Twain)  | #CAN.E.H.Twa.7 |  - 7½" x ¾" x R". 'New Arrival'. 7.5" x 3/4" x RL (16"-83"). Sheet prints 'Amercian Hickory' (supplier typo). COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - NOVELLA - Hickory (Twain)  | #CAN.E.H.Twa.7 |  - 7½" x ¾" x R". 'New Arrival'. 7.5" x 3/4" x RL (16"-83"). Sheet prints 'Amercian Hickory' (supplier typo). COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF40" t="inlineStr">
@@ -5035,7 +5035,7 @@
       </c>
       <c r="BC41" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - NOVELLA - Hickory (Tolkein)  | #CAN.E.H.Tol.7 |  - 7½" x ¾" x". 'New Arrival'. 7.5" x 3/4" x RL (16"-83"). Sheet prints 'Amercian Hickory' (supplier typo). COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - NOVELLA - Hickory (Tolkein)  | #CAN.E.H.Tol.7 |  - 7½" x ¾" x". 'New Arrival'. 7.5" x 3/4" x RL (16"-83"). Sheet prints 'Amercian Hickory' (supplier typo). COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF41" t="inlineStr">
@@ -5137,7 +5137,7 @@
       </c>
       <c r="BC42" t="inlineStr">
         <is>
-          <t>'New Arrival'. 7.5" x 3/4" x RL (16"-83"). Sheet prints 'Amercian Hickory' (supplier typo). COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>'New Arrival'. 7.5" x 3/4" x RL (16"-83"). Sheet prints 'Amercian Hickory' (supplier typo). COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF42" t="inlineStr">
@@ -5239,7 +5239,7 @@
       </c>
       <c r="BC43" t="inlineStr">
         <is>
-          <t>'New Arrival'. 7.5" x 3/4" x RL (16"-83"). Sheet prints 'Amercian Hickory' (supplier typo). COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>'New Arrival'. 7.5" x 3/4" x RL (16"-83"). Sheet prints 'Amercian Hickory' (supplier typo). COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF43" t="inlineStr">
@@ -5341,7 +5341,7 @@
       </c>
       <c r="BC44" t="inlineStr">
         <is>
-          <t>'New Arrival'. 7.5" x 3/4" x RL (16"-83"). Sheet prints 'Amercian Hickory' (supplier typo). COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>'New Arrival'. 7.5" x 3/4" x RL (16"-83"). Sheet prints 'Amercian Hickory' (supplier typo). COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF44" t="inlineStr">
@@ -5458,7 +5458,7 @@
       </c>
       <c r="BC45" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - NOVELLA - American Oak (Alcott) T&amp;G | #CAN.E.H.Alc.6 |  - 6½"". T&amp;G Engineered. 6.5" x 3/4" x RL (16"-71"). Species printed only as 'Oak'. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - NOVELLA - American Oak (Alcott) T&amp;G | #CAN.E.H.Alc.6 |  - 6½"". T&amp;G Engineered. 6.5" x 3/4" x RL (16"-71"). Species printed only as 'Oak'. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF45" t="inlineStr">
@@ -5575,7 +5575,7 @@
       </c>
       <c r="BC46" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - NOVELLA - American Oak (Atwood) T&amp;G | #CAN.E.H.Atw.6 |  - 6½"". T&amp;G Engineered. 6.5" x 3/4" x RL (16"-71"). Species printed only as 'Oak'. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - NOVELLA - American Oak (Atwood) T&amp;G | #CAN.E.H.Atw.6 |  - 6½"". T&amp;G Engineered. 6.5" x 3/4" x RL (16"-71"). Species printed only as 'Oak'. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF46" t="inlineStr">
@@ -5692,7 +5692,7 @@
       </c>
       <c r="BC47" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - NOVELLA - American Oak (Austen) T&amp;G | #CAN.E.H.Aus.6 |  - 6½"". T&amp;G Engineered. 6.5" x 3/4" x RL (16"-71"). Species printed only as 'Oak'. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - NOVELLA - American Oak (Austen) T&amp;G | #CAN.E.H.Aus.6 |  - 6½"". T&amp;G Engineered. 6.5" x 3/4" x RL (16"-71"). Species printed only as 'Oak'. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF47" t="inlineStr">
@@ -5809,7 +5809,7 @@
       </c>
       <c r="BC48" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - NOVELLA - American Oak (Rowling) T&amp;G | #CAN.E.H.Row.6 |  - 6½". T&amp;G Engineered. 6.5" x 3/4" x RL (16"-71"). Species printed only as 'Oak'. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - NOVELLA - American Oak (Rowling) T&amp;G | #CAN.E.H.Row.6 |  - 6½". T&amp;G Engineered. 6.5" x 3/4" x RL (16"-71"). Species printed only as 'Oak'. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF48" t="inlineStr">
@@ -5926,7 +5926,7 @@
       </c>
       <c r="BC49" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - NOVELLA - American Oak (Woolf) T&amp;G | #CAN.E.H.Woo.6 |  - 6½" ". T&amp;G Engineered. 6.5" x 3/4" x RL (16"-71"). Species printed only as 'Oak'. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - NOVELLA - American Oak (Woolf) T&amp;G | #CAN.E.H.Woo.6 |  - 6½" ". T&amp;G Engineered. 6.5" x 3/4" x RL (16"-71"). Species printed only as 'Oak'. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF49" t="inlineStr">
@@ -6043,7 +6043,7 @@
       </c>
       <c r="BC50" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - NOVELLA - Hickory (Dickens) T&amp;G | #CAN.E.O.Dic.6 |  - 6½" x ¾". T&amp;G Engineered. 6.5" x 3/4" x RL (16"-75"). COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - NOVELLA - Hickory (Dickens) T&amp;G | #CAN.E.O.Dic.6 |  - 6½" x ¾". T&amp;G Engineered. 6.5" x 3/4" x RL (16"-75"). COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF50" t="inlineStr">
@@ -6160,7 +6160,7 @@
       </c>
       <c r="BC51" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - NOVELLA - Hickory (Fitzgerald) T&amp;G | #CAN.E.O.Fit.6 |  - 6½" ". T&amp;G Engineered. 6.5" x 3/4" x RL (16"-75"). COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - NOVELLA - Hickory (Fitzgerald) T&amp;G | #CAN.E.O.Fit.6 |  - 6½" ". T&amp;G Engineered. 6.5" x 3/4" x RL (16"-75"). COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF51" t="inlineStr">
@@ -6277,7 +6277,7 @@
       </c>
       <c r="BC52" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - NOVELLA - Hickory (Hemingway) T&amp;G | #CAN.E.O.Hem.6 |  - 6½" x". T&amp;G Engineered. 6.5" x 3/4" x RL (16"-75"). COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - NOVELLA - Hickory (Hemingway) T&amp;G | #CAN.E.O.Hem.6 |  - 6½" x". T&amp;G Engineered. 6.5" x 3/4" x RL (16"-75"). COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF52" t="inlineStr">
@@ -6394,7 +6394,7 @@
       </c>
       <c r="BC53" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - NOVELLA - Hickory (Orwell) T&amp;G | #CAN.E.O.Orw.6 |  - 6½" x ¾"". T&amp;G Engineered. 6.5" x 3/4" x RL (16"-75"). COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - NOVELLA - Hickory (Orwell) T&amp;G | #CAN.E.O.Orw.6 |  - 6½" x ¾"". T&amp;G Engineered. 6.5" x 3/4" x RL (16"-75"). COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF53" t="inlineStr">
@@ -6511,7 +6511,7 @@
       </c>
       <c r="BC54" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - NOVELLA - Hickory (Steinbeck) T&amp;G | #CAN.E.O.Ste.6 |  - 6½" x". T&amp;G Engineered. 6.5" x 3/4" x RL (16"-75"). COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - NOVELLA - Hickory (Steinbeck) T&amp;G | #CAN.E.O.Ste.6 |  - 6½" x". T&amp;G Engineered. 6.5" x 3/4" x RL (16"-75"). COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF54" t="inlineStr">
@@ -6628,7 +6628,7 @@
       </c>
       <c r="BC55" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Origins XL - Oak (Carissa) T&amp;G | #CAN.E.O.Car.7 |  - 7½" x ¾"". T&amp;G Engineered, 20"-83" random length, 4 Sided Micro Bevel. ORIGINS XL carries NO promotion header - single price only. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Origins XL - Oak (Carissa) T&amp;G | #CAN.E.O.Car.7 |  - 7½" x ¾"". T&amp;G Engineered, 20"-83" random length, 4 Sided Micro Bevel. ORIGINS XL carries NO promotion header - single price only. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF55" t="inlineStr">
@@ -6745,7 +6745,7 @@
       </c>
       <c r="BC56" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Origins XL - Oak (Geraldine) T&amp;G | #CAN.E.O.Ger.7 |  - 7½" x ". T&amp;G Engineered, 20"-83" random length, 4 Sided Micro Bevel. ORIGINS XL carries NO promotion header - single price only. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Origins XL - Oak (Geraldine) T&amp;G | #CAN.E.O.Ger.7 |  - 7½" x ". T&amp;G Engineered, 20"-83" random length, 4 Sided Micro Bevel. ORIGINS XL carries NO promotion header - single price only. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF56" t="inlineStr">
@@ -6862,7 +6862,7 @@
       </c>
       <c r="BC57" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Origins XL - Oak (Charleston) T&amp;G | #CAN.E.O.Cha.7 |  - 7½" x". T&amp;G Engineered, 20"-83" random length, 4 Sided Micro Bevel. ORIGINS XL carries NO promotion header - single price only. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Origins XL - Oak (Charleston) T&amp;G | #CAN.E.O.Cha.7 |  - 7½" x". T&amp;G Engineered, 20"-83" random length, 4 Sided Micro Bevel. ORIGINS XL carries NO promotion header - single price only. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF57" t="inlineStr">
@@ -6979,7 +6979,7 @@
       </c>
       <c r="BC58" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Origins XL - Oak (Hudson) T&amp;G | #CAN.E.O.Hud.7 |  - 7½" x ¾" ". T&amp;G Engineered, 20"-83" random length, 4 Sided Micro Bevel. ORIGINS XL carries NO promotion header - single price only. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Origins XL - Oak (Hudson) T&amp;G | #CAN.E.O.Hud.7 |  - 7½" x ¾" ". T&amp;G Engineered, 20"-83" random length, 4 Sided Micro Bevel. ORIGINS XL carries NO promotion header - single price only. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF58" t="inlineStr">
@@ -7096,7 +7096,7 @@
       </c>
       <c r="BC59" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Origins XL - Oak (Maxine) T&amp;G | #CAN.E.O.Max.7 |  - 7½" x ¾" ". T&amp;G Engineered, 20"-83" random length, 4 Sided Micro Bevel. ORIGINS XL carries NO promotion header - single price only. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Origins XL - Oak (Maxine) T&amp;G | #CAN.E.O.Max.7 |  - 7½" x ¾" ". T&amp;G Engineered, 20"-83" random length, 4 Sided Micro Bevel. ORIGINS XL carries NO promotion header - single price only. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF59" t="inlineStr">
@@ -7218,7 +7218,7 @@
       </c>
       <c r="BC60" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Origins XL - Oak (Webster) T&amp;G | #CAN.E.O.Web.7 |  - 7½" x ¾"". T&amp;G Engineered, 20"-83" random length, 4 Sided Micro Bevel. ORIGINS XL carries NO promotion header - single price only. Supplier marks this colour *DISCONTINUE ITEM* on the Aug 31 2026 list -&gt; Stock status = Discontinued, Active = FALSE. Confirm remaining stock before import. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Origins XL - Oak (Webster) T&amp;G | #CAN.E.O.Web.7 |  - 7½" x ¾"". T&amp;G Engineered, 20"-83" random length, 4 Sided Micro Bevel. ORIGINS XL carries NO promotion header - single price only. Supplier marks this colour *DISCONTINUE ITEM* on the Aug 31 2026 list -&gt; Stock status = Discontinued, Active = FALSE. Confirm remaining stock before import. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF60" t="inlineStr">
@@ -7335,7 +7335,7 @@
       </c>
       <c r="BC61" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Origins XL - Hickory (Barrymore) T&amp;G | #CAN.E.H.Bar.7 |  - 7½". T&amp;G Engineered, 20"-83" random length, 4 Sided Micro Bevel. ORIGINS XL carries NO promotion header - single price only. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Origins XL - Hickory (Barrymore) T&amp;G | #CAN.E.H.Bar.7 |  - 7½". T&amp;G Engineered, 20"-83" random length, 4 Sided Micro Bevel. ORIGINS XL carries NO promotion header - single price only. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF61" t="inlineStr">
@@ -7452,7 +7452,7 @@
       </c>
       <c r="BC62" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Origins XL - Hickory (Chesterfield) T&amp;G | #CAN.E.H.Che.7 |  -". T&amp;G Engineered, 20"-83" random length, 4 Sided Micro Bevel. ORIGINS XL carries NO promotion header - single price only. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Origins XL - Hickory (Chesterfield) T&amp;G | #CAN.E.H.Che.7 |  -". T&amp;G Engineered, 20"-83" random length, 4 Sided Micro Bevel. ORIGINS XL carries NO promotion header - single price only. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF62" t="inlineStr">
@@ -7569,7 +7569,7 @@
       </c>
       <c r="BC63" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Origins XL - Hickory (Claremore) T&amp;G | #CAN.E.H.Cla.7 |  - 7½". T&amp;G Engineered, 20"-83" random length, 4 Sided Micro Bevel. ORIGINS XL carries NO promotion header - single price only. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Origins XL - Hickory (Claremore) T&amp;G | #CAN.E.H.Cla.7 |  - 7½". T&amp;G Engineered, 20"-83" random length, 4 Sided Micro Bevel. ORIGINS XL carries NO promotion header - single price only. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF63" t="inlineStr">
@@ -7686,7 +7686,7 @@
       </c>
       <c r="BC64" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Origins XL - Hickory (Hayward) T&amp;G | #CAN.E.H.Hay.7 |  - 7½" ". T&amp;G Engineered, 20"-83" random length, 4 Sided Micro Bevel. ORIGINS XL carries NO promotion header - single price only. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Origins XL - Hickory (Hayward) T&amp;G | #CAN.E.H.Hay.7 |  - 7½" ". T&amp;G Engineered, 20"-83" random length, 4 Sided Micro Bevel. ORIGINS XL carries NO promotion header - single price only. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF64" t="inlineStr">
@@ -7803,7 +7803,7 @@
       </c>
       <c r="BC65" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Origins XL - Hickory (Thatcher) T&amp;G | #CAN.E.H.Tha.7 |  - 7½"". T&amp;G Engineered, 20"-83" random length, 4 Sided Micro Bevel. ORIGINS XL carries NO promotion header - single price only. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Origins XL - Hickory (Thatcher) T&amp;G | #CAN.E.H.Tha.7 |  - 7½"". T&amp;G Engineered, 20"-83" random length, 4 Sided Micro Bevel. ORIGINS XL carries NO promotion header - single price only. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF65" t="inlineStr">
@@ -7920,7 +7920,7 @@
       </c>
       <c r="BC66" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Origins XL - Hickory (Townsend) T&amp;G | #CAN.E.H.Tow.7 |  - 7½"". T&amp;G Engineered, 20"-83" random length, 4 Sided Micro Bevel. ORIGINS XL carries NO promotion header - single price only. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Origins XL - Hickory (Townsend) T&amp;G | #CAN.E.H.Tow.7 |  - 7½"". T&amp;G Engineered, 20"-83" random length, 4 Sided Micro Bevel. ORIGINS XL carries NO promotion header - single price only. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF66" t="inlineStr">
@@ -8037,7 +8037,7 @@
       </c>
       <c r="BC67" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Origins XL - Oak (Evelyn) T&amp;G | #CAN.E.H.Eve.7 |  - 7½" x ¾" ". T&amp;G Engineered, 20"-83" random length, 4 Sided Micro Bevel. ORIGINS XL carries NO promotion header - single price only. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Origins XL - Oak (Evelyn) T&amp;G | #CAN.E.H.Eve.7 |  - 7½" x ¾" ". T&amp;G Engineered, 20"-83" random length, 4 Sided Micro Bevel. ORIGINS XL carries NO promotion header - single price only. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF67" t="inlineStr">
@@ -8154,7 +8154,7 @@
       </c>
       <c r="BC68" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Origins XL - Oak (Constance) T&amp;G | #CAN.E.H.Con.7 |  - 7½" x ". T&amp;G Engineered, 20"-83" random length, 4 Sided Micro Bevel. ORIGINS XL carries NO promotion header - single price only. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Origins XL - Oak (Constance) T&amp;G | #CAN.E.H.Con.7 |  - 7½" x ". T&amp;G Engineered, 20"-83" random length, 4 Sided Micro Bevel. ORIGINS XL carries NO promotion header - single price only. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF68" t="inlineStr">
@@ -8271,7 +8271,7 @@
       </c>
       <c r="BC69" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Origins XL - Oak (Charlotte (Smoked)) T&amp;G | #CAN.E.H.ChaSm.7 ". T&amp;G Engineered, 20"-83" random length, 4 Sided Micro Bevel. ORIGINS XL carries NO promotion header - single price only. '(Smoked)' printed against the colour name - kept in the colour and mirrored into Finish type. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Origins XL - Oak (Charlotte (Smoked)) T&amp;G | #CAN.E.H.ChaSm.7 ". T&amp;G Engineered, 20"-83" random length, 4 Sided Micro Bevel. ORIGINS XL carries NO promotion header - single price only. '(Smoked)' printed against the colour name - kept in the colour and mirrored into Finish type. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF69" t="inlineStr">
@@ -8388,7 +8388,7 @@
       </c>
       <c r="BC70" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Origins XL - Oak (Emily (Smoked)) T&amp;G | #CAN.E.H.EmiSm.7 |  -". T&amp;G Engineered, 20"-83" random length, 4 Sided Micro Bevel. ORIGINS XL carries NO promotion header - single price only. '(Smoked)' printed against the colour name - kept in the colour and mirrored into Finish type. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Origins XL - Oak (Emily (Smoked)) T&amp;G | #CAN.E.H.EmiSm.7 |  -". T&amp;G Engineered, 20"-83" random length, 4 Sided Micro Bevel. ORIGINS XL carries NO promotion header - single price only. '(Smoked)' printed against the colour name - kept in the colour and mirrored into Finish type. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF70" t="inlineStr">
@@ -8505,7 +8505,7 @@
       </c>
       <c r="BC71" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Origins XL - Oak (Leah (Smoked)) T&amp;G | #CAN.E.H.LeaSm.7 |  - ". T&amp;G Engineered, 20"-83" random length, 4 Sided Micro Bevel. ORIGINS XL carries NO promotion header - single price only. '(Smoked)' printed against the colour name - kept in the colour and mirrored into Finish type. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Origins XL - Oak (Leah (Smoked)) T&amp;G | #CAN.E.H.LeaSm.7 |  - ". T&amp;G Engineered, 20"-83" random length, 4 Sided Micro Bevel. ORIGINS XL carries NO promotion header - single price only. '(Smoked)' printed against the colour name - kept in the colour and mirrored into Finish type. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF71" t="inlineStr">
@@ -8635,7 +8635,7 @@
       </c>
       <c r="BC72" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANENG - Origins - Oak (Irish Tea) T&amp;G | #CAN.E.O.IriTea.6 |  - 6½". PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). Promo Code: LOYAL399. Promo price $3.99 / Reg. price $4.79. 6.5" x 3/4" x RL (16"-75"). Supplier marks this colour *DISCONTINUE ITEM* on the Aug 31 2026 list -&gt; Stock status = Discontinued, Active = FALSE. Confirm remaining stock before import. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANENG - Origins - Oak (Irish Tea) T&amp;G | #CAN.E.O.IriTea.6 |  - 6½". PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). Promo Code: LOYAL399. Promo price $3.99 / Reg. price $4.79. 6.5" x 3/4" x RL (16"-75"). Supplier marks this colour *DISCONTINUE ITEM* on the Aug 31 2026 list -&gt; Stock status = Discontinued, Active = FALSE. Confirm remaining stock before import. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF72" t="inlineStr">
@@ -8760,7 +8760,7 @@
       </c>
       <c r="BC73" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANENG - Origins - Oak (Planetary Silver) T&amp;G | #CAN.E.O.PlaSil.6 ". PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). Promo Code: LOYAL399. Promo price $3.99 / Reg. price $4.79. 6.5" x 3/4" x RL (16"-75"). COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANENG - Origins - Oak (Planetary Silver) T&amp;G | #CAN.E.O.PlaSil.6 ". PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). Promo Code: LOYAL399. Promo price $3.99 / Reg. price $4.79. 6.5" x 3/4" x RL (16"-75"). COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF73" t="inlineStr">
@@ -8890,7 +8890,7 @@
       </c>
       <c r="BC74" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANENG - Origins - Oak (Polo Pony) T&amp;G | #CAN.E.O.PolPon.6 |  - 6½". PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). Promo Code: LOYAL399. Promo price $3.99 / Reg. price $4.79. 6.5" x 3/4" x RL (16"-75"). Supplier marks this colour *DISCONTINUE ITEM* on the Aug 31 2026 list -&gt; Stock status = Discontinued, Active = FALSE. Confirm remaining stock before import. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANENG - Origins - Oak (Polo Pony) T&amp;G | #CAN.E.O.PolPon.6 |  - 6½". PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). Promo Code: LOYAL399. Promo price $3.99 / Reg. price $4.79. 6.5" x 3/4" x RL (16"-75"). Supplier marks this colour *DISCONTINUE ITEM* on the Aug 31 2026 list -&gt; Stock status = Discontinued, Active = FALSE. Confirm remaining stock before import. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF74" t="inlineStr">
@@ -9020,7 +9020,7 @@
       </c>
       <c r="BC75" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANENG - Origins - Oak (Shoreline Grey) T&amp;G | #CAN.E.O.ShoGre.6 | ". PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). Promo Code: LOYAL399. Promo price $3.99 / Reg. price $4.79. 6.5" x 3/4" x RL (16"-75"). Supplier marks this colour *DISCONTINUE ITEM* on the Aug 31 2026 list -&gt; Stock status = Discontinued, Active = FALSE. Confirm remaining stock before import. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANENG - Origins - Oak (Shoreline Grey) T&amp;G | #CAN.E.O.ShoGre.6 | ". PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). Promo Code: LOYAL399. Promo price $3.99 / Reg. price $4.79. 6.5" x 3/4" x RL (16"-75"). Supplier marks this colour *DISCONTINUE ITEM* on the Aug 31 2026 list -&gt; Stock status = Discontinued, Active = FALSE. Confirm remaining stock before import. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF75" t="inlineStr">
@@ -9145,7 +9145,7 @@
       </c>
       <c r="BC76" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANENG - Origins - Oak (Subtle White) T&amp;G | #CAN.E.O.SubWhi.6 |  -". PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). Promo Code: LOYAL399. Promo price $3.99 / Reg. price $4.79. 6.5" x 3/4" x RL (16"-75"). COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANENG - Origins - Oak (Subtle White) T&amp;G | #CAN.E.O.SubWhi.6 |  -". PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). Promo Code: LOYAL399. Promo price $3.99 / Reg. price $4.79. 6.5" x 3/4" x RL (16"-75"). COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF76" t="inlineStr">
@@ -9270,7 +9270,7 @@
       </c>
       <c r="BC77" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "*****DISCONTINUED********(P) CANENG - Origins - Hickory (Forest Trail)". PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). Promo Code: LOYAL399. Promo price $3.99 / Reg. price $4.79. 6.5" x 3/4" x RL (16"-75"). COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "*****DISCONTINUED********(P) CANENG - Origins - Hickory (Forest Trail)". PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). Promo Code: LOYAL399. Promo price $3.99 / Reg. price $4.79. 6.5" x 3/4" x RL (16"-75"). COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF77" t="inlineStr">
@@ -9395,7 +9395,7 @@
       </c>
       <c r="BC78" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "*****DISCONTINUED********(P) CANENG - Origins - Hickory (Greysmith) T&amp;". PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). Promo Code: LOYAL399. Promo price $3.99 / Reg. price $4.79. 6.5" x 3/4" x RL (16"-75"). COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "*****DISCONTINUED********(P) CANENG - Origins - Hickory (Greysmith) T&amp;". PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). Promo Code: LOYAL399. Promo price $3.99 / Reg. price $4.79. 6.5" x 3/4" x RL (16"-75"). COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF78" t="inlineStr">
@@ -9520,7 +9520,7 @@
       </c>
       <c r="BC79" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANENG - Origins - Hickory (Nottingham) T&amp;G | #CAN.E.H.Not.6 |  - ". PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). Promo Code: LOYAL399. Promo price $3.99 / Reg. price $4.79. 6.5" x 3/4" x RL (16"-75"). COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANENG - Origins - Hickory (Nottingham) T&amp;G | #CAN.E.H.Not.6 |  - ". PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). Promo Code: LOYAL399. Promo price $3.99 / Reg. price $4.79. 6.5" x 3/4" x RL (16"-75"). COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF79" t="inlineStr">
@@ -9645,7 +9645,7 @@
       </c>
       <c r="BC80" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "*****DISCONTINUED********(P) CANENG - Origins - Hickory (Warm Heritage". PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). Promo Code: LOYAL399. Promo price $3.99 / Reg. price $4.79. 6.5" x 3/4" x RL (16"-75"). COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "*****DISCONTINUED********(P) CANENG - Origins - Hickory (Warm Heritage". PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). Promo Code: LOYAL399. Promo price $3.99 / Reg. price $4.79. 6.5" x 3/4" x RL (16"-75"). COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF80" t="inlineStr">
@@ -9775,7 +9775,7 @@
       </c>
       <c r="BC81" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANENG - Origins - Hickory (Winchester) T&amp;G | #CAN.E.H.Win.6 |  - ". PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). Promo Code: LOYAL399. Promo price $3.99 / Reg. price $4.79. 6.5" x 3/4" x RL (16"-75"). Supplier marks this colour *DISCONTINUE ITEM* on the Aug 31 2026 list -&gt; Stock status = Discontinued, Active = FALSE. Confirm remaining stock before import. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANENG - Origins - Hickory (Winchester) T&amp;G | #CAN.E.H.Win.6 |  - ". PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). Promo Code: LOYAL399. Promo price $3.99 / Reg. price $4.79. 6.5" x 3/4" x RL (16"-75"). Supplier marks this colour *DISCONTINUE ITEM* on the Aug 31 2026 list -&gt; Stock status = Discontinued, Active = FALSE. Confirm remaining stock before import. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF81" t="inlineStr">
@@ -9892,7 +9892,7 @@
       </c>
       <c r="BC82" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Origins - Oak (Grayson) T&amp;G | #CAN.E.O.Gra.7 |  - 7½" x ¾" x ". Sits under a 'Promotion Valid until October 31, 2026' section header but prints only ONE price - treated as a regular price, no promo fields applied. Confirm with supplier. 7.5" x 3/4" x RL (16"-75"). COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Origins - Oak (Grayson) T&amp;G | #CAN.E.O.Gra.7 |  - 7½" x ¾" x ". Sits under a 'Promotion Valid until October 31, 2026' section header but prints only ONE price - treated as a regular price, no promo fields applied. Confirm with supplier. 7.5" x 3/4" x RL (16"-75"). COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF82" t="inlineStr">
@@ -10009,7 +10009,7 @@
       </c>
       <c r="BC83" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Origins - Oak (Hampshire) T&amp;G | #CAN.E.O.Ham.7 |  - 7½" x ¾" ". Sits under a 'Promotion Valid until October 31, 2026' section header but prints only ONE price - treated as a regular price, no promo fields applied. Confirm with supplier. 7.5" x 3/4" x RL (16"-75"). COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Origins - Oak (Hampshire) T&amp;G | #CAN.E.O.Ham.7 |  - 7½" x ¾" ". Sits under a 'Promotion Valid until October 31, 2026' section header but prints only ONE price - treated as a regular price, no promo fields applied. Confirm with supplier. 7.5" x 3/4" x RL (16"-75"). COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF83" t="inlineStr">
@@ -10131,7 +10131,7 @@
       </c>
       <c r="BC84" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Origins - Oak (Kate) T&amp;G | #CAN.E.O.Kat.7 |  - 7½" x ¾" x RL ". Sits under a 'Promotion Valid until October 31, 2026' section header but prints only ONE price - treated as a regular price, no promo fields applied. Confirm with supplier. 7.5" x 3/4" x RL (16"-75"). Supplier marks this colour *DISCONTINUE ITEM* on the Aug 31 2026 list -&gt; Stock status = Discontinued, Active = FALSE. Confirm remaining stock before import. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Origins - Oak (Kate) T&amp;G | #CAN.E.O.Kat.7 |  - 7½" x ¾" x RL ". Sits under a 'Promotion Valid until October 31, 2026' section header but prints only ONE price - treated as a regular price, no promo fields applied. Confirm with supplier. 7.5" x 3/4" x RL (16"-75"). Supplier marks this colour *DISCONTINUE ITEM* on the Aug 31 2026 list -&gt; Stock status = Discontinued, Active = FALSE. Confirm remaining stock before import. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF84" t="inlineStr">
@@ -10248,7 +10248,7 @@
       </c>
       <c r="BC85" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Origins - Oak (Kinsey) T&amp;G | #CAN.E.O.Kin.7 |  - 7½" x ¾" x R". Sits under a 'Promotion Valid until October 31, 2026' section header but prints only ONE price - treated as a regular price, no promo fields applied. Confirm with supplier. 7.5" x 3/4" x RL (16"-75"). COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Origins - Oak (Kinsey) T&amp;G | #CAN.E.O.Kin.7 |  - 7½" x ¾" x R". Sits under a 'Promotion Valid until October 31, 2026' section header but prints only ONE price - treated as a regular price, no promo fields applied. Confirm with supplier. 7.5" x 3/4" x RL (16"-75"). COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF85" t="inlineStr">
@@ -10365,7 +10365,7 @@
       </c>
       <c r="BC86" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Origins - Oak (Sedrick) T&amp;G | #CAN.E.O.Sed.7 |  - 7½" x ¾" x ". Sits under a 'Promotion Valid until October 31, 2026' section header but prints only ONE price - treated as a regular price, no promo fields applied. Confirm with supplier. 7.5" x 3/4" x RL (16"-75"). COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Origins - Oak (Sedrick) T&amp;G | #CAN.E.O.Sed.7 |  - 7½" x ¾" x ". Sits under a 'Promotion Valid until October 31, 2026' section header but prints only ONE price - treated as a regular price, no promo fields applied. Confirm with supplier. 7.5" x 3/4" x RL (16"-75"). COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF86" t="inlineStr">
@@ -10487,7 +10487,7 @@
       </c>
       <c r="BC87" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Origins - Oak (Tiffany) T&amp;G | #CAN.E.O.Tif.7 |  - 7½" x ¾" x ". Sits under a 'Promotion Valid until October 31, 2026' section header but prints only ONE price - treated as a regular price, no promo fields applied. Confirm with supplier. 7.5" x 3/4" x RL (16"-75"). Supplier marks this colour *DISCONTINUE ITEM* on the Aug 31 2026 list -&gt; Stock status = Discontinued, Active = FALSE. Confirm remaining stock before import. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Origins - Oak (Tiffany) T&amp;G | #CAN.E.O.Tif.7 |  - 7½" x ¾" x ". Sits under a 'Promotion Valid until October 31, 2026' section header but prints only ONE price - treated as a regular price, no promo fields applied. Confirm with supplier. 7.5" x 3/4" x RL (16"-75"). Supplier marks this colour *DISCONTINUE ITEM* on the Aug 31 2026 list -&gt; Stock status = Discontinued, Active = FALSE. Confirm remaining stock before import. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF87" t="inlineStr">
@@ -10604,7 +10604,7 @@
       </c>
       <c r="BC88" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Origins - American Walnut (Astoria) T&amp;G | #CAN.E.H.Ast.7 |  -". Sits under a 'Promotion Valid until October 31, 2026' section header but prints only ONE price - treated as a regular price, no promo fields applied. Confirm with supplier. 7.5" x 3/4" x RL. Duchy Estate is annotated '(FLAT FINISH)' on the sheet. Radiant heat: American Walnut - the global Black Walnut rule covers American Black Walnut; the sheet says 'American Walnut' only, so Radiant heat compatible left blank pending confirmation. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Origins - American Walnut (Astoria) T&amp;G | #CAN.E.H.Ast.7 |  -". Sits under a 'Promotion Valid until October 31, 2026' section header but prints only ONE price - treated as a regular price, no promo fields applied. Confirm with supplier. 7.5" x 3/4" x RL. Duchy Estate is annotated '(FLAT FINISH)' on the sheet. Radiant heat: American Walnut - the global Black Walnut rule covers American Black Walnut; the sheet says 'American Walnut' only, so Radiant heat compatible left blank pending confirmation. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF88" t="inlineStr">
@@ -10721,7 +10721,7 @@
       </c>
       <c r="BC89" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour variant match to Lightspeed product "CANENG - Origins - American Walnut (Dushy Estate (FLAT FINISH)) T&amp;G | ". Sits under a 'Promotion Valid until October 31, 2026' section header but prints only ONE price - treated as a regular price, no promo fields applied. Confirm with supplier. 7.5" x 3/4" x RL. Duchy Estate is annotated '(FLAT FINISH)' on the sheet. Radiant heat: American Walnut - the global Black Walnut rule covers American Black Walnut; the sheet says 'American Walnut' only, so Radiant heat compatible left blank pending confirmation. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour variant match to Lightspeed product "CANENG - Origins - American Walnut (Dushy Estate (FLAT FINISH)) T&amp;G | ". Sits under a 'Promotion Valid until October 31, 2026' section header but prints only ONE price - treated as a regular price, no promo fields applied. Confirm with supplier. 7.5" x 3/4" x RL. Duchy Estate is annotated '(FLAT FINISH)' on the sheet. Radiant heat: American Walnut - the global Black Walnut rule covers American Black Walnut; the sheet says 'American Walnut' only, so Radiant heat compatible left blank pending confirmation. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF89" t="inlineStr">
@@ -10838,7 +10838,7 @@
       </c>
       <c r="BC90" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Origins - American Walnut (Royal Mile) T&amp;G | #CAN.E.H.RoyMil.". Sits under a 'Promotion Valid until October 31, 2026' section header but prints only ONE price - treated as a regular price, no promo fields applied. Confirm with supplier. 7.5" x 3/4" x RL. Duchy Estate is annotated '(FLAT FINISH)' on the sheet. Radiant heat: American Walnut - the global Black Walnut rule covers American Black Walnut; the sheet says 'American Walnut' only, so Radiant heat compatible left blank pending confirmation. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Origins - American Walnut (Royal Mile) T&amp;G | #CAN.E.H.RoyMil.". Sits under a 'Promotion Valid until October 31, 2026' section header but prints only ONE price - treated as a regular price, no promo fields applied. Confirm with supplier. 7.5" x 3/4" x RL. Duchy Estate is annotated '(FLAT FINISH)' on the sheet. Radiant heat: American Walnut - the global Black Walnut rule covers American Black Walnut; the sheet says 'American Walnut' only, so Radiant heat compatible left blank pending confirmation. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF90" t="inlineStr">
@@ -10955,7 +10955,7 @@
       </c>
       <c r="BC91" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Origins - American Walnut (Surrey Hills) T&amp;G | #CAN.E.H.SurHi". Sits under a 'Promotion Valid until October 31, 2026' section header but prints only ONE price - treated as a regular price, no promo fields applied. Confirm with supplier. 7.5" x 3/4" x RL. Duchy Estate is annotated '(FLAT FINISH)' on the sheet. Radiant heat: American Walnut - the global Black Walnut rule covers American Black Walnut; the sheet says 'American Walnut' only, so Radiant heat compatible left blank pending confirmation. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Origins - American Walnut (Surrey Hills) T&amp;G | #CAN.E.H.SurHi". Sits under a 'Promotion Valid until October 31, 2026' section header but prints only ONE price - treated as a regular price, no promo fields applied. Confirm with supplier. 7.5" x 3/4" x RL. Duchy Estate is annotated '(FLAT FINISH)' on the sheet. Radiant heat: American Walnut - the global Black Walnut rule covers American Black Walnut; the sheet says 'American Walnut' only, so Radiant heat compatible left blank pending confirmation. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF91" t="inlineStr">
@@ -11072,7 +11072,7 @@
       </c>
       <c r="BC92" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Origins - American Walnut (Yorkshire) T&amp;G | #CAN.E.H.Yor.7 | ". Sits under a 'Promotion Valid until October 31, 2026' section header but prints only ONE price - treated as a regular price, no promo fields applied. Confirm with supplier. 7.5" x 3/4" x RL. Duchy Estate is annotated '(FLAT FINISH)' on the sheet. Radiant heat: American Walnut - the global Black Walnut rule covers American Black Walnut; the sheet says 'American Walnut' only, so Radiant heat compatible left blank pending confirmation. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Origins - American Walnut (Yorkshire) T&amp;G | #CAN.E.H.Yor.7 | ". Sits under a 'Promotion Valid until October 31, 2026' section header but prints only ONE price - treated as a regular price, no promo fields applied. Confirm with supplier. 7.5" x 3/4" x RL. Duchy Estate is annotated '(FLAT FINISH)' on the sheet. Radiant heat: American Walnut - the global Black Walnut rule covers American Black Walnut; the sheet says 'American Walnut' only, so Radiant heat compatible left blank pending confirmation. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF92" t="inlineStr">
@@ -11198,7 +11198,7 @@
       </c>
       <c r="BC93" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANVIN - Vanntett Plus (SPC) -  (Dawson)  | #CAN.V.Daw.9 |  - 9" x". PROMO (deviation flagged): VANNTETT PLUS prints a paired 'Promotion Price $2.10' / 'Regular Price $2.49' but NO promotion window. Global sale-item logic applied (Cost = Regular, Promo cost = Promotion) and the global month-end default used for the end date -&gt; 2026-09-30. The run brief said VANNTETT gets no promo fields; the document contradicts that, so the discount is captured rather than dropped. Albert to confirm the end date. 9" x 60" x 7mm, 7mm SPC + IXPE backing, 100% waterproof, micro-bevelled edges. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANVIN - Vanntett Plus (SPC) -  (Dawson)  | #CAN.V.Daw.9 |  - 9" x". PROMO (deviation flagged): VANNTETT PLUS prints a paired 'Promotion Price $2.10' / 'Regular Price $2.49' but NO promotion window. Global sale-item logic applied (Cost = Regular, Promo cost = Promotion) and the global month-end default used for the end date -&gt; 2026-09-30. The run brief said VANNTETT gets no promo fields; the document contradicts that, so the discount is captured rather than dropped. Albert to confirm the end date. 9" x 60" x 7mm, 7mm SPC + IXPE backing, 100% waterproof, micro-bevelled edges. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF93" t="inlineStr">
@@ -11324,7 +11324,7 @@
       </c>
       <c r="BC94" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANVIN - Vanntett Plus (SPC) -  (Eddi)  | #CAN.V.Edd.9 |  - 9" x 6". PROMO (deviation flagged): VANNTETT PLUS prints a paired 'Promotion Price $2.10' / 'Regular Price $2.49' but NO promotion window. Global sale-item logic applied (Cost = Regular, Promo cost = Promotion) and the global month-end default used for the end date -&gt; 2026-09-30. The run brief said VANNTETT gets no promo fields; the document contradicts that, so the discount is captured rather than dropped. Albert to confirm the end date. 9" x 60" x 7mm, 7mm SPC + IXPE backing, 100% waterproof, micro-bevelled edges. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANVIN - Vanntett Plus (SPC) -  (Eddi)  | #CAN.V.Edd.9 |  - 9" x 6". PROMO (deviation flagged): VANNTETT PLUS prints a paired 'Promotion Price $2.10' / 'Regular Price $2.49' but NO promotion window. Global sale-item logic applied (Cost = Regular, Promo cost = Promotion) and the global month-end default used for the end date -&gt; 2026-09-30. The run brief said VANNTETT gets no promo fields; the document contradicts that, so the discount is captured rather than dropped. Albert to confirm the end date. 9" x 60" x 7mm, 7mm SPC + IXPE backing, 100% waterproof, micro-bevelled edges. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF94" t="inlineStr">
@@ -11450,7 +11450,7 @@
       </c>
       <c r="BC95" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANVIN - Vanntett Plus (SPC) -  (Ellis)  | #CAN.V.Ell.9 |  - 9" x ". PROMO (deviation flagged): VANNTETT PLUS prints a paired 'Promotion Price $2.10' / 'Regular Price $2.49' but NO promotion window. Global sale-item logic applied (Cost = Regular, Promo cost = Promotion) and the global month-end default used for the end date -&gt; 2026-09-30. The run brief said VANNTETT gets no promo fields; the document contradicts that, so the discount is captured rather than dropped. Albert to confirm the end date. 9" x 60" x 7mm, 7mm SPC + IXPE backing, 100% waterproof, micro-bevelled edges. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANVIN - Vanntett Plus (SPC) -  (Ellis)  | #CAN.V.Ell.9 |  - 9" x ". PROMO (deviation flagged): VANNTETT PLUS prints a paired 'Promotion Price $2.10' / 'Regular Price $2.49' but NO promotion window. Global sale-item logic applied (Cost = Regular, Promo cost = Promotion) and the global month-end default used for the end date -&gt; 2026-09-30. The run brief said VANNTETT gets no promo fields; the document contradicts that, so the discount is captured rather than dropped. Albert to confirm the end date. 9" x 60" x 7mm, 7mm SPC + IXPE backing, 100% waterproof, micro-bevelled edges. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF95" t="inlineStr">
@@ -11576,7 +11576,7 @@
       </c>
       <c r="BC96" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANVIN - Vanntett Plus (SPC) -  (Ernest)  | #CAN.V.Ern.9 |  - 9" x". PROMO (deviation flagged): VANNTETT PLUS prints a paired 'Promotion Price $2.10' / 'Regular Price $2.49' but NO promotion window. Global sale-item logic applied (Cost = Regular, Promo cost = Promotion) and the global month-end default used for the end date -&gt; 2026-09-30. The run brief said VANNTETT gets no promo fields; the document contradicts that, so the discount is captured rather than dropped. Albert to confirm the end date. 9" x 60" x 7mm, 7mm SPC + IXPE backing, 100% waterproof, micro-bevelled edges. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANVIN - Vanntett Plus (SPC) -  (Ernest)  | #CAN.V.Ern.9 |  - 9" x". PROMO (deviation flagged): VANNTETT PLUS prints a paired 'Promotion Price $2.10' / 'Regular Price $2.49' but NO promotion window. Global sale-item logic applied (Cost = Regular, Promo cost = Promotion) and the global month-end default used for the end date -&gt; 2026-09-30. The run brief said VANNTETT gets no promo fields; the document contradicts that, so the discount is captured rather than dropped. Albert to confirm the end date. 9" x 60" x 7mm, 7mm SPC + IXPE backing, 100% waterproof, micro-bevelled edges. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF96" t="inlineStr">
@@ -11702,7 +11702,7 @@
       </c>
       <c r="BC97" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANVIN - Vanntett Plus (SPC) -  (Lesley)  | #CAN.V.Les.9 |  - 9" x". PROMO (deviation flagged): VANNTETT PLUS prints a paired 'Promotion Price $2.10' / 'Regular Price $2.49' but NO promotion window. Global sale-item logic applied (Cost = Regular, Promo cost = Promotion) and the global month-end default used for the end date -&gt; 2026-09-30. The run brief said VANNTETT gets no promo fields; the document contradicts that, so the discount is captured rather than dropped. Albert to confirm the end date. 9" x 60" x 7mm, 7mm SPC + IXPE backing, 100% waterproof, micro-bevelled edges. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANVIN - Vanntett Plus (SPC) -  (Lesley)  | #CAN.V.Les.9 |  - 9" x". PROMO (deviation flagged): VANNTETT PLUS prints a paired 'Promotion Price $2.10' / 'Regular Price $2.49' but NO promotion window. Global sale-item logic applied (Cost = Regular, Promo cost = Promotion) and the global month-end default used for the end date -&gt; 2026-09-30. The run brief said VANNTETT gets no promo fields; the document contradicts that, so the discount is captured rather than dropped. Albert to confirm the end date. 9" x 60" x 7mm, 7mm SPC + IXPE backing, 100% waterproof, micro-bevelled edges. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF97" t="inlineStr">
@@ -11828,7 +11828,7 @@
       </c>
       <c r="BC98" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANVIN - Vanntett Plus (SPC) -  (Nadine)  | #CAN.V.Nad.9 |  - 9" x". PROMO (deviation flagged): VANNTETT PLUS prints a paired 'Promotion Price $2.10' / 'Regular Price $2.49' but NO promotion window. Global sale-item logic applied (Cost = Regular, Promo cost = Promotion) and the global month-end default used for the end date -&gt; 2026-09-30. The run brief said VANNTETT gets no promo fields; the document contradicts that, so the discount is captured rather than dropped. Albert to confirm the end date. 9" x 60" x 7mm, 7mm SPC + IXPE backing, 100% waterproof, micro-bevelled edges. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANVIN - Vanntett Plus (SPC) -  (Nadine)  | #CAN.V.Nad.9 |  - 9" x". PROMO (deviation flagged): VANNTETT PLUS prints a paired 'Promotion Price $2.10' / 'Regular Price $2.49' but NO promotion window. Global sale-item logic applied (Cost = Regular, Promo cost = Promotion) and the global month-end default used for the end date -&gt; 2026-09-30. The run brief said VANNTETT gets no promo fields; the document contradicts that, so the discount is captured rather than dropped. Albert to confirm the end date. 9" x 60" x 7mm, 7mm SPC + IXPE backing, 100% waterproof, micro-bevelled edges. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF98" t="inlineStr">
@@ -11954,7 +11954,7 @@
       </c>
       <c r="BC99" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANVIN - Vanntett Plus (SPC) -  (Percy)  | #CAN.V.Per.9 |  - 9" x ". PROMO (deviation flagged): VANNTETT PLUS prints a paired 'Promotion Price $2.10' / 'Regular Price $2.49' but NO promotion window. Global sale-item logic applied (Cost = Regular, Promo cost = Promotion) and the global month-end default used for the end date -&gt; 2026-09-30. The run brief said VANNTETT gets no promo fields; the document contradicts that, so the discount is captured rather than dropped. Albert to confirm the end date. 9" x 60" x 7mm, 7mm SPC + IXPE backing, 100% waterproof, micro-bevelled edges. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANVIN - Vanntett Plus (SPC) -  (Percy)  | #CAN.V.Per.9 |  - 9" x ". PROMO (deviation flagged): VANNTETT PLUS prints a paired 'Promotion Price $2.10' / 'Regular Price $2.49' but NO promotion window. Global sale-item logic applied (Cost = Regular, Promo cost = Promotion) and the global month-end default used for the end date -&gt; 2026-09-30. The run brief said VANNTETT gets no promo fields; the document contradicts that, so the discount is captured rather than dropped. Albert to confirm the end date. 9" x 60" x 7mm, 7mm SPC + IXPE backing, 100% waterproof, micro-bevelled edges. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF99" t="inlineStr">
@@ -12080,7 +12080,7 @@
       </c>
       <c r="BC100" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANVIN - Vanntett Plus (SPC) -  (Phoebe)  | #CAN.V.Pho.9 |  - 9" x". PROMO (deviation flagged): VANNTETT PLUS prints a paired 'Promotion Price $2.10' / 'Regular Price $2.49' but NO promotion window. Global sale-item logic applied (Cost = Regular, Promo cost = Promotion) and the global month-end default used for the end date -&gt; 2026-09-30. The run brief said VANNTETT gets no promo fields; the document contradicts that, so the discount is captured rather than dropped. Albert to confirm the end date. 9" x 60" x 7mm, 7mm SPC + IXPE backing, 100% waterproof, micro-bevelled edges. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANVIN - Vanntett Plus (SPC) -  (Phoebe)  | #CAN.V.Pho.9 |  - 9" x". PROMO (deviation flagged): VANNTETT PLUS prints a paired 'Promotion Price $2.10' / 'Regular Price $2.49' but NO promotion window. Global sale-item logic applied (Cost = Regular, Promo cost = Promotion) and the global month-end default used for the end date -&gt; 2026-09-30. The run brief said VANNTETT gets no promo fields; the document contradicts that, so the discount is captured rather than dropped. Albert to confirm the end date. 9" x 60" x 7mm, 7mm SPC + IXPE backing, 100% waterproof, micro-bevelled edges. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF100" t="inlineStr">
@@ -12201,7 +12201,7 @@
       </c>
       <c r="BC101" t="inlineStr">
         <is>
-          <t>PROMO (deviation flagged): VANNTETT PLUS prints a paired 'Promotion Price $2.10' / 'Regular Price $2.49' but NO promotion window. Global sale-item logic applied (Cost = Regular, Promo cost = Promotion) and the global month-end default used for the end date -&gt; 2026-09-30. The run brief said VANNTETT gets no promo fields; the document contradicts that, so the discount is captured rather than dropped. Albert to confirm the end date. 9" x 60" x 7mm, 7mm SPC + IXPE backing, 100% waterproof, micro-bevelled edges. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>PROMO (deviation flagged): VANNTETT PLUS prints a paired 'Promotion Price $2.10' / 'Regular Price $2.49' but NO promotion window. Global sale-item logic applied (Cost = Regular, Promo cost = Promotion) and the global month-end default used for the end date -&gt; 2026-09-30. The run brief said VANNTETT gets no promo fields; the document contradicts that, so the discount is captured rather than dropped. Albert to confirm the end date. 9" x 60" x 7mm, 7mm SPC + IXPE backing, 100% waterproof, micro-bevelled edges. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF101" t="inlineStr">
@@ -12327,7 +12327,7 @@
       </c>
       <c r="BC102" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANVIN - Vanntett Plus (SPC) -  (Ross)  | #CAN.V.Ros.9 |  - 9" x 6". PROMO (deviation flagged): VANNTETT PLUS prints a paired 'Promotion Price $2.10' / 'Regular Price $2.49' but NO promotion window. Global sale-item logic applied (Cost = Regular, Promo cost = Promotion) and the global month-end default used for the end date -&gt; 2026-09-30. The run brief said VANNTETT gets no promo fields; the document contradicts that, so the discount is captured rather than dropped. Albert to confirm the end date. 9" x 60" x 7mm, 7mm SPC + IXPE backing, 100% waterproof, micro-bevelled edges. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANVIN - Vanntett Plus (SPC) -  (Ross)  | #CAN.V.Ros.9 |  - 9" x 6". PROMO (deviation flagged): VANNTETT PLUS prints a paired 'Promotion Price $2.10' / 'Regular Price $2.49' but NO promotion window. Global sale-item logic applied (Cost = Regular, Promo cost = Promotion) and the global month-end default used for the end date -&gt; 2026-09-30. The run brief said VANNTETT gets no promo fields; the document contradicts that, so the discount is captured rather than dropped. Albert to confirm the end date. 9" x 60" x 7mm, 7mm SPC + IXPE backing, 100% waterproof, micro-bevelled edges. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF102" t="inlineStr">
@@ -12405,7 +12405,7 @@
       </c>
       <c r="BC103" t="inlineStr">
         <is>
-          <t>Per-piece trim, 2400mm x 45mm x 7mm. Cross-supplier accessory markup applied (T-Moulding/Reducer +$10, Stair Nose +$15) -&gt; Retail $28.00/pc. Supplier: 'Due to the fragile nature of this product, all sales are final. No Returns or Exchanges.' Sheet groups 'T Moulding / Reducer' at $18.00 (2400x45x7mm) and 'Stair Nose Overlap' at $22.00 (2400x53x18mm). COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example). Single SKU covering VANNTETT PLUS and VANNTETTPRO: identical dimensions and price, one physical part.</t>
+          <t>Per-piece trim, 2400mm x 45mm x 7mm. Cross-supplier accessory markup applied (T-Moulding/Reducer +$10, Stair Nose +$15) -&gt; Retail $28.00/pc. Supplier: 'Due to the fragile nature of this product, all sales are final. No Returns or Exchanges.' Sheet groups 'T Moulding / Reducer' at $18.00 (2400x45x7mm) and 'Stair Nose Overlap' at $22.00 (2400x53x18mm). COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example). Single SKU covering VANNTETT PLUS and VANNTETTPRO: identical dimensions and price, one physical part.</t>
         </is>
       </c>
       <c r="BF103" t="inlineStr">
@@ -12483,7 +12483,7 @@
       </c>
       <c r="BC104" t="inlineStr">
         <is>
-          <t>Per-piece trim, 2400mm x 45mm x 7mm. Cross-supplier accessory markup applied (T-Moulding/Reducer +$10, Stair Nose +$15) -&gt; Retail $28.00/pc. Supplier: 'Due to the fragile nature of this product, all sales are final. No Returns or Exchanges.' Sheet groups 'T Moulding / Reducer' at $18.00 (2400x45x7mm) and 'Stair Nose Overlap' at $22.00 (2400x53x18mm). COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example). Single SKU covering VANNTETT PLUS and VANNTETTPRO: identical dimensions and price, one physical part.</t>
+          <t>Per-piece trim, 2400mm x 45mm x 7mm. Cross-supplier accessory markup applied (T-Moulding/Reducer +$10, Stair Nose +$15) -&gt; Retail $28.00/pc. Supplier: 'Due to the fragile nature of this product, all sales are final. No Returns or Exchanges.' Sheet groups 'T Moulding / Reducer' at $18.00 (2400x45x7mm) and 'Stair Nose Overlap' at $22.00 (2400x53x18mm). COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example). Single SKU covering VANNTETT PLUS and VANNTETTPRO: identical dimensions and price, one physical part.</t>
         </is>
       </c>
       <c r="BF104" t="inlineStr">
@@ -12561,7 +12561,7 @@
       </c>
       <c r="BC105" t="inlineStr">
         <is>
-          <t>Per-piece trim, 2400mm x 53mm x 18mm. Cross-supplier accessory markup applied (T-Moulding/Reducer +$10, Stair Nose +$15) -&gt; Retail $37.00/pc. Supplier: 'Due to the fragile nature of this product, all sales are final. No Returns or Exchanges.' Sheet groups 'T Moulding / Reducer' at $18.00 (2400x45x7mm) and 'Stair Nose Overlap' at $22.00 (2400x53x18mm). COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example). Single SKU covering VANNTETT PLUS and VANNTETTPRO: identical dimensions and price, one physical part.</t>
+          <t>Per-piece trim, 2400mm x 53mm x 18mm. Cross-supplier accessory markup applied (T-Moulding/Reducer +$10, Stair Nose +$15) -&gt; Retail $37.00/pc. Supplier: 'Due to the fragile nature of this product, all sales are final. No Returns or Exchanges.' Sheet groups 'T Moulding / Reducer' at $18.00 (2400x45x7mm) and 'Stair Nose Overlap' at $22.00 (2400x53x18mm). COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example). Single SKU covering VANNTETT PLUS and VANNTETTPRO: identical dimensions and price, one physical part.</t>
         </is>
       </c>
       <c r="BF105" t="inlineStr">
@@ -12682,7 +12682,7 @@
       </c>
       <c r="BC106" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANVIN - Vanetettpro SPC LVP -  (Copenhagen)  | #CAN.V.0.Cop.7 |  - 7"". 7" x 48" x 5.2mm, 5.2mm SPC + IXPE backing, 100% waterproof. Single price, no promo pair. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANVIN - Vanetettpro SPC LVP -  (Copenhagen)  | #CAN.V.0.Cop.7 |  - 7"". 7" x 48" x 5.2mm, 5.2mm SPC + IXPE backing, 100% waterproof. Single price, no promo pair. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF106" t="inlineStr">
@@ -12803,7 +12803,7 @@
       </c>
       <c r="BC107" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANVIN - Vanetettpro SPC LVP -  (Cozy Space)  | #CAN.V.0.CozSpa.7 |  -". 7" x 48" x 5.2mm, 5.2mm SPC + IXPE backing, 100% waterproof. Single price, no promo pair. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANVIN - Vanetettpro SPC LVP -  (Cozy Space)  | #CAN.V.0.CozSpa.7 |  -". 7" x 48" x 5.2mm, 5.2mm SPC + IXPE backing, 100% waterproof. Single price, no promo pair. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF107" t="inlineStr">
@@ -12924,7 +12924,7 @@
       </c>
       <c r="BC108" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANVIN - Vanetettpro SPC LVP -  (Grey Shimmer)  | #CAN.V.0.GreShi.7 | ". 7" x 48" x 5.2mm, 5.2mm SPC + IXPE backing, 100% waterproof. Single price, no promo pair. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANVIN - Vanetettpro SPC LVP -  (Grey Shimmer)  | #CAN.V.0.GreShi.7 | ". 7" x 48" x 5.2mm, 5.2mm SPC + IXPE backing, 100% waterproof. Single price, no promo pair. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF108" t="inlineStr">
@@ -13045,7 +13045,7 @@
       </c>
       <c r="BC109" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANVIN - Vanetettpro SPC LVP -  (Irish Loft)  | #CAN.V.0.IriLof.7 |  -". 7" x 48" x 5.2mm, 5.2mm SPC + IXPE backing, 100% waterproof. Single price, no promo pair. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANVIN - Vanetettpro SPC LVP -  (Irish Loft)  | #CAN.V.0.IriLof.7 |  -". 7" x 48" x 5.2mm, 5.2mm SPC + IXPE backing, 100% waterproof. Single price, no promo pair. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF109" t="inlineStr">
@@ -13166,7 +13166,7 @@
       </c>
       <c r="BC110" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANVIN - Vanetettpro SPC LVP -  (Morning Coffee)  | #CAN.V.0.MorCof.7 ". 7" x 48" x 5.2mm, 5.2mm SPC + IXPE backing, 100% waterproof. Single price, no promo pair. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANVIN - Vanetettpro SPC LVP -  (Morning Coffee)  | #CAN.V.0.MorCof.7 ". 7" x 48" x 5.2mm, 5.2mm SPC + IXPE backing, 100% waterproof. Single price, no promo pair. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF110" t="inlineStr">
@@ -13287,7 +13287,7 @@
       </c>
       <c r="BC111" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANVIN - Vanetettpro SPC LVP -  (Nordic Loft)  | #CAN.V.0.NorLof.7 |  ". 7" x 48" x 5.2mm, 5.2mm SPC + IXPE backing, 100% waterproof. Single price, no promo pair. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANVIN - Vanetettpro SPC LVP -  (Nordic Loft)  | #CAN.V.0.NorLof.7 |  ". 7" x 48" x 5.2mm, 5.2mm SPC + IXPE backing, 100% waterproof. Single price, no promo pair. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF111" t="inlineStr">
@@ -13413,7 +13413,7 @@
       </c>
       <c r="BC112" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANVIN - Vanetettpro SPC LVP -  (Silver Leaf)  | #CAN.V.0.SilLea.7 |  ". 7" x 48" x 5.2mm, 5.2mm SPC + IXPE backing, 100% waterproof. Single price, no promo pair. Supplier marks this colour *DISCONTINUE ITEM* on the Aug 31 2026 list -&gt; Stock status = Discontinued, Active = FALSE. Confirm remaining stock before import. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANVIN - Vanetettpro SPC LVP -  (Silver Leaf)  | #CAN.V.0.SilLea.7 |  ". 7" x 48" x 5.2mm, 5.2mm SPC + IXPE backing, 100% waterproof. Single price, no promo pair. Supplier marks this colour *DISCONTINUE ITEM* on the Aug 31 2026 list -&gt; Stock status = Discontinued, Active = FALSE. Confirm remaining stock before import. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF112" t="inlineStr">
@@ -13539,7 +13539,7 @@
       </c>
       <c r="BC113" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANVIN - Vanetettpro SPC LVP -  (Swedish Brown)  | #CAN.V.0.SweBro.7 |". 7" x 48" x 5.2mm, 5.2mm SPC + IXPE backing, 100% waterproof. Single price, no promo pair. Supplier marks this colour *DISCONTINUE ITEM* on the Aug 31 2026 list -&gt; Stock status = Discontinued, Active = FALSE. Confirm remaining stock before import. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANVIN - Vanetettpro SPC LVP -  (Swedish Brown)  | #CAN.V.0.SweBro.7 |". 7" x 48" x 5.2mm, 5.2mm SPC + IXPE backing, 100% waterproof. Single price, no promo pair. Supplier marks this colour *DISCONTINUE ITEM* on the Aug 31 2026 list -&gt; Stock status = Discontinued, Active = FALSE. Confirm remaining stock before import. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF113" t="inlineStr">
@@ -13651,7 +13651,7 @@
       </c>
       <c r="BC114" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANHAR - Brand Coverings - Maple (Chelsea Grey) T&amp;G | #CAN.H.DM.CheGre". Solid hardwood T&amp;G. Material type left blank (solid hardwood has no core layer). '(Arc Saw &amp; Distressed)' is finish language with no word 'Grade' -&gt; Grade left blank, descriptors stored in Finish type. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANHAR - Brand Coverings - Maple (Chelsea Grey) T&amp;G | #CAN.H.DM.CheGre". Solid hardwood T&amp;G. Material type left blank (solid hardwood has no core layer). '(Arc Saw &amp; Distressed)' is finish language with no word 'Grade' -&gt; Grade left blank, descriptors stored in Finish type. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF114" t="inlineStr">
@@ -13763,7 +13763,7 @@
       </c>
       <c r="BC115" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANHAR - Brand Coverings - Maple (Kingsport) T&amp;G | #CAN.H.M.Kin.0 |  -". Solid hardwood T&amp;G. Material type left blank (solid hardwood has no core layer). '(Arc Saw &amp; Distressed)' is finish language with no word 'Grade' -&gt; Grade left blank, descriptors stored in Finish type. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANHAR - Brand Coverings - Maple (Kingsport) T&amp;G | #CAN.H.M.Kin.0 |  -". Solid hardwood T&amp;G. Material type left blank (solid hardwood has no core layer). '(Arc Saw &amp; Distressed)' is finish language with no word 'Grade' -&gt; Grade left blank, descriptors stored in Finish type. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF115" t="inlineStr">
@@ -13875,7 +13875,7 @@
       </c>
       <c r="BC116" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANHAR - Brand Coverings - Maple (Pale Oats) T&amp;G | #CAN.H.M.PalOat.0 |". Solid hardwood T&amp;G. Material type left blank (solid hardwood has no core layer). '(Arc Saw &amp; Distressed)' is finish language with no word 'Grade' -&gt; Grade left blank, descriptors stored in Finish type. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANHAR - Brand Coverings - Maple (Pale Oats) T&amp;G | #CAN.H.M.PalOat.0 |". Solid hardwood T&amp;G. Material type left blank (solid hardwood has no core layer). '(Arc Saw &amp; Distressed)' is finish language with no word 'Grade' -&gt; Grade left blank, descriptors stored in Finish type. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF116" t="inlineStr">
@@ -13992,7 +13992,7 @@
       </c>
       <c r="BC117" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANHAR - Brand Coverings - Maple (Roasted Marshmallow) T&amp;G | #CAN.H.DM". Solid hardwood T&amp;G. Material type left blank (solid hardwood has no core layer). '(Arc Saw &amp; Distressed)' is finish language with no word 'Grade' -&gt; Grade left blank, descriptors stored in Finish type. Supplier marks this colour *DISCONTINUE ITEM* on the Aug 31 2026 list -&gt; Stock status = Discontinued, Active = FALSE. Confirm remaining stock before import. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANHAR - Brand Coverings - Maple (Roasted Marshmallow) T&amp;G | #CAN.H.DM". Solid hardwood T&amp;G. Material type left blank (solid hardwood has no core layer). '(Arc Saw &amp; Distressed)' is finish language with no word 'Grade' -&gt; Grade left blank, descriptors stored in Finish type. Supplier marks this colour *DISCONTINUE ITEM* on the Aug 31 2026 list -&gt; Stock status = Discontinued, Active = FALSE. Confirm remaining stock before import. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF117" t="inlineStr">
@@ -14104,7 +14104,7 @@
       </c>
       <c r="BC118" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANHAR - Brand Coverings - Maple (Saybrook) T&amp;G | #CAN.H.M.Say.0 |  - ". Solid hardwood T&amp;G. Material type left blank (solid hardwood has no core layer). '(Arc Saw &amp; Distressed)' is finish language with no word 'Grade' -&gt; Grade left blank, descriptors stored in Finish type. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANHAR - Brand Coverings - Maple (Saybrook) T&amp;G | #CAN.H.M.Say.0 |  - ". Solid hardwood T&amp;G. Material type left blank (solid hardwood has no core layer). '(Arc Saw &amp; Distressed)' is finish language with no word 'Grade' -&gt; Grade left blank, descriptors stored in Finish type. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF118" t="inlineStr">
@@ -14216,7 +14216,7 @@
       </c>
       <c r="BC119" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour variant match to Lightspeed product "CANHAR - Brand Coverings - Teak (Loretto) T&amp;G | #CAN.H.T.Lor.4 |  - 4-". Solid hardwood T&amp;G. Material type left blank (solid hardwood has no core layer). COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour variant match to Lightspeed product "CANHAR - Brand Coverings - Teak (Loretto) T&amp;G | #CAN.H.T.Lor.4 |  - 4-". Solid hardwood T&amp;G. Material type left blank (solid hardwood has no core layer). COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF119" t="inlineStr">
@@ -14328,7 +14328,7 @@
       </c>
       <c r="BC120" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANHAR - Brand Coverings - Teak (Owen) T&amp;G | #CAN.H.T.Owe.4 |  - 4-3/4". Solid hardwood T&amp;G. Material type left blank (solid hardwood has no core layer). COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANHAR - Brand Coverings - Teak (Owen) T&amp;G | #CAN.H.T.Owe.4 |  - 4-3/4". Solid hardwood T&amp;G. Material type left blank (solid hardwood has no core layer). COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF120" t="inlineStr">
@@ -14440,7 +14440,7 @@
       </c>
       <c r="BC121" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANHAR - Brand Coverings - Teak (Maylis) T&amp;G | #CAN.H.T.May.4 |  - 4-3". Solid hardwood T&amp;G. Material type left blank (solid hardwood has no core layer). COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANHAR - Brand Coverings - Teak (Maylis) T&amp;G | #CAN.H.T.May.4 |  - 4-3". Solid hardwood T&amp;G. Material type left blank (solid hardwood has no core layer). COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF121" t="inlineStr">
@@ -14552,7 +14552,7 @@
       </c>
       <c r="BC122" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANHAR - Brand Coverings - Teak (Haley) T&amp;G | #CAN.H.T.Hal.4 |  - 4-3/". Solid hardwood T&amp;G. Material type left blank (solid hardwood has no core layer). COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANHAR - Brand Coverings - Teak (Haley) T&amp;G | #CAN.H.T.Hal.4 |  - 4-3/". Solid hardwood T&amp;G. Material type left blank (solid hardwood has no core layer). COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF122" t="inlineStr">
@@ -14664,7 +14664,7 @@
       </c>
       <c r="BC123" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANHAR - Brand Coverings - Teak (Rowan) T&amp;G | #CAN.H.T.Row.4 |  - 4-3/". Solid hardwood T&amp;G. Material type left blank (solid hardwood has no core layer). COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANHAR - Brand Coverings - Teak (Rowan) T&amp;G | #CAN.H.T.Row.4 |  - 4-3/". Solid hardwood T&amp;G. Material type left blank (solid hardwood has no core layer). COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF123" t="inlineStr">
@@ -14776,7 +14776,7 @@
       </c>
       <c r="BC124" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANHAR - Brand Coverings - Acacia (Metropolis) T&amp;G | #CAN.H.A.Met.4.1 ". Solid hardwood T&amp;G. Material type left blank (solid hardwood has no core layer). COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANHAR - Brand Coverings - Acacia (Metropolis) T&amp;G | #CAN.H.A.Met.4.1 ". Solid hardwood T&amp;G. Material type left blank (solid hardwood has no core layer). COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF124" t="inlineStr">
@@ -14888,7 +14888,7 @@
       </c>
       <c r="BC125" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANHAR - Brand Coverings - Acacia (Silver Fox) T&amp;G | #CAN.H.A.SilFox.4". Solid hardwood T&amp;G. Material type left blank (solid hardwood has no core layer). COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANHAR - Brand Coverings - Acacia (Silver Fox) T&amp;G | #CAN.H.A.SilFox.4". Solid hardwood T&amp;G. Material type left blank (solid hardwood has no core layer). COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF125" t="inlineStr">
@@ -15000,7 +15000,7 @@
       </c>
       <c r="BC126" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANHAR - Brand Coverings - Acacia (Smoke Infusion) T&amp;G | #CAN.H.A.SmoI". Solid hardwood T&amp;G. Material type left blank (solid hardwood has no core layer). COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANHAR - Brand Coverings - Acacia (Smoke Infusion) T&amp;G | #CAN.H.A.SmoI". Solid hardwood T&amp;G. Material type left blank (solid hardwood has no core layer). COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF126" t="inlineStr">
@@ -15107,7 +15107,7 @@
       </c>
       <c r="BC127" t="inlineStr">
         <is>
-          <t>Solid hardwood T&amp;G. Material type left blank (solid hardwood has no core layer). COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>Solid hardwood T&amp;G. Material type left blank (solid hardwood has no core layer). COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF127" t="inlineStr">
@@ -15219,7 +15219,7 @@
       </c>
       <c r="BC128" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANHAR - Brand Coverings - Distressed Hickory (Coffee Gelato) T&amp;G | #C". Solid hardwood T&amp;G. Material type left blank (solid hardwood has no core layer). Sheet labels the row 'Distressed Hickory (Handscraped)'. 'Distressed' appears without the word 'Grade' -&gt; finish language, NOT a grade: Grade left blank, both descriptors in Finish type. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANHAR - Brand Coverings - Distressed Hickory (Coffee Gelato) T&amp;G | #C". Solid hardwood T&amp;G. Material type left blank (solid hardwood has no core layer). Sheet labels the row 'Distressed Hickory (Handscraped)'. 'Distressed' appears without the word 'Grade' -&gt; finish language, NOT a grade: Grade left blank, both descriptors in Finish type. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF128" t="inlineStr">
@@ -15331,7 +15331,7 @@
       </c>
       <c r="BC129" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANHAR - Brand Coverings - Distressed Hickory (Gingerbread) T&amp;G | #CAN". Solid hardwood T&amp;G. Material type left blank (solid hardwood has no core layer). Sheet labels the row 'Distressed Hickory (Handscraped)'. 'Distressed' appears without the word 'Grade' -&gt; finish language, NOT a grade: Grade left blank, both descriptors in Finish type. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANHAR - Brand Coverings - Distressed Hickory (Gingerbread) T&amp;G | #CAN". Solid hardwood T&amp;G. Material type left blank (solid hardwood has no core layer). Sheet labels the row 'Distressed Hickory (Handscraped)'. 'Distressed' appears without the word 'Grade' -&gt; finish language, NOT a grade: Grade left blank, both descriptors in Finish type. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF129" t="inlineStr">
@@ -15443,7 +15443,7 @@
       </c>
       <c r="BC130" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANHAR - Brand Coverings - Distressed Hickory (Madison Avenue) T&amp;G | #". Solid hardwood T&amp;G. Material type left blank (solid hardwood has no core layer). Sheet labels the row 'Distressed Hickory (Handscraped)'. 'Distressed' appears without the word 'Grade' -&gt; finish language, NOT a grade: Grade left blank, both descriptors in Finish type. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANHAR - Brand Coverings - Distressed Hickory (Madison Avenue) T&amp;G | #". Solid hardwood T&amp;G. Material type left blank (solid hardwood has no core layer). Sheet labels the row 'Distressed Hickory (Handscraped)'. 'Distressed' appears without the word 'Grade' -&gt; finish language, NOT a grade: Grade left blank, both descriptors in Finish type. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF130" t="inlineStr">
@@ -15555,7 +15555,7 @@
       </c>
       <c r="BC131" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANHAR - Brand Coverings - White Oak (Alexanian) T&amp;G | #CAN.H.WO.Ale.5". Solid hardwood T&amp;G. Material type left blank (solid hardwood has no core layer). COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANHAR - Brand Coverings - White Oak (Alexanian) T&amp;G | #CAN.H.WO.Ale.5". Solid hardwood T&amp;G. Material type left blank (solid hardwood has no core layer). COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF131" t="inlineStr">
@@ -15667,7 +15667,7 @@
       </c>
       <c r="BC132" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANHAR - Brand Coverings - White Oak (Granite Dust) T&amp;G | #CAN.H.WO.Gr". Solid hardwood T&amp;G. Material type left blank (solid hardwood has no core layer). COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANHAR - Brand Coverings - White Oak (Granite Dust) T&amp;G | #CAN.H.WO.Gr". Solid hardwood T&amp;G. Material type left blank (solid hardwood has no core layer). COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF132" t="inlineStr">
@@ -15779,7 +15779,7 @@
       </c>
       <c r="BC133" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANHAR - Brand Coverings - White Oak (Princeton) T&amp;G | #CAN.H.WO.Pri.5". Solid hardwood T&amp;G. Material type left blank (solid hardwood has no core layer). COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANHAR - Brand Coverings - White Oak (Princeton) T&amp;G | #CAN.H.WO.Pri.5". Solid hardwood T&amp;G. Material type left blank (solid hardwood has no core layer). COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF133" t="inlineStr">
@@ -15891,7 +15891,7 @@
       </c>
       <c r="BC134" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour variant match to Lightspeed product "CANHAR - Brand Coverings - White Oak (Smoke Expose) T&amp;G | #CAN.H.WO.Sm". Solid hardwood T&amp;G. Material type left blank (solid hardwood has no core layer). COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour variant match to Lightspeed product "CANHAR - Brand Coverings - White Oak (Smoke Expose) T&amp;G | #CAN.H.WO.Sm". Solid hardwood T&amp;G. Material type left blank (solid hardwood has no core layer). COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF134" t="inlineStr">
@@ -16003,7 +16003,7 @@
       </c>
       <c r="BC135" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANHAR - Brand Coverings - White Oak (Smoked Tobacco) T&amp;G | #CAN.H.WO.". Solid hardwood T&amp;G. Material type left blank (solid hardwood has no core layer). COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANHAR - Brand Coverings - White Oak (Smoked Tobacco) T&amp;G | #CAN.H.WO.". Solid hardwood T&amp;G. Material type left blank (solid hardwood has no core layer). COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF135" t="inlineStr">
@@ -16115,7 +16115,7 @@
       </c>
       <c r="BC136" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Brand Surfaces (Click) - Maple (Berkeley) Click | #CAN.E.M.Be". Brand Surfaces 'Engineered Click' - floating click engineered. 'New Arrival'. 6.5" x 1/2" x RL. Sits under a 'Promotion Valid until October 31, 2026' section header but prints only ONE price - treated as a regular price, no promo fields applied. Confirm with supplier. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Brand Surfaces (Click) - Maple (Berkeley) Click | #CAN.E.M.Be". Brand Surfaces 'Engineered Click' - floating click engineered. 'New Arrival'. 6.5" x 1/2" x RL. Sits under a 'Promotion Valid until October 31, 2026' section header but prints only ONE price - treated as a regular price, no promo fields applied. Confirm with supplier. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF136" t="inlineStr">
@@ -16227,7 +16227,7 @@
       </c>
       <c r="BC137" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Brand Surfaces (Click) - Maple (Santee) Click | #CAN.E.M.San.". Brand Surfaces 'Engineered Click' - floating click engineered. 'New Arrival'. 6.5" x 1/2" x RL. Sits under a 'Promotion Valid until October 31, 2026' section header but prints only ONE price - treated as a regular price, no promo fields applied. Confirm with supplier. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Brand Surfaces (Click) - Maple (Santee) Click | #CAN.E.M.San.". Brand Surfaces 'Engineered Click' - floating click engineered. 'New Arrival'. 6.5" x 1/2" x RL. Sits under a 'Promotion Valid until October 31, 2026' section header but prints only ONE price - treated as a regular price, no promo fields applied. Confirm with supplier. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF137" t="inlineStr">
@@ -16339,7 +16339,7 @@
       </c>
       <c r="BC138" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Brand Surfaces (Click) - Maple (Sequoia) Click | #CAN.E.M.Seq". Brand Surfaces 'Engineered Click' - floating click engineered. 'New Arrival'. 6.5" x 1/2" x RL. Sits under a 'Promotion Valid until October 31, 2026' section header but prints only ONE price - treated as a regular price, no promo fields applied. Confirm with supplier. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Brand Surfaces (Click) - Maple (Sequoia) Click | #CAN.E.M.Seq". Brand Surfaces 'Engineered Click' - floating click engineered. 'New Arrival'. 6.5" x 1/2" x RL. Sits under a 'Promotion Valid until October 31, 2026' section header but prints only ONE price - treated as a regular price, no promo fields applied. Confirm with supplier. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF138" t="inlineStr">
@@ -16451,7 +16451,7 @@
       </c>
       <c r="BC139" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Brand Surfaces (Click) - Maple (La Jolla) Click | #CAN.E.M.La". Brand Surfaces 'Engineered Click' - floating click engineered. 'New Arrival'. 6.5" x 1/2" x RL. Sits under a 'Promotion Valid until October 31, 2026' section header but prints only ONE price - treated as a regular price, no promo fields applied. Confirm with supplier. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Brand Surfaces (Click) - Maple (La Jolla) Click | #CAN.E.M.La". Brand Surfaces 'Engineered Click' - floating click engineered. 'New Arrival'. 6.5" x 1/2" x RL. Sits under a 'Promotion Valid until October 31, 2026' section header but prints only ONE price - treated as a regular price, no promo fields applied. Confirm with supplier. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF139" t="inlineStr">
@@ -16563,7 +16563,7 @@
       </c>
       <c r="BC140" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Brand Surfaces (Click) - HDF Hickory (Boston Legacy) Click | ". Brand Surfaces 'Engineered Click' - floating click engineered. 6.5" x 3/8" x RL. Sheet annotates this sub-group '(HDF)' -&gt; Material type = HDF core (the only Brand Surfaces group with an HDF core; the rest are hardwood plywood). Sits under a 'Promotion Valid until October 31, 2026' section header but prints only ONE price - treated as a regular price, no promo fields applied. Confirm with supplier. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Brand Surfaces (Click) - HDF Hickory (Boston Legacy) Click | ". Brand Surfaces 'Engineered Click' - floating click engineered. 6.5" x 3/8" x RL. Sheet annotates this sub-group '(HDF)' -&gt; Material type = HDF core (the only Brand Surfaces group with an HDF core; the rest are hardwood plywood). Sits under a 'Promotion Valid until October 31, 2026' section header but prints only ONE price - treated as a regular price, no promo fields applied. Confirm with supplier. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF140" t="inlineStr">
@@ -16675,7 +16675,7 @@
       </c>
       <c r="BC141" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Brand Surfaces (Click) - HDF Hickory (Parisian House) Click |". Brand Surfaces 'Engineered Click' - floating click engineered. 6.5" x 3/8" x RL. Sheet annotates this sub-group '(HDF)' -&gt; Material type = HDF core (the only Brand Surfaces group with an HDF core; the rest are hardwood plywood). Sits under a 'Promotion Valid until October 31, 2026' section header but prints only ONE price - treated as a regular price, no promo fields applied. Confirm with supplier. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Brand Surfaces (Click) - HDF Hickory (Parisian House) Click |". Brand Surfaces 'Engineered Click' - floating click engineered. 6.5" x 3/8" x RL. Sheet annotates this sub-group '(HDF)' -&gt; Material type = HDF core (the only Brand Surfaces group with an HDF core; the rest are hardwood plywood). Sits under a 'Promotion Valid until October 31, 2026' section header but prints only ONE price - treated as a regular price, no promo fields applied. Confirm with supplier. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF141" t="inlineStr">
@@ -16787,7 +16787,7 @@
       </c>
       <c r="BC142" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Brand Surfaces (Click) - HDF Hickory (Oregon Coast) Click | #". Brand Surfaces 'Engineered Click' - floating click engineered. 6.5" x 3/8" x RL. Sheet annotates this sub-group '(HDF)' -&gt; Material type = HDF core (the only Brand Surfaces group with an HDF core; the rest are hardwood plywood). Sits under a 'Promotion Valid until October 31, 2026' section header but prints only ONE price - treated as a regular price, no promo fields applied. Confirm with supplier. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Brand Surfaces (Click) - HDF Hickory (Oregon Coast) Click | #". Brand Surfaces 'Engineered Click' - floating click engineered. 6.5" x 3/8" x RL. Sheet annotates this sub-group '(HDF)' -&gt; Material type = HDF core (the only Brand Surfaces group with an HDF core; the rest are hardwood plywood). Sits under a 'Promotion Valid until October 31, 2026' section header but prints only ONE price - treated as a regular price, no promo fields applied. Confirm with supplier. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF142" t="inlineStr">
@@ -16899,7 +16899,7 @@
       </c>
       <c r="BC143" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Brand Surfaces (Click) - HDF Hickory (Sapphire Grey) Click | ". Brand Surfaces 'Engineered Click' - floating click engineered. 6.5" x 3/8" x RL. Sheet annotates this sub-group '(HDF)' -&gt; Material type = HDF core (the only Brand Surfaces group with an HDF core; the rest are hardwood plywood). Sits under a 'Promotion Valid until October 31, 2026' section header but prints only ONE price - treated as a regular price, no promo fields applied. Confirm with supplier. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Brand Surfaces (Click) - HDF Hickory (Sapphire Grey) Click | ". Brand Surfaces 'Engineered Click' - floating click engineered. 6.5" x 3/8" x RL. Sheet annotates this sub-group '(HDF)' -&gt; Material type = HDF core (the only Brand Surfaces group with an HDF core; the rest are hardwood plywood). Sits under a 'Promotion Valid until October 31, 2026' section header but prints only ONE price - treated as a regular price, no promo fields applied. Confirm with supplier. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF143" t="inlineStr">
@@ -17011,7 +17011,7 @@
       </c>
       <c r="BC144" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Brand Surfaces (Click) - HDF Hickory (Wooden Wagon) Click | #". Brand Surfaces 'Engineered Click' - floating click engineered. 6.5" x 3/8" x RL. Sheet annotates this sub-group '(HDF)' -&gt; Material type = HDF core (the only Brand Surfaces group with an HDF core; the rest are hardwood plywood). Sits under a 'Promotion Valid until October 31, 2026' section header but prints only ONE price - treated as a regular price, no promo fields applied. Confirm with supplier. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Brand Surfaces (Click) - HDF Hickory (Wooden Wagon) Click | #". Brand Surfaces 'Engineered Click' - floating click engineered. 6.5" x 3/8" x RL. Sheet annotates this sub-group '(HDF)' -&gt; Material type = HDF core (the only Brand Surfaces group with an HDF core; the rest are hardwood plywood). Sits under a 'Promotion Valid until October 31, 2026' section header but prints only ONE price - treated as a regular price, no promo fields applied. Confirm with supplier. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF144" t="inlineStr">
@@ -17136,7 +17136,7 @@
       </c>
       <c r="BC145" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANENG - Brand Surfaces (Click) - Hickory (Morro Bay) Click | #CAN". Brand Surfaces 'Engineered Click' - floating click engineered. 6.5" x 1/2" x RL. PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANENG - Brand Surfaces (Click) - Hickory (Morro Bay) Click | #CAN". Brand Surfaces 'Engineered Click' - floating click engineered. 6.5" x 1/2" x RL. PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF145" t="inlineStr">
@@ -17261,7 +17261,7 @@
       </c>
       <c r="BC146" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANENG - Brand Surfaces (Click) - Hickory (Ventura) Click | #CAN.E". Brand Surfaces 'Engineered Click' - floating click engineered. 6.5" x 1/2" x RL. PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANENG - Brand Surfaces (Click) - Hickory (Ventura) Click | #CAN.E". Brand Surfaces 'Engineered Click' - floating click engineered. 6.5" x 1/2" x RL. PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF146" t="inlineStr">
@@ -17386,7 +17386,7 @@
       </c>
       <c r="BC147" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANENG - Brand Surfaces (Click) - Hickory (Great Sur) Click | #CAN". Brand Surfaces 'Engineered Click' - floating click engineered. 6.5" x 1/2" x RL. PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANENG - Brand Surfaces (Click) - Hickory (Great Sur) Click | #CAN". Brand Surfaces 'Engineered Click' - floating click engineered. 6.5" x 1/2" x RL. PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF147" t="inlineStr">
@@ -17511,7 +17511,7 @@
       </c>
       <c r="BC148" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANENG - Brand Surfaces (Click) - Hickory (Summerland) Click | #CA". Brand Surfaces 'Engineered Click' - floating click engineered. 6.5" x 1/2" x RL. PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANENG - Brand Surfaces (Click) - Hickory (Summerland) Click | #CA". Brand Surfaces 'Engineered Click' - floating click engineered. 6.5" x 1/2" x RL. PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF148" t="inlineStr">
@@ -17636,7 +17636,7 @@
       </c>
       <c r="BC149" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANENG - Brand Surfaces (Click) - Hickory (Baywood) Click | #CAN.E". Brand Surfaces 'Engineered Click' - floating click engineered. 6.5" x 1/2" x RL. PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANENG - Brand Surfaces (Click) - Hickory (Baywood) Click | #CAN.E". Brand Surfaces 'Engineered Click' - floating click engineered. 6.5" x 1/2" x RL. PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF149" t="inlineStr">
@@ -17761,7 +17761,7 @@
       </c>
       <c r="BC150" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANENG - Brand Surfaces (Click) - Oak (Sausalito) Click | #CAN.E.O". Brand Surfaces 'Engineered Click' - floating click engineered. 6.5" x 1/2" x RL. PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANENG - Brand Surfaces (Click) - Oak (Sausalito) Click | #CAN.E.O". Brand Surfaces 'Engineered Click' - floating click engineered. 6.5" x 1/2" x RL. PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF150" t="inlineStr">
@@ -17886,7 +17886,7 @@
       </c>
       <c r="BC151" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANENG - Brand Surfaces (Click) - Oak (Moss Landing) Click | #CAN.". Brand Surfaces 'Engineered Click' - floating click engineered. 6.5" x 1/2" x RL. PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANENG - Brand Surfaces (Click) - Oak (Moss Landing) Click | #CAN.". Brand Surfaces 'Engineered Click' - floating click engineered. 6.5" x 1/2" x RL. PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF151" t="inlineStr">
@@ -18011,7 +18011,7 @@
       </c>
       <c r="BC152" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANENG - Brand Surfaces (Click) - Oak (Monterey) Click | #CAN.E.O.". Brand Surfaces 'Engineered Click' - floating click engineered. 6.5" x 1/2" x RL. PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANENG - Brand Surfaces (Click) - Oak (Monterey) Click | #CAN.E.O.". Brand Surfaces 'Engineered Click' - floating click engineered. 6.5" x 1/2" x RL. PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF152" t="inlineStr">
@@ -18136,7 +18136,7 @@
       </c>
       <c r="BC153" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANENG - Brand Surfaces (Click) - Oak (Santa Maria) Click | #CAN.E". Brand Surfaces 'Engineered Click' - floating click engineered. 6.5" x 1/2" x RL. PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANENG - Brand Surfaces (Click) - Oak (Santa Maria) Click | #CAN.E". Brand Surfaces 'Engineered Click' - floating click engineered. 6.5" x 1/2" x RL. PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF153" t="inlineStr">
@@ -18261,7 +18261,7 @@
       </c>
       <c r="BC154" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANENG - Brand Surfaces (Click) - Oak (Napa Valley) Click | #CAN.E". Brand Surfaces 'Engineered Click' - floating click engineered. 6.5" x 1/2" x RL. PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANENG - Brand Surfaces (Click) - Oak (Napa Valley) Click | #CAN.E". Brand Surfaces 'Engineered Click' - floating click engineered. 6.5" x 1/2" x RL. PROMO: sheet prints paired Promotion/Regular prices under 'Promotion Valid until October 31, 2026'. Cost = Regular, Promo cost = Promotion, Promo end date = 2026-10-31 (printed window). COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF154" t="inlineStr">
@@ -18378,7 +18378,7 @@
       </c>
       <c r="BC155" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Brand Surfaces (Click) - Oak (Midtown Brown) Click | #CAN.E.O". Brand Surfaces 'Engineered Click' - floating click engineered. 6" x 1/2" x RL. AMBIGUOUS LAYOUT: one price cell ($3.69) and one size cell span seven colours, but TWO box-size cells (29.70 and 34.36 sf/box) sit inside the block; split into two box-size sub-groups by vertical alignment (FAW multi-sub-group precedent). Confirm which colours box at which size. Sits under a 'Promotion Valid until October 31, 2026' section header but prints only ONE price - treated as a regular price, no promo fields applied. Confirm with supplier. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Brand Surfaces (Click) - Oak (Midtown Brown) Click | #CAN.E.O". Brand Surfaces 'Engineered Click' - floating click engineered. 6" x 1/2" x RL. AMBIGUOUS LAYOUT: one price cell ($3.69) and one size cell span seven colours, but TWO box-size cells (29.70 and 34.36 sf/box) sit inside the block; split into two box-size sub-groups by vertical alignment (FAW multi-sub-group precedent). Confirm which colours box at which size. Sits under a 'Promotion Valid until October 31, 2026' section header but prints only ONE price - treated as a regular price, no promo fields applied. Confirm with supplier. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF155" t="inlineStr">
@@ -18495,7 +18495,7 @@
       </c>
       <c r="BC156" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Brand Surfaces (Click) - Oak (Whisper White) Click | #CAN.E.O". Brand Surfaces 'Engineered Click' - floating click engineered. 6" x 1/2" x RL. AMBIGUOUS LAYOUT: one price cell ($3.69) and one size cell span seven colours, but TWO box-size cells (29.70 and 34.36 sf/box) sit inside the block; split into two box-size sub-groups by vertical alignment (FAW multi-sub-group precedent). Confirm which colours box at which size. Sits under a 'Promotion Valid until October 31, 2026' section header but prints only ONE price - treated as a regular price, no promo fields applied. Confirm with supplier. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Brand Surfaces (Click) - Oak (Whisper White) Click | #CAN.E.O". Brand Surfaces 'Engineered Click' - floating click engineered. 6" x 1/2" x RL. AMBIGUOUS LAYOUT: one price cell ($3.69) and one size cell span seven colours, but TWO box-size cells (29.70 and 34.36 sf/box) sit inside the block; split into two box-size sub-groups by vertical alignment (FAW multi-sub-group precedent). Confirm which colours box at which size. Sits under a 'Promotion Valid until October 31, 2026' section header but prints only ONE price - treated as a regular price, no promo fields applied. Confirm with supplier. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF156" t="inlineStr">
@@ -18612,7 +18612,7 @@
       </c>
       <c r="BC157" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Brand Surfaces (Click) - Oak (Offshore Grey) Click | #CAN.E.O". Brand Surfaces 'Engineered Click' - floating click engineered. 6" x 1/2" x RL. AMBIGUOUS LAYOUT: one price cell ($3.69) and one size cell span seven colours, but TWO box-size cells (29.70 and 34.36 sf/box) sit inside the block; split into two box-size sub-groups by vertical alignment (FAW multi-sub-group precedent). Confirm which colours box at which size. Sits under a 'Promotion Valid until October 31, 2026' section header but prints only ONE price - treated as a regular price, no promo fields applied. Confirm with supplier. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Brand Surfaces (Click) - Oak (Offshore Grey) Click | #CAN.E.O". Brand Surfaces 'Engineered Click' - floating click engineered. 6" x 1/2" x RL. AMBIGUOUS LAYOUT: one price cell ($3.69) and one size cell span seven colours, but TWO box-size cells (29.70 and 34.36 sf/box) sit inside the block; split into two box-size sub-groups by vertical alignment (FAW multi-sub-group precedent). Confirm which colours box at which size. Sits under a 'Promotion Valid until October 31, 2026' section header but prints only ONE price - treated as a regular price, no promo fields applied. Confirm with supplier. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF157" t="inlineStr">
@@ -18729,7 +18729,7 @@
       </c>
       <c r="BC158" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Brand Surfaces (Click) - Oak (Park Avenue) Click | #CAN.E.O.P". Brand Surfaces 'Engineered Click' - floating click engineered. 6" x 1/2" x RL. AMBIGUOUS LAYOUT: one price cell ($3.69) and one size cell span seven colours, but TWO box-size cells (29.70 and 34.36 sf/box) sit inside the block; split into two box-size sub-groups by vertical alignment (FAW multi-sub-group precedent). Confirm which colours box at which size. Sits under a 'Promotion Valid until October 31, 2026' section header but prints only ONE price - treated as a regular price, no promo fields applied. Confirm with supplier. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Brand Surfaces (Click) - Oak (Park Avenue) Click | #CAN.E.O.P". Brand Surfaces 'Engineered Click' - floating click engineered. 6" x 1/2" x RL. AMBIGUOUS LAYOUT: one price cell ($3.69) and one size cell span seven colours, but TWO box-size cells (29.70 and 34.36 sf/box) sit inside the block; split into two box-size sub-groups by vertical alignment (FAW multi-sub-group precedent). Confirm which colours box at which size. Sits under a 'Promotion Valid until October 31, 2026' section header but prints only ONE price - treated as a regular price, no promo fields applied. Confirm with supplier. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF158" t="inlineStr">
@@ -18846,7 +18846,7 @@
       </c>
       <c r="BC159" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Brand Surfaces (Click) - Oak (Eclectic Grey) Click | #CAN.E.O". Brand Surfaces 'Engineered Click' - floating click engineered. 6" x 1/2" x RL. AMBIGUOUS LAYOUT: one price cell ($3.69) and one size cell span seven colours, but TWO box-size cells (29.70 and 34.36 sf/box) sit inside the block; split into two box-size sub-groups by vertical alignment (FAW multi-sub-group precedent). Confirm which colours box at which size. Sits under a 'Promotion Valid until October 31, 2026' section header but prints only ONE price - treated as a regular price, no promo fields applied. Confirm with supplier. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Brand Surfaces (Click) - Oak (Eclectic Grey) Click | #CAN.E.O". Brand Surfaces 'Engineered Click' - floating click engineered. 6" x 1/2" x RL. AMBIGUOUS LAYOUT: one price cell ($3.69) and one size cell span seven colours, but TWO box-size cells (29.70 and 34.36 sf/box) sit inside the block; split into two box-size sub-groups by vertical alignment (FAW multi-sub-group precedent). Confirm which colours box at which size. Sits under a 'Promotion Valid until October 31, 2026' section header but prints only ONE price - treated as a regular price, no promo fields applied. Confirm with supplier. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF159" t="inlineStr">
@@ -18963,7 +18963,7 @@
       </c>
       <c r="BC160" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Brand Surfaces (Click) - Oak (Margaret) Click | #CAN.E.O.Mar.". Brand Surfaces 'Engineered Click' - floating click engineered. 6" x 1/2" x RL. AMBIGUOUS LAYOUT: one price cell ($3.69) and one size cell span seven colours, but TWO box-size cells (29.70 and 34.36 sf/box) sit inside the block; split into two box-size sub-groups by vertical alignment (FAW multi-sub-group precedent). Confirm which colours box at which size. Sits under a 'Promotion Valid until October 31, 2026' section header but prints only ONE price - treated as a regular price, no promo fields applied. Confirm with supplier. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Brand Surfaces (Click) - Oak (Margaret) Click | #CAN.E.O.Mar.". Brand Surfaces 'Engineered Click' - floating click engineered. 6" x 1/2" x RL. AMBIGUOUS LAYOUT: one price cell ($3.69) and one size cell span seven colours, but TWO box-size cells (29.70 and 34.36 sf/box) sit inside the block; split into two box-size sub-groups by vertical alignment (FAW multi-sub-group precedent). Confirm which colours box at which size. Sits under a 'Promotion Valid until October 31, 2026' section header but prints only ONE price - treated as a regular price, no promo fields applied. Confirm with supplier. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF160" t="inlineStr">
@@ -19080,7 +19080,7 @@
       </c>
       <c r="BC161" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Brand Surfaces (Click) - Oak (Wesley) Click | #CAN.E.O.Wes.6 ". Brand Surfaces 'Engineered Click' - floating click engineered. 6" x 1/2" x RL. AMBIGUOUS LAYOUT: one price cell ($3.69) and one size cell span seven colours, but TWO box-size cells (29.70 and 34.36 sf/box) sit inside the block; split into two box-size sub-groups by vertical alignment (FAW multi-sub-group precedent). Confirm which colours box at which size. Sits under a 'Promotion Valid until October 31, 2026' section header but prints only ONE price - treated as a regular price, no promo fields applied. Confirm with supplier. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Brand Surfaces (Click) - Oak (Wesley) Click | #CAN.E.O.Wes.6 ". Brand Surfaces 'Engineered Click' - floating click engineered. 6" x 1/2" x RL. AMBIGUOUS LAYOUT: one price cell ($3.69) and one size cell span seven colours, but TWO box-size cells (29.70 and 34.36 sf/box) sit inside the block; split into two box-size sub-groups by vertical alignment (FAW multi-sub-group precedent). Confirm which colours box at which size. Sits under a 'Promotion Valid until October 31, 2026' section header but prints only ONE price - treated as a regular price, no promo fields applied. Confirm with supplier. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF161" t="inlineStr">
@@ -19197,7 +19197,7 @@
       </c>
       <c r="BC162" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Brand Surfaces (T&amp;G) - Hickory (Crafted Timber) T&amp;G | #CAN.E.". Brand Surfaces 'Engineered T&amp;G'. No promotion header on this section. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Brand Surfaces (T&amp;G) - Hickory (Crafted Timber) T&amp;G | #CAN.E.". Brand Surfaces 'Engineered T&amp;G'. No promotion header on this section. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF162" t="inlineStr">
@@ -19314,7 +19314,7 @@
       </c>
       <c r="BC163" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Brand Surfaces (T&amp;G) - Hickory (Smoked Tree Trunk) T&amp;G | #CAN". Brand Surfaces 'Engineered T&amp;G'. No promotion header on this section. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Brand Surfaces (T&amp;G) - Hickory (Smoked Tree Trunk) T&amp;G | #CAN". Brand Surfaces 'Engineered T&amp;G'. No promotion header on this section. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF163" t="inlineStr">
@@ -19431,7 +19431,7 @@
       </c>
       <c r="BC164" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Brand Surfaces (T&amp;G) - Hickory (Smoky Shadow) T&amp;G | #CAN.E.H.". Brand Surfaces 'Engineered T&amp;G'. No promotion header on this section. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Brand Surfaces (T&amp;G) - Hickory (Smoky Shadow) T&amp;G | #CAN.E.H.". Brand Surfaces 'Engineered T&amp;G'. No promotion header on this section. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF164" t="inlineStr">
@@ -19548,7 +19548,7 @@
       </c>
       <c r="BC165" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Brand Surfaces (T&amp;G) - Hickory (Transitional Grey) T&amp;G | #CAN". Brand Surfaces 'Engineered T&amp;G'. No promotion header on this section. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Brand Surfaces (T&amp;G) - Hickory (Transitional Grey) T&amp;G | #CAN". Brand Surfaces 'Engineered T&amp;G'. No promotion header on this section. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF165" t="inlineStr">
@@ -19660,7 +19660,7 @@
       </c>
       <c r="BC166" t="inlineStr">
         <is>
-          <t>Brand Surfaces 'Engineered T&amp;G'. No promotion header on this section. AMBIGUOUS: the sheet repeats 'Crafted Timber' and 'Smoked Tree Trunk' a second time with a leading asterisk and a different box size (19.53 vs 19.5 sf/box), same price and spec. Both sub-groups created (FAW 'Tobermory duplicate' precedent); asterisk preserved in the colour name. Confirm with the rep whether these are two real products or a sheet duplication. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>Brand Surfaces 'Engineered T&amp;G'. No promotion header on this section. AMBIGUOUS: the sheet repeats 'Crafted Timber' and 'Smoked Tree Trunk' a second time with a leading asterisk and a different box size (19.53 vs 19.5 sf/box), same price and spec. Both sub-groups created (FAW 'Tobermory duplicate' precedent); asterisk preserved in the colour name. Confirm with the rep whether these are two real products or a sheet duplication. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF166" t="inlineStr">
@@ -19772,7 +19772,7 @@
       </c>
       <c r="BC167" t="inlineStr">
         <is>
-          <t>Brand Surfaces 'Engineered T&amp;G'. No promotion header on this section. AMBIGUOUS: the sheet repeats 'Crafted Timber' and 'Smoked Tree Trunk' a second time with a leading asterisk and a different box size (19.53 vs 19.5 sf/box), same price and spec. Both sub-groups created (FAW 'Tobermory duplicate' precedent); asterisk preserved in the colour name. Confirm with the rep whether these are two real products or a sheet duplication. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>Brand Surfaces 'Engineered T&amp;G'. No promotion header on this section. AMBIGUOUS: the sheet repeats 'Crafted Timber' and 'Smoked Tree Trunk' a second time with a leading asterisk and a different box size (19.53 vs 19.5 sf/box), same price and spec. Both sub-groups created (FAW 'Tobermory duplicate' precedent); asterisk preserved in the colour name. Confirm with the rep whether these are two real products or a sheet duplication. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF167" t="inlineStr">
@@ -19889,7 +19889,7 @@
       </c>
       <c r="BC168" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Brand Surfaces (T&amp;G) - Oak (Cobblestone) T&amp;G | #CAN.E.O.Cob.6". Brand Surfaces 'Engineered T&amp;G'. No promotion header on this section. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Brand Surfaces (T&amp;G) - Oak (Cobblestone) T&amp;G | #CAN.E.O.Cob.6". Brand Surfaces 'Engineered T&amp;G'. No promotion header on this section. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF168" t="inlineStr">
@@ -20011,7 +20011,7 @@
       </c>
       <c r="BC169" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Brand Surfaces (T&amp;G) - Oak (Pure Smoked) T&amp;G | #CAN.E.O.PurSm". Brand Surfaces 'Engineered T&amp;G'. No promotion header on this section. Supplier marks this colour *DISCONTINUE ITEM* on the Aug 31 2026 list -&gt; Stock status = Discontinued, Active = FALSE. Confirm remaining stock before import. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Brand Surfaces (T&amp;G) - Oak (Pure Smoked) T&amp;G | #CAN.E.O.PurSm". Brand Surfaces 'Engineered T&amp;G'. No promotion header on this section. Supplier marks this colour *DISCONTINUE ITEM* on the Aug 31 2026 list -&gt; Stock status = Discontinued, Active = FALSE. Confirm remaining stock before import. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF169" t="inlineStr">
@@ -20128,7 +20128,7 @@
       </c>
       <c r="BC170" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Brand Surfaces (T&amp;G) - Oak (Vintage Boulder) T&amp;G | #CAN.E.O.V". Brand Surfaces 'Engineered T&amp;G'. No promotion header on this section. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Brand Surfaces (T&amp;G) - Oak (Vintage Boulder) T&amp;G | #CAN.E.O.V". Brand Surfaces 'Engineered T&amp;G'. No promotion header on this section. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF170" t="inlineStr">
@@ -20250,7 +20250,7 @@
       </c>
       <c r="BC171" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Brand Surfaces (T&amp;G) - Oak (Smoked Accent) T&amp;G | #CAN.E.O.Smo". Brand Surfaces 'Engineered T&amp;G'. No promotion header on this section. Supplier marks this colour *DISCONTINUE ITEM* on the Aug 31 2026 list -&gt; Stock status = Discontinued, Active = FALSE. Confirm remaining stock before import. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Brand Surfaces (T&amp;G) - Oak (Smoked Accent) T&amp;G | #CAN.E.O.Smo". Brand Surfaces 'Engineered T&amp;G'. No promotion header on this section. Supplier marks this colour *DISCONTINUE ITEM* on the Aug 31 2026 list -&gt; Stock status = Discontinued, Active = FALSE. Confirm remaining stock before import. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF171" t="inlineStr">
@@ -20367,7 +20367,7 @@
       </c>
       <c r="BC172" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Brand Surfaces (T&amp;G) - Oak (Dusty Lead) T&amp;G | #CAN.E.O.DusLea". Brand Surfaces 'Engineered T&amp;G'. No promotion header on this section. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Brand Surfaces (T&amp;G) - Oak (Dusty Lead) T&amp;G | #CAN.E.O.DusLea". Brand Surfaces 'Engineered T&amp;G'. No promotion header on this section. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF172" t="inlineStr">
@@ -20484,7 +20484,7 @@
       </c>
       <c r="BC173" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Brand Surfaces (T&amp;G) - Oak (Elusive Forest) T&amp;G | #CAN.E.O.El". Brand Surfaces 'Engineered T&amp;G'. No promotion header on this section. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Brand Surfaces (T&amp;G) - Oak (Elusive Forest) T&amp;G | #CAN.E.O.El". Brand Surfaces 'Engineered T&amp;G'. No promotion header on this section. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF173" t="inlineStr">
@@ -20601,7 +20601,7 @@
       </c>
       <c r="BC174" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Brand Surfaces (T&amp;G) - Oak (Grind Concrete) T&amp;G | #CAN.E.O.Gr". Brand Surfaces 'Engineered T&amp;G'. No promotion header on this section. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Brand Surfaces (T&amp;G) - Oak (Grind Concrete) T&amp;G | #CAN.E.O.Gr". Brand Surfaces 'Engineered T&amp;G'. No promotion header on this section. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF174" t="inlineStr">
@@ -20723,7 +20723,7 @@
       </c>
       <c r="BC175" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Brand Surfaces (T&amp;G) - Oak (Satin Snow) T&amp;G | #CAN.E.O.SatSno". Brand Surfaces 'Engineered T&amp;G'. No promotion header on this section. Supplier marks this colour *DISCONTINUE ITEM* on the Aug 31 2026 list -&gt; Stock status = Discontinued, Active = FALSE. Confirm remaining stock before import. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Brand Surfaces (T&amp;G) - Oak (Satin Snow) T&amp;G | #CAN.E.O.SatSno". Brand Surfaces 'Engineered T&amp;G'. No promotion header on this section. Supplier marks this colour *DISCONTINUE ITEM* on the Aug 31 2026 list -&gt; Stock status = Discontinued, Active = FALSE. Confirm remaining stock before import. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF175" t="inlineStr">
@@ -20845,7 +20845,7 @@
       </c>
       <c r="BC176" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Brand Surfaces (T&amp;G) - Oak (Smoked Expose) T&amp;G | #CAN.E.O.Smo". Brand Surfaces 'Engineered T&amp;G'. No promotion header on this section. Supplier marks this colour *DISCONTINUE ITEM* on the Aug 31 2026 list -&gt; Stock status = Discontinued, Active = FALSE. Confirm remaining stock before import. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Brand Surfaces (T&amp;G) - Oak (Smoked Expose) T&amp;G | #CAN.E.O.Smo". Brand Surfaces 'Engineered T&amp;G'. No promotion header on this section. Supplier marks this colour *DISCONTINUE ITEM* on the Aug 31 2026 list -&gt; Stock status = Discontinued, Active = FALSE. Confirm remaining stock before import. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF176" t="inlineStr">
@@ -20962,7 +20962,7 @@
       </c>
       <c r="BC177" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour variant match to Lightspeed product "CANENG - Brand Surfaces (T&amp;G) - Oak (Smoke Tobacco) T&amp;G | #CAN.E.O.Smo". Brand Surfaces 'Engineered T&amp;G'. No promotion header on this section. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour variant match to Lightspeed product "CANENG - Brand Surfaces (T&amp;G) - Oak (Smoke Tobacco) T&amp;G | #CAN.E.O.Smo". Brand Surfaces 'Engineered T&amp;G'. No promotion header on this section. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF177" t="inlineStr">
@@ -21079,7 +21079,7 @@
       </c>
       <c r="BC178" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Brand Surfaces (T&amp;G) - Maple (Blacksmith) T&amp;G | #CAN.E.M.Bla.". Brand Surfaces 'Engineered T&amp;G'. No promotion header on this section. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Brand Surfaces (T&amp;G) - Maple (Blacksmith) T&amp;G | #CAN.E.M.Bla.". Brand Surfaces 'Engineered T&amp;G'. No promotion header on this section. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF178" t="inlineStr">
@@ -21196,7 +21196,7 @@
       </c>
       <c r="BC179" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Brand Surfaces (T&amp;G) - Maple (Chimney Smoke) T&amp;G | #CAN.E.M.C". Brand Surfaces 'Engineered T&amp;G'. No promotion header on this section. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Brand Surfaces (T&amp;G) - Maple (Chimney Smoke) T&amp;G | #CAN.E.M.C". Brand Surfaces 'Engineered T&amp;G'. No promotion header on this section. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF179" t="inlineStr">
@@ -21313,7 +21313,7 @@
       </c>
       <c r="BC180" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Brand Surfaces (T&amp;G) - Maple (Cotton Ball) T&amp;G | #CAN.E.M.Cot". Brand Surfaces 'Engineered T&amp;G'. No promotion header on this section. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Brand Surfaces (T&amp;G) - Maple (Cotton Ball) T&amp;G | #CAN.E.M.Cot". Brand Surfaces 'Engineered T&amp;G'. No promotion header on this section. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF180" t="inlineStr">
@@ -21430,7 +21430,7 @@
       </c>
       <c r="BC181" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Brand Surfaces (T&amp;G) - Maple (Millstead) T&amp;G | #CAN.E.M.Mil.7". Brand Surfaces 'Engineered T&amp;G'. No promotion header on this section. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Brand Surfaces (T&amp;G) - Maple (Millstead) T&amp;G | #CAN.E.M.Mil.7". Brand Surfaces 'Engineered T&amp;G'. No promotion header on this section. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF181" t="inlineStr">
@@ -21547,7 +21547,7 @@
       </c>
       <c r="BC182" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Brand Surfaces (T&amp;G) - Maple (Pottery Barn) T&amp;G | #CAN.E.M.Po". Brand Surfaces 'Engineered T&amp;G'. No promotion header on this section. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Brand Surfaces (T&amp;G) - Maple (Pottery Barn) T&amp;G | #CAN.E.M.Po". Brand Surfaces 'Engineered T&amp;G'. No promotion header on this section. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF182" t="inlineStr">
@@ -21664,7 +21664,7 @@
       </c>
       <c r="BC183" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Brand Surfaces (T&amp;G) - Maple (Warm Onyx) T&amp;G | #CAN.E.M.WarOn". Brand Surfaces 'Engineered T&amp;G'. No promotion header on this section. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Brand Surfaces (T&amp;G) - Maple (Warm Onyx) T&amp;G | #CAN.E.M.WarOn". Brand Surfaces 'Engineered T&amp;G'. No promotion header on this section. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF183" t="inlineStr">
@@ -21781,7 +21781,7 @@
       </c>
       <c r="BC184" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour variant match to Lightspeed product "CANENG - Brand Surfaces (T&amp;G) - Maple (Winbledon) T&amp;G | #CAN.E.M.Win.7". Brand Surfaces 'Engineered T&amp;G'. No promotion header on this section. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour variant match to Lightspeed product "CANENG - Brand Surfaces (T&amp;G) - Maple (Winbledon) T&amp;G | #CAN.E.M.Win.7". Brand Surfaces 'Engineered T&amp;G'. No promotion header on this section. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF184" t="inlineStr">
@@ -21898,7 +21898,7 @@
       </c>
       <c r="BC185" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Brand Surfaces (T&amp;G) - Maple (Wool Coat) T&amp;G | #CAN.E.M.WooCo". Brand Surfaces 'Engineered T&amp;G'. No promotion header on this section. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Brand Surfaces (T&amp;G) - Maple (Wool Coat) T&amp;G | #CAN.E.M.WooCo". Brand Surfaces 'Engineered T&amp;G'. No promotion header on this section. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF185" t="inlineStr">
@@ -22013,7 +22013,7 @@
       </c>
       <c r="BC186" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANLAM - 8MM Laminate Planks -  (Crown Point)  | #CAN.L.CroPoi.1 |". PROMO (no window printed): 'Soft Launch Special' prints 'Special Price $1.29' / 'Regular Price $1.79'. Global sale-item logic applied; global month-end default used for the end date -&gt; 2026-09-30 (the list is effective 31-Aug-2026 and today is 03-Sep-2026). Confirm the real end date. 196mm x 1215mm x 8mm; Width (in) 7.72 converted from 196mm. 'New Arrival'. Supplier marks this colour *DISCONTINUE ITEM* on the Aug 31 2026 list -&gt; Stock status = Discontinued, Active = FALSE. Confirm remaining stock before import. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANLAM - 8MM Laminate Planks -  (Crown Point)  | #CAN.L.CroPoi.1 |". PROMO (no window printed): 'Soft Launch Special' prints 'Special Price $1.29' / 'Regular Price $1.79'. Global sale-item logic applied; global month-end default used for the end date -&gt; 2026-09-30 (the list is effective 31-Aug-2026 and today is 03-Sep-2026). Confirm the real end date. 196mm x 1215mm x 8mm; Width (in) 7.72 converted from 196mm. 'New Arrival'. Supplier marks this colour *DISCONTINUE ITEM* on the Aug 31 2026 list -&gt; Stock status = Discontinued, Active = FALSE. Confirm remaining stock before import. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF186" t="inlineStr">
@@ -22123,7 +22123,7 @@
       </c>
       <c r="BC187" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANLAM - 8MM Laminate Planks -  (Five Peaks)  | #CAN.L.FivPea.1 | ". PROMO (no window printed): 'Soft Launch Special' prints 'Special Price $1.29' / 'Regular Price $1.79'. Global sale-item logic applied; global month-end default used for the end date -&gt; 2026-09-30 (the list is effective 31-Aug-2026 and today is 03-Sep-2026). Confirm the real end date. 196mm x 1215mm x 8mm; Width (in) 7.72 converted from 196mm. 'New Arrival'. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANLAM - 8MM Laminate Planks -  (Five Peaks)  | #CAN.L.FivPea.1 | ". PROMO (no window printed): 'Soft Launch Special' prints 'Special Price $1.29' / 'Regular Price $1.79'. Global sale-item logic applied; global month-end default used for the end date -&gt; 2026-09-30 (the list is effective 31-Aug-2026 and today is 03-Sep-2026). Confirm the real end date. 196mm x 1215mm x 8mm; Width (in) 7.72 converted from 196mm. 'New Arrival'. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF187" t="inlineStr">
@@ -22233,7 +22233,7 @@
       </c>
       <c r="BC188" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANLAM - 8MM Laminate Planks -  (Lake View)  | #CAN.L.LakVie.1 |  ". PROMO (no window printed): 'Soft Launch Special' prints 'Special Price $1.29' / 'Regular Price $1.79'. Global sale-item logic applied; global month-end default used for the end date -&gt; 2026-09-30 (the list is effective 31-Aug-2026 and today is 03-Sep-2026). Confirm the real end date. 196mm x 1215mm x 8mm; Width (in) 7.72 converted from 196mm. 'New Arrival'. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANLAM - 8MM Laminate Planks -  (Lake View)  | #CAN.L.LakVie.1 |  ". PROMO (no window printed): 'Soft Launch Special' prints 'Special Price $1.29' / 'Regular Price $1.79'. Global sale-item logic applied; global month-end default used for the end date -&gt; 2026-09-30 (the list is effective 31-Aug-2026 and today is 03-Sep-2026). Confirm the real end date. 196mm x 1215mm x 8mm; Width (in) 7.72 converted from 196mm. 'New Arrival'. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF188" t="inlineStr">
@@ -22343,7 +22343,7 @@
       </c>
       <c r="BC189" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANLAM - 8MM Laminate Planks -  (Laurel Ridge)  | #CAN.L.LauRid.1 ". PROMO (no window printed): 'Soft Launch Special' prints 'Special Price $1.29' / 'Regular Price $1.79'. Global sale-item logic applied; global month-end default used for the end date -&gt; 2026-09-30 (the list is effective 31-Aug-2026 and today is 03-Sep-2026). Confirm the real end date. 196mm x 1215mm x 8mm; Width (in) 7.72 converted from 196mm. 'New Arrival'. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANLAM - 8MM Laminate Planks -  (Laurel Ridge)  | #CAN.L.LauRid.1 ". PROMO (no window printed): 'Soft Launch Special' prints 'Special Price $1.29' / 'Regular Price $1.79'. Global sale-item logic applied; global month-end default used for the end date -&gt; 2026-09-30 (the list is effective 31-Aug-2026 and today is 03-Sep-2026). Confirm the real end date. 196mm x 1215mm x 8mm; Width (in) 7.72 converted from 196mm. 'New Arrival'. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF189" t="inlineStr">
@@ -22453,7 +22453,7 @@
       </c>
       <c r="BC190" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANLAM - 8MM Laminate Planks -  (Oak Bridge)  | #CAN.L.OakBri.1 | ". PROMO (no window printed): 'Soft Launch Special' prints 'Special Price $1.29' / 'Regular Price $1.79'. Global sale-item logic applied; global month-end default used for the end date -&gt; 2026-09-30 (the list is effective 31-Aug-2026 and today is 03-Sep-2026). Confirm the real end date. 196mm x 1215mm x 8mm; Width (in) 7.72 converted from 196mm. 'New Arrival'. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANLAM - 8MM Laminate Planks -  (Oak Bridge)  | #CAN.L.OakBri.1 | ". PROMO (no window printed): 'Soft Launch Special' prints 'Special Price $1.29' / 'Regular Price $1.79'. Global sale-item logic applied; global month-end default used for the end date -&gt; 2026-09-30 (the list is effective 31-Aug-2026 and today is 03-Sep-2026). Confirm the real end date. 196mm x 1215mm x 8mm; Width (in) 7.72 converted from 196mm. 'New Arrival'. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF190" t="inlineStr">
@@ -22563,7 +22563,7 @@
       </c>
       <c r="BC191" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANLAM - 8MM Laminate Planks -  (Town Mill)  | #CAN.L.TowMil.1 |  ". PROMO (no window printed): 'Soft Launch Special' prints 'Special Price $1.29' / 'Regular Price $1.79'. Global sale-item logic applied; global month-end default used for the end date -&gt; 2026-09-30 (the list is effective 31-Aug-2026 and today is 03-Sep-2026). Confirm the real end date. 196mm x 1215mm x 8mm; Width (in) 7.72 converted from 196mm. 'New Arrival'. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANLAM - 8MM Laminate Planks -  (Town Mill)  | #CAN.L.TowMil.1 |  ". PROMO (no window printed): 'Soft Launch Special' prints 'Special Price $1.29' / 'Regular Price $1.79'. Global sale-item logic applied; global month-end default used for the end date -&gt; 2026-09-30 (the list is effective 31-Aug-2026 and today is 03-Sep-2026). Confirm the real end date. 196mm x 1215mm x 8mm; Width (in) 7.72 converted from 196mm. 'New Arrival'. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF191" t="inlineStr">
@@ -22673,7 +22673,7 @@
       </c>
       <c r="BC192" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANLAM - 8MM Laminate Planks -  (Willow Creek)  | #CAN.L.WilCre.1 ". PROMO (no window printed): 'Soft Launch Special' prints 'Special Price $1.29' / 'Regular Price $1.79'. Global sale-item logic applied; global month-end default used for the end date -&gt; 2026-09-30 (the list is effective 31-Aug-2026 and today is 03-Sep-2026). Confirm the real end date. 196mm x 1215mm x 8mm; Width (in) 7.72 converted from 196mm. 'New Arrival'. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANLAM - 8MM Laminate Planks -  (Willow Creek)  | #CAN.L.WilCre.1 ". PROMO (no window printed): 'Soft Launch Special' prints 'Special Price $1.29' / 'Regular Price $1.79'. Global sale-item logic applied; global month-end default used for the end date -&gt; 2026-09-30 (the list is effective 31-Aug-2026 and today is 03-Sep-2026). Confirm the real end date. 196mm x 1215mm x 8mm; Width (in) 7.72 converted from 196mm. 'New Arrival'. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF192" t="inlineStr">
@@ -22783,7 +22783,7 @@
       </c>
       <c r="BC193" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANLAM - 8MM Laminate Planks -  (Wood Land)  | #CAN.L.WooLan.1 |  ". PROMO (no window printed): 'Soft Launch Special' prints 'Special Price $1.29' / 'Regular Price $1.79'. Global sale-item logic applied; global month-end default used for the end date -&gt; 2026-09-30 (the list is effective 31-Aug-2026 and today is 03-Sep-2026). Confirm the real end date. 196mm x 1215mm x 8mm; Width (in) 7.72 converted from 196mm. 'New Arrival'. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "(P) CANLAM - 8MM Laminate Planks -  (Wood Land)  | #CAN.L.WooLan.1 |  ". PROMO (no window printed): 'Soft Launch Special' prints 'Special Price $1.29' / 'Regular Price $1.79'. Global sale-item logic applied; global month-end default used for the end date -&gt; 2026-09-30 (the list is effective 31-Aug-2026 and today is 03-Sep-2026). Confirm the real end date. 196mm x 1215mm x 8mm; Width (in) 7.72 converted from 196mm. 'New Arrival'. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF193" t="inlineStr">
@@ -22893,7 +22893,7 @@
       </c>
       <c r="BC194" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - EGGER PRO -  (Lasken Oak)  | #EPL136 | AC4 - 50.87" x 7.6" x ". EGGER PRO Laminate, made in Germany. 12mm AC4, R10 slip-resistance, 'HDF Swell Barrier+' -&gt; Material type = HDF core (stated). 50.87" x 7.6" x 12mm. R10 slip rating recorded here; the schema has no slip-rating field. 'Gray Leoma Wlanut' / 'Sand Biege' are the supplier's spellings, kept verbatim. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - EGGER PRO -  (Lasken Oak)  | #EPL136 | AC4 - 50.87" x 7.6" x ". EGGER PRO Laminate, made in Germany. 12mm AC4, R10 slip-resistance, 'HDF Swell Barrier+' -&gt; Material type = HDF core (stated). 50.87" x 7.6" x 12mm. R10 slip rating recorded here; the schema has no slip-rating field. 'Gray Leoma Wlanut' / 'Sand Biege' are the supplier's spellings, kept verbatim. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF194" t="inlineStr">
@@ -23003,7 +23003,7 @@
       </c>
       <c r="BC195" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - EGGER PRO -  (Light Nakina Oak)  | #EPL163 | AC4 - 50.87" x 7". EGGER PRO Laminate, made in Germany. 12mm AC4, R10 slip-resistance, 'HDF Swell Barrier+' -&gt; Material type = HDF core (stated). 50.87" x 7.6" x 12mm. R10 slip rating recorded here; the schema has no slip-rating field. 'Gray Leoma Wlanut' / 'Sand Biege' are the supplier's spellings, kept verbatim. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - EGGER PRO -  (Light Nakina Oak)  | #EPL163 | AC4 - 50.87" x 7". EGGER PRO Laminate, made in Germany. 12mm AC4, R10 slip-resistance, 'HDF Swell Barrier+' -&gt; Material type = HDF core (stated). 50.87" x 7.6" x 12mm. R10 slip rating recorded here; the schema has no slip-rating field. 'Gray Leoma Wlanut' / 'Sand Biege' are the supplier's spellings, kept verbatim. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF195" t="inlineStr">
@@ -23113,7 +23113,7 @@
       </c>
       <c r="BC196" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - EGGER PRO -  (Murom Oak Gray)  | #EPL138 | AC4 - 50.87" x 7.6". EGGER PRO Laminate, made in Germany. 12mm AC4, R10 slip-resistance, 'HDF Swell Barrier+' -&gt; Material type = HDF core (stated). 50.87" x 7.6" x 12mm. R10 slip rating recorded here; the schema has no slip-rating field. 'Gray Leoma Wlanut' / 'Sand Biege' are the supplier's spellings, kept verbatim. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - EGGER PRO -  (Murom Oak Gray)  | #EPL138 | AC4 - 50.87" x 7.6". EGGER PRO Laminate, made in Germany. 12mm AC4, R10 slip-resistance, 'HDF Swell Barrier+' -&gt; Material type = HDF core (stated). 50.87" x 7.6" x 12mm. R10 slip rating recorded here; the schema has no slip-rating field. 'Gray Leoma Wlanut' / 'Sand Biege' are the supplier's spellings, kept verbatim. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF196" t="inlineStr">
@@ -23228,7 +23228,7 @@
       </c>
       <c r="BC197" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - EGGER PRO -  (Olchon Oak Honey)  | #EPL144 | AC4 - 50.87" x 7". EGGER PRO Laminate, made in Germany. 12mm AC4, R10 slip-resistance, 'HDF Swell Barrier+' -&gt; Material type = HDF core (stated). 50.87" x 7.6" x 12mm. R10 slip rating recorded here; the schema has no slip-rating field. 'Gray Leoma Wlanut' / 'Sand Biege' are the supplier's spellings, kept verbatim. Supplier marks this colour *DISCONTINUE ITEM* on the Aug 31 2026 list -&gt; Stock status = Discontinued, Active = FALSE. Confirm remaining stock before import. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - EGGER PRO -  (Olchon Oak Honey)  | #EPL144 | AC4 - 50.87" x 7". EGGER PRO Laminate, made in Germany. 12mm AC4, R10 slip-resistance, 'HDF Swell Barrier+' -&gt; Material type = HDF core (stated). 50.87" x 7.6" x 12mm. R10 slip rating recorded here; the schema has no slip-rating field. 'Gray Leoma Wlanut' / 'Sand Biege' are the supplier's spellings, kept verbatim. Supplier marks this colour *DISCONTINUE ITEM* on the Aug 31 2026 list -&gt; Stock status = Discontinued, Active = FALSE. Confirm remaining stock before import. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF197" t="inlineStr">
@@ -23343,7 +23343,7 @@
       </c>
       <c r="BC198" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - EGGER PRO -  (Olchon Oak White)  | #EPL141 | AC4 - 50.87" x 7". EGGER PRO Laminate, made in Germany. 12mm AC4, R10 slip-resistance, 'HDF Swell Barrier+' -&gt; Material type = HDF core (stated). 50.87" x 7.6" x 12mm. R10 slip rating recorded here; the schema has no slip-rating field. 'Gray Leoma Wlanut' / 'Sand Biege' are the supplier's spellings, kept verbatim. Supplier marks this colour *DISCONTINUE ITEM* on the Aug 31 2026 list -&gt; Stock status = Discontinued, Active = FALSE. Confirm remaining stock before import. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - EGGER PRO -  (Olchon Oak White)  | #EPL141 | AC4 - 50.87" x 7". EGGER PRO Laminate, made in Germany. 12mm AC4, R10 slip-resistance, 'HDF Swell Barrier+' -&gt; Material type = HDF core (stated). 50.87" x 7.6" x 12mm. R10 slip rating recorded here; the schema has no slip-rating field. 'Gray Leoma Wlanut' / 'Sand Biege' are the supplier's spellings, kept verbatim. Supplier marks this colour *DISCONTINUE ITEM* on the Aug 31 2026 list -&gt; Stock status = Discontinued, Active = FALSE. Confirm remaining stock before import. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF198" t="inlineStr">
@@ -23458,7 +23458,7 @@
       </c>
       <c r="BC199" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - EGGER PRO -  (Sand Biege (Olchon Oak))  | #EPL142 | AC4 - 50.". EGGER PRO Laminate, made in Germany. 12mm AC4, R10 slip-resistance, 'HDF Swell Barrier+' -&gt; Material type = HDF core (stated). 50.87" x 7.6" x 12mm. R10 slip rating recorded here; the schema has no slip-rating field. 'Gray Leoma Wlanut' / 'Sand Biege' are the supplier's spellings, kept verbatim. Supplier marks this colour *DISCONTINUE ITEM* on the Aug 31 2026 list -&gt; Stock status = Discontinued, Active = FALSE. Confirm remaining stock before import. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - EGGER PRO -  (Sand Biege (Olchon Oak))  | #EPL142 | AC4 - 50.". EGGER PRO Laminate, made in Germany. 12mm AC4, R10 slip-resistance, 'HDF Swell Barrier+' -&gt; Material type = HDF core (stated). 50.87" x 7.6" x 12mm. R10 slip rating recorded here; the schema has no slip-rating field. 'Gray Leoma Wlanut' / 'Sand Biege' are the supplier's spellings, kept verbatim. Supplier marks this colour *DISCONTINUE ITEM* on the Aug 31 2026 list -&gt; Stock status = Discontinued, Active = FALSE. Confirm remaining stock before import. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF199" t="inlineStr">
@@ -23568,7 +23568,7 @@
       </c>
       <c r="BC200" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - EGGER PRO -  (Valley Oak Mocca)  | #EPL016 | AC4 - 50.87" x 7". EGGER PRO Laminate, made in Germany. 12mm AC4, R10 slip-resistance, 'HDF Swell Barrier+' -&gt; Material type = HDF core (stated). 50.87" x 7.6" x 12mm. R10 slip rating recorded here; the schema has no slip-rating field. 'Gray Leoma Wlanut' / 'Sand Biege' are the supplier's spellings, kept verbatim. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - EGGER PRO -  (Valley Oak Mocca)  | #EPL016 | AC4 - 50.87" x 7". EGGER PRO Laminate, made in Germany. 12mm AC4, R10 slip-resistance, 'HDF Swell Barrier+' -&gt; Material type = HDF core (stated). 50.87" x 7.6" x 12mm. R10 slip rating recorded here; the schema has no slip-rating field. 'Gray Leoma Wlanut' / 'Sand Biege' are the supplier's spellings, kept verbatim. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF200" t="inlineStr">
@@ -23678,7 +23678,7 @@
       </c>
       <c r="BC201" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - EGGER PRO -  (Gray Sorgono Pine)  | #EPL160 | AC4 - 50.87" x ". EGGER PRO Laminate, made in Germany. 12mm AC4, R10 slip-resistance, 'HDF Swell Barrier+' -&gt; Material type = HDF core (stated). 50.87" x 7.6" x 12mm. R10 slip rating recorded here; the schema has no slip-rating field. 'Gray Leoma Wlanut' / 'Sand Biege' are the supplier's spellings, kept verbatim. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - EGGER PRO -  (Gray Sorgono Pine)  | #EPL160 | AC4 - 50.87" x ". EGGER PRO Laminate, made in Germany. 12mm AC4, R10 slip-resistance, 'HDF Swell Barrier+' -&gt; Material type = HDF core (stated). 50.87" x 7.6" x 12mm. R10 slip rating recorded here; the schema has no slip-rating field. 'Gray Leoma Wlanut' / 'Sand Biege' are the supplier's spellings, kept verbatim. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF201" t="inlineStr">
@@ -23788,7 +23788,7 @@
       </c>
       <c r="BC202" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - EGGER PRO -  (Gray Leoma Wlanut)  | #EPL161 | AC4 - 50.87" x ". EGGER PRO Laminate, made in Germany. 12mm AC4, R10 slip-resistance, 'HDF Swell Barrier+' -&gt; Material type = HDF core (stated). 50.87" x 7.6" x 12mm. R10 slip rating recorded here; the schema has no slip-rating field. 'Gray Leoma Wlanut' / 'Sand Biege' are the supplier's spellings, kept verbatim. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - EGGER PRO -  (Gray Leoma Wlanut)  | #EPL161 | AC4 - 50.87" x ". EGGER PRO Laminate, made in Germany. 12mm AC4, R10 slip-resistance, 'HDF Swell Barrier+' -&gt; Material type = HDF core (stated). 50.87" x 7.6" x 12mm. R10 slip rating recorded here; the schema has no slip-rating field. 'Gray Leoma Wlanut' / 'Sand Biege' are the supplier's spellings, kept verbatim. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF202" t="inlineStr">
@@ -23898,7 +23898,7 @@
       </c>
       <c r="BC203" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - EGGER PRO -  (Mansonia Walnut)  | #EPL109 | AC4 - 50.87" x 7.". EGGER PRO Laminate, made in Germany. 12mm AC4, R10 slip-resistance, 'HDF Swell Barrier+' -&gt; Material type = HDF core (stated). 50.87" x 7.6" x 12mm. R10 slip rating recorded here; the schema has no slip-rating field. 'Gray Leoma Wlanut' / 'Sand Biege' are the supplier's spellings, kept verbatim. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - EGGER PRO -  (Mansonia Walnut)  | #EPL109 | AC4 - 50.87" x 7.". EGGER PRO Laminate, made in Germany. 12mm AC4, R10 slip-resistance, 'HDF Swell Barrier+' -&gt; Material type = HDF core (stated). 50.87" x 7.6" x 12mm. R10 slip rating recorded here; the schema has no slip-rating field. 'Gray Leoma Wlanut' / 'Sand Biege' are the supplier's spellings, kept verbatim. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF203" t="inlineStr">
@@ -24003,7 +24003,7 @@
       </c>
       <c r="BC204" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - EGGER AQUA+ - Wood Grain (Bardolino Oak)  | #EPL036 |  - 50.8". EGGER AQUA+ Laminate, made in Germany. 50.87" x 7.6" x 12mm (WOOD GRAIN). AMBIGUOUS: 'AQUA+' is a water-resistance claim short of 'waterproof' -&gt; Waterproof left blank (not FALSE, not TRUE) pending confirmation; Material type set to Water-Resistant Core. AC rating not stated for AQUA+ (only EGGER PRO states AC4) -&gt; left blank. EVERY colour in this sub-group is marked *DISCONTINUE ITEM*. Supplier marks this colour *DISCONTINUE ITEM* on the Aug 31 2026 list -&gt; Stock status = Discontinued, Active = FALSE. Confirm remaining stock before import. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - EGGER AQUA+ - Wood Grain (Bardolino Oak)  | #EPL036 |  - 50.8". EGGER AQUA+ Laminate, made in Germany. 50.87" x 7.6" x 12mm (WOOD GRAIN). AMBIGUOUS: 'AQUA+' is a water-resistance claim short of 'waterproof' -&gt; Waterproof left blank (not FALSE, not TRUE) pending confirmation; Material type set to Water-Resistant Core. AC rating not stated for AQUA+ (only EGGER PRO states AC4) -&gt; left blank. EVERY colour in this sub-group is marked *DISCONTINUE ITEM*. Supplier marks this colour *DISCONTINUE ITEM* on the Aug 31 2026 list -&gt; Stock status = Discontinued, Active = FALSE. Confirm remaining stock before import. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF204" t="inlineStr">
@@ -24108,7 +24108,7 @@
       </c>
       <c r="BC205" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - EGGER AQUA+ - Wood Grain (Dark Abergele)  | #EPL068 |  - 50.8". EGGER AQUA+ Laminate, made in Germany. 50.87" x 7.6" x 12mm (WOOD GRAIN). AMBIGUOUS: 'AQUA+' is a water-resistance claim short of 'waterproof' -&gt; Waterproof left blank (not FALSE, not TRUE) pending confirmation; Material type set to Water-Resistant Core. AC rating not stated for AQUA+ (only EGGER PRO states AC4) -&gt; left blank. EVERY colour in this sub-group is marked *DISCONTINUE ITEM*. Supplier marks this colour *DISCONTINUE ITEM* on the Aug 31 2026 list -&gt; Stock status = Discontinued, Active = FALSE. Confirm remaining stock before import. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - EGGER AQUA+ - Wood Grain (Dark Abergele)  | #EPL068 |  - 50.8". EGGER AQUA+ Laminate, made in Germany. 50.87" x 7.6" x 12mm (WOOD GRAIN). AMBIGUOUS: 'AQUA+' is a water-resistance claim short of 'waterproof' -&gt; Waterproof left blank (not FALSE, not TRUE) pending confirmation; Material type set to Water-Resistant Core. AC rating not stated for AQUA+ (only EGGER PRO states AC4) -&gt; left blank. EVERY colour in this sub-group is marked *DISCONTINUE ITEM*. Supplier marks this colour *DISCONTINUE ITEM* on the Aug 31 2026 list -&gt; Stock status = Discontinued, Active = FALSE. Confirm remaining stock before import. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF205" t="inlineStr">
@@ -24213,7 +24213,7 @@
       </c>
       <c r="BC206" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - EGGER AQUA+ - Wood Grain (Natural Bardolino Oak)  | #EPL165 |". EGGER AQUA+ Laminate, made in Germany. 50.87" x 7.6" x 12mm (WOOD GRAIN). AMBIGUOUS: 'AQUA+' is a water-resistance claim short of 'waterproof' -&gt; Waterproof left blank (not FALSE, not TRUE) pending confirmation; Material type set to Water-Resistant Core. AC rating not stated for AQUA+ (only EGGER PRO states AC4) -&gt; left blank. EVERY colour in this sub-group is marked *DISCONTINUE ITEM*. Supplier marks this colour *DISCONTINUE ITEM* on the Aug 31 2026 list -&gt; Stock status = Discontinued, Active = FALSE. Confirm remaining stock before import. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - EGGER AQUA+ - Wood Grain (Natural Bardolino Oak)  | #EPL165 |". EGGER AQUA+ Laminate, made in Germany. 50.87" x 7.6" x 12mm (WOOD GRAIN). AMBIGUOUS: 'AQUA+' is a water-resistance claim short of 'waterproof' -&gt; Waterproof left blank (not FALSE, not TRUE) pending confirmation; Material type set to Water-Resistant Core. AC rating not stated for AQUA+ (only EGGER PRO states AC4) -&gt; left blank. EVERY colour in this sub-group is marked *DISCONTINUE ITEM*. Supplier marks this colour *DISCONTINUE ITEM* on the Aug 31 2026 list -&gt; Stock status = Discontinued, Active = FALSE. Confirm remaining stock before import. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF206" t="inlineStr">
@@ -24318,7 +24318,7 @@
       </c>
       <c r="BC207" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - EGGER AQUA+ - Wood Grain (Natural Valley Oak)  | #EPL159 |  -". EGGER AQUA+ Laminate, made in Germany. 50.87" x 7.6" x 12mm (WOOD GRAIN). AMBIGUOUS: 'AQUA+' is a water-resistance claim short of 'waterproof' -&gt; Waterproof left blank (not FALSE, not TRUE) pending confirmation; Material type set to Water-Resistant Core. AC rating not stated for AQUA+ (only EGGER PRO states AC4) -&gt; left blank. EVERY colour in this sub-group is marked *DISCONTINUE ITEM*. Supplier marks this colour *DISCONTINUE ITEM* on the Aug 31 2026 list -&gt; Stock status = Discontinued, Active = FALSE. Confirm remaining stock before import. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - EGGER AQUA+ - Wood Grain (Natural Valley Oak)  | #EPL159 |  -". EGGER AQUA+ Laminate, made in Germany. 50.87" x 7.6" x 12mm (WOOD GRAIN). AMBIGUOUS: 'AQUA+' is a water-resistance claim short of 'waterproof' -&gt; Waterproof left blank (not FALSE, not TRUE) pending confirmation; Material type set to Water-Resistant Core. AC rating not stated for AQUA+ (only EGGER PRO states AC4) -&gt; left blank. EVERY colour in this sub-group is marked *DISCONTINUE ITEM*. Supplier marks this colour *DISCONTINUE ITEM* on the Aug 31 2026 list -&gt; Stock status = Discontinued, Active = FALSE. Confirm remaining stock before import. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF207" t="inlineStr">
@@ -24423,7 +24423,7 @@
       </c>
       <c r="BC208" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - EGGER AQUA+ - Wood Grain (Valley Oak Smoke)  | #EPL015 |  - 5". EGGER AQUA+ Laminate, made in Germany. 50.87" x 7.6" x 12mm (WOOD GRAIN). AMBIGUOUS: 'AQUA+' is a water-resistance claim short of 'waterproof' -&gt; Waterproof left blank (not FALSE, not TRUE) pending confirmation; Material type set to Water-Resistant Core. AC rating not stated for AQUA+ (only EGGER PRO states AC4) -&gt; left blank. EVERY colour in this sub-group is marked *DISCONTINUE ITEM*. Supplier marks this colour *DISCONTINUE ITEM* on the Aug 31 2026 list -&gt; Stock status = Discontinued, Active = FALSE. Confirm remaining stock before import. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - EGGER AQUA+ - Wood Grain (Valley Oak Smoke)  | #EPL015 |  - 5". EGGER AQUA+ Laminate, made in Germany. 50.87" x 7.6" x 12mm (WOOD GRAIN). AMBIGUOUS: 'AQUA+' is a water-resistance claim short of 'waterproof' -&gt; Waterproof left blank (not FALSE, not TRUE) pending confirmation; Material type set to Water-Resistant Core. AC rating not stated for AQUA+ (only EGGER PRO states AC4) -&gt; left blank. EVERY colour in this sub-group is marked *DISCONTINUE ITEM*. Supplier marks this colour *DISCONTINUE ITEM* on the Aug 31 2026 list -&gt; Stock status = Discontinued, Active = FALSE. Confirm remaining stock before import. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF208" t="inlineStr">
@@ -24528,7 +24528,7 @@
       </c>
       <c r="BC209" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - EGGER AQUA+ - Wood Grain (White Valley Oak)  | #EPL158 |  - 5". EGGER AQUA+ Laminate, made in Germany. 50.87" x 7.6" x 12mm (WOOD GRAIN). AMBIGUOUS: 'AQUA+' is a water-resistance claim short of 'waterproof' -&gt; Waterproof left blank (not FALSE, not TRUE) pending confirmation; Material type set to Water-Resistant Core. AC rating not stated for AQUA+ (only EGGER PRO states AC4) -&gt; left blank. EVERY colour in this sub-group is marked *DISCONTINUE ITEM*. Supplier marks this colour *DISCONTINUE ITEM* on the Aug 31 2026 list -&gt; Stock status = Discontinued, Active = FALSE. Confirm remaining stock before import. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - EGGER AQUA+ - Wood Grain (White Valley Oak)  | #EPL158 |  - 5". EGGER AQUA+ Laminate, made in Germany. 50.87" x 7.6" x 12mm (WOOD GRAIN). AMBIGUOUS: 'AQUA+' is a water-resistance claim short of 'waterproof' -&gt; Waterproof left blank (not FALSE, not TRUE) pending confirmation; Material type set to Water-Resistant Core. AC rating not stated for AQUA+ (only EGGER PRO states AC4) -&gt; left blank. EVERY colour in this sub-group is marked *DISCONTINUE ITEM*. Supplier marks this colour *DISCONTINUE ITEM* on the Aug 31 2026 list -&gt; Stock status = Discontinued, Active = FALSE. Confirm remaining stock before import. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF209" t="inlineStr">
@@ -24628,7 +24628,7 @@
       </c>
       <c r="BC210" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - EGGER AQUA+ - TILE (Light Gray Chicago Concrete)  | #EPL166 |". EGGER AQUA+ Laminate 'Concrete (TILE)', made in Germany. 50.87" x 12.88" x 8mm. Laminate tile format -&gt; Category = Laminate (Tile format field is for the Tile / Stone category only, left blank). Waterproof left blank - 'AQUA+' is water-resistance, not a waterproof claim. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - EGGER AQUA+ - TILE (Light Gray Chicago Concrete)  | #EPL166 |". EGGER AQUA+ Laminate 'Concrete (TILE)', made in Germany. 50.87" x 12.88" x 8mm. Laminate tile format -&gt; Category = Laminate (Tile format field is for the Tile / Stone category only, left blank). Waterproof left blank - 'AQUA+' is water-resistance, not a waterproof claim. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF210" t="inlineStr">
@@ -24728,7 +24728,7 @@
       </c>
       <c r="BC211" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - EGGER AQUA+ - TILE (Slate Black Classic)  | #EPL157 |  - 50.8". EGGER AQUA+ Laminate 'Concrete (TILE)', made in Germany. 50.87" x 12.88" x 8mm. Laminate tile format -&gt; Category = Laminate (Tile format field is for the Tile / Stone category only, left blank). Waterproof left blank - 'AQUA+' is water-resistance, not a waterproof claim. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - EGGER AQUA+ - TILE (Slate Black Classic)  | #EPL157 |  - 50.8". EGGER AQUA+ Laminate 'Concrete (TILE)', made in Germany. 50.87" x 12.88" x 8mm. Laminate tile format -&gt; Category = Laminate (Tile format field is for the Tile / Stone category only, left blank). Waterproof left blank - 'AQUA+' is water-resistance, not a waterproof claim. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF211" t="inlineStr">
@@ -24833,7 +24833,7 @@
       </c>
       <c r="BC212" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - EGGER AQUA+ - TILE (White Chromix)  | #EPL168 |  - 50.87" x 1". EGGER AQUA+ Laminate 'Concrete (TILE)', made in Germany. 50.87" x 12.88" x 8mm. Laminate tile format -&gt; Category = Laminate (Tile format field is for the Tile / Stone category only, left blank). Waterproof left blank - 'AQUA+' is water-resistance, not a waterproof claim. Supplier marks this colour *DISCONTINUE ITEM* on the Aug 31 2026 list -&gt; Stock status = Discontinued, Active = FALSE. Confirm remaining stock before import. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - EGGER AQUA+ - TILE (White Chromix)  | #EPL168 |  - 50.87" x 1". EGGER AQUA+ Laminate 'Concrete (TILE)', made in Germany. 50.87" x 12.88" x 8mm. Laminate tile format -&gt; Category = Laminate (Tile format field is for the Tile / Stone category only, left blank). Waterproof left blank - 'AQUA+' is water-resistance, not a waterproof claim. Supplier marks this colour *DISCONTINUE ITEM* on the Aug 31 2026 list -&gt; Stock status = Discontinued, Active = FALSE. Confirm remaining stock before import. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF212" t="inlineStr">
@@ -24953,7 +24953,7 @@
       </c>
       <c r="BC213" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - Inhaus 12mm AC4 - Dynamic Highlands (Hemlock (Dark Beige))  |". Inhaus 12mm AC4 Laminate, MegaLoc (G5) locking, imported from Germany. Material type left BLANK: the sheet states no core construction for this line and no supplier subsection exists to default it. Waterproof = FALSE (no water claim printed). 1286 x 194 x 12mm; Width (in) 7.64 converted from 194mm. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - Inhaus 12mm AC4 - Dynamic Highlands (Hemlock (Dark Beige))  |". Inhaus 12mm AC4 Laminate, MegaLoc (G5) locking, imported from Germany. Material type left BLANK: the sheet states no core construction for this line and no supplier subsection exists to default it. Waterproof = FALSE (no water claim printed). 1286 x 194 x 12mm; Width (in) 7.64 converted from 194mm. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF213" t="inlineStr">
@@ -25073,7 +25073,7 @@
       </c>
       <c r="BC214" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - Inhaus 12mm AC4 - Dynamic Highlands (Quarry Oak)  | #35726 | ". Inhaus 12mm AC4 Laminate, MegaLoc (G5) locking, imported from Germany. Material type left BLANK: the sheet states no core construction for this line and no supplier subsection exists to default it. Waterproof = FALSE (no water claim printed). 1286 x 194 x 12mm; Width (in) 7.64 converted from 194mm. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - Inhaus 12mm AC4 - Dynamic Highlands (Quarry Oak)  | #35726 | ". Inhaus 12mm AC4 Laminate, MegaLoc (G5) locking, imported from Germany. Material type left BLANK: the sheet states no core construction for this line and no supplier subsection exists to default it. Waterproof = FALSE (no water claim printed). 1286 x 194 x 12mm; Width (in) 7.64 converted from 194mm. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF214" t="inlineStr">
@@ -25198,7 +25198,7 @@
       </c>
       <c r="BC215" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - Inhaus 12mm AC5 - Dynamic Highlands (Lismore (Beige Grey))  |". Inhaus 12mm AC4 Laminate, MegaLoc (G5) locking, imported from Germany. Material type left BLANK: the sheet states no core construction for this line and no supplier subsection exists to default it. Waterproof = FALSE (no water claim printed). 1286 x 194 x 12mm; Width (in) 7.64 converted from 194mm. Supplier header: 'DISCONTINUED (LIMITED STOCK ON BELOW ITEMS)' -&gt; phased out with limited remaining inventory = Clearance (kept Active). COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - Inhaus 12mm AC5 - Dynamic Highlands (Lismore (Beige Grey))  |". Inhaus 12mm AC4 Laminate, MegaLoc (G5) locking, imported from Germany. Material type left BLANK: the sheet states no core construction for this line and no supplier subsection exists to default it. Waterproof = FALSE (no water claim printed). 1286 x 194 x 12mm; Width (in) 7.64 converted from 194mm. Supplier header: 'DISCONTINUED (LIMITED STOCK ON BELOW ITEMS)' -&gt; phased out with limited remaining inventory = Clearance (kept Active). COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF215" t="inlineStr">
@@ -25323,7 +25323,7 @@
       </c>
       <c r="BC216" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - Inhaus 12mm AC6 - Dynamic Highlands (Rustic Pecan(Pecan Brown". Inhaus 12mm AC4 Laminate, MegaLoc (G5) locking, imported from Germany. Material type left BLANK: the sheet states no core construction for this line and no supplier subsection exists to default it. Waterproof = FALSE (no water claim printed). 1286 x 194 x 12mm; Width (in) 7.64 converted from 194mm. Supplier header: 'DISCONTINUED (LIMITED STOCK ON BELOW ITEMS)' -&gt; phased out with limited remaining inventory = Clearance (kept Active). COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - Inhaus 12mm AC6 - Dynamic Highlands (Rustic Pecan(Pecan Brown". Inhaus 12mm AC4 Laminate, MegaLoc (G5) locking, imported from Germany. Material type left BLANK: the sheet states no core construction for this line and no supplier subsection exists to default it. Waterproof = FALSE (no water claim printed). 1286 x 194 x 12mm; Width (in) 7.64 converted from 194mm. Supplier header: 'DISCONTINUED (LIMITED STOCK ON BELOW ITEMS)' -&gt; phased out with limited remaining inventory = Clearance (kept Active). COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF216" t="inlineStr">
@@ -25448,7 +25448,7 @@
       </c>
       <c r="BC217" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - Inhaus 12mm AC4 - Dynamic Highlands (Shasta Oak)  | #44335 | ". Inhaus 12mm AC4 Laminate, MegaLoc (G5) locking, imported from Germany. Material type left BLANK: the sheet states no core construction for this line and no supplier subsection exists to default it. Waterproof = FALSE (no water claim printed). 1286 x 194 x 12mm; Width (in) 7.64 converted from 194mm. Supplier header: 'DISCONTINUED (LIMITED STOCK ON BELOW ITEMS)' -&gt; phased out with limited remaining inventory = Clearance (kept Active). COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - Inhaus 12mm AC4 - Dynamic Highlands (Shasta Oak)  | #44335 | ". Inhaus 12mm AC4 Laminate, MegaLoc (G5) locking, imported from Germany. Material type left BLANK: the sheet states no core construction for this line and no supplier subsection exists to default it. Waterproof = FALSE (no water claim printed). 1286 x 194 x 12mm; Width (in) 7.64 converted from 194mm. Supplier header: 'DISCONTINUED (LIMITED STOCK ON BELOW ITEMS)' -&gt; phased out with limited remaining inventory = Clearance (kept Active). COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF217" t="inlineStr">
@@ -25568,7 +25568,7 @@
       </c>
       <c r="BC218" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - Inhaus 12mm AC4 - Dynamic Highlands (Canyon Oak)  | #44333 | ". Inhaus 12mm AC4 Laminate, MegaLoc (G5) locking, imported from Germany. Material type left BLANK: the sheet states no core construction for this line and no supplier subsection exists to default it. Waterproof = FALSE (no water claim printed). 1286 x 160 x 12mm; Width (in) 6.3 converted from 160mm. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - Inhaus 12mm AC4 - Dynamic Highlands (Canyon Oak)  | #44333 | ". Inhaus 12mm AC4 Laminate, MegaLoc (G5) locking, imported from Germany. Material type left BLANK: the sheet states no core construction for this line and no supplier subsection exists to default it. Waterproof = FALSE (no water claim printed). 1286 x 160 x 12mm; Width (in) 6.3 converted from 160mm. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF218" t="inlineStr">
@@ -25688,7 +25688,7 @@
       </c>
       <c r="BC219" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - Inhaus 12mm AC4 - Natural Vintage (Hartford)  | #44314 | AC4 ". Inhaus 12mm AC4 Laminate, MegaLoc (G5) locking, imported from Germany. Material type left BLANK: the sheet states no core construction for this line and no supplier subsection exists to default it. Waterproof = FALSE (no water claim printed). 1286 x 160 x 12mm; Width (in) 6.3 converted from 160mm. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - Inhaus 12mm AC4 - Natural Vintage (Hartford)  | #44314 | AC4 ". Inhaus 12mm AC4 Laminate, MegaLoc (G5) locking, imported from Germany. Material type left BLANK: the sheet states no core construction for this line and no supplier subsection exists to default it. Waterproof = FALSE (no water claim printed). 1286 x 160 x 12mm; Width (in) 6.3 converted from 160mm. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF219" t="inlineStr">
@@ -25813,7 +25813,7 @@
       </c>
       <c r="BC220" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - Inhaus 12mm AC4 - Natural Vintage (Tofino)  | #45604 | AC4 - ". Inhaus 12mm AC4 Laminate, MegaLoc (G5) locking, imported from Germany. Material type left BLANK: the sheet states no core construction for this line and no supplier subsection exists to default it. Waterproof = FALSE (no water claim printed). 1286 x 160 x 12mm; Width (in) 6.3 converted from 160mm. Supplier header: 'DISCONTINUED (LIMITED STOCK ON BELOW ITEMS)' -&gt; phased out with limited remaining inventory = Clearance (kept Active). COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - Inhaus 12mm AC4 - Natural Vintage (Tofino)  | #45604 | AC4 - ". Inhaus 12mm AC4 Laminate, MegaLoc (G5) locking, imported from Germany. Material type left BLANK: the sheet states no core construction for this line and no supplier subsection exists to default it. Waterproof = FALSE (no water claim printed). 1286 x 160 x 12mm; Width (in) 6.3 converted from 160mm. Supplier header: 'DISCONTINUED (LIMITED STOCK ON BELOW ITEMS)' -&gt; phased out with limited remaining inventory = Clearance (kept Active). COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF220" t="inlineStr">
@@ -25933,7 +25933,7 @@
       </c>
       <c r="BC221" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - Inhaus 12mm AC4 - Precious Highlands (Mountain)  | #35714 | A". Inhaus 12mm AC4 Laminate, MegaLoc (G5) locking, imported from Germany. Material type left BLANK: the sheet states no core construction for this line and no supplier subsection exists to default it. Waterproof = FALSE (no water claim printed). 1286 x 160 x 12mm; Width (in) 6.3 converted from 160mm. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - Inhaus 12mm AC4 - Precious Highlands (Mountain)  | #35714 | A". Inhaus 12mm AC4 Laminate, MegaLoc (G5) locking, imported from Germany. Material type left BLANK: the sheet states no core construction for this line and no supplier subsection exists to default it. Waterproof = FALSE (no water claim printed). 1286 x 160 x 12mm; Width (in) 6.3 converted from 160mm. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF221" t="inlineStr">
@@ -26058,7 +26058,7 @@
       </c>
       <c r="BC222" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - Inhaus 12mm AC5 - Precious Highlands (Vancouver Walnut)  | #4". Inhaus 12mm AC4 Laminate, MegaLoc (G5) locking, imported from Germany. Material type left BLANK: the sheet states no core construction for this line and no supplier subsection exists to default it. Waterproof = FALSE (no water claim printed). 1286 x 160 x 12mm; Width (in) 6.3 converted from 160mm. Supplier header: 'DISCONTINUED (LIMITED STOCK ON BELOW ITEMS)' -&gt; phased out with limited remaining inventory = Clearance (kept Active). COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - Inhaus 12mm AC5 - Precious Highlands (Vancouver Walnut)  | #4". Inhaus 12mm AC4 Laminate, MegaLoc (G5) locking, imported from Germany. Material type left BLANK: the sheet states no core construction for this line and no supplier subsection exists to default it. Waterproof = FALSE (no water claim printed). 1286 x 160 x 12mm; Width (in) 6.3 converted from 160mm. Supplier header: 'DISCONTINUED (LIMITED STOCK ON BELOW ITEMS)' -&gt; phased out with limited remaining inventory = Clearance (kept Active). COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF222" t="inlineStr">
@@ -26178,7 +26178,7 @@
       </c>
       <c r="BC223" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - Elandura Plank 4mm+1mm AC4 - Wood Grain (Caraway)  | #55031 |". Inhaus Elandura '4mm+1mm AC4 Rigid Core', MegaLoc (G5), imported from Germany. AMBIGUOUS CATEGORY: a rigid-core product that also carries an AC (laminate abrasion) rating - it could equally be Laminate. Assigned on plank-vs-tile format; Material type left BLANK because the sheet says only 'Rigid Core' (not SPC/WPC). Thickness 5mm = 4mm core + 1mm assumed attached pad (pad material not named). Confirm construction with Albert/supplier. 50.79 in (1290mm) x 6.81 in (173mm). COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - Elandura Plank 4mm+1mm AC4 - Wood Grain (Caraway)  | #55031 |". Inhaus Elandura '4mm+1mm AC4 Rigid Core', MegaLoc (G5), imported from Germany. AMBIGUOUS CATEGORY: a rigid-core product that also carries an AC (laminate abrasion) rating - it could equally be Laminate. Assigned on plank-vs-tile format; Material type left BLANK because the sheet says only 'Rigid Core' (not SPC/WPC). Thickness 5mm = 4mm core + 1mm assumed attached pad (pad material not named). Confirm construction with Albert/supplier. 50.79 in (1290mm) x 6.81 in (173mm). COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF223" t="inlineStr">
@@ -26298,7 +26298,7 @@
       </c>
       <c r="BC224" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - Elandura Plank 4mm+1mm AC4 - Wood Grain (Clove)  | #55030 |  ". Inhaus Elandura '4mm+1mm AC4 Rigid Core', MegaLoc (G5), imported from Germany. AMBIGUOUS CATEGORY: a rigid-core product that also carries an AC (laminate abrasion) rating - it could equally be Laminate. Assigned on plank-vs-tile format; Material type left BLANK because the sheet says only 'Rigid Core' (not SPC/WPC). Thickness 5mm = 4mm core + 1mm assumed attached pad (pad material not named). Confirm construction with Albert/supplier. 50.79 in (1290mm) x 6.81 in (173mm). COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - Elandura Plank 4mm+1mm AC4 - Wood Grain (Clove)  | #55030 |  ". Inhaus Elandura '4mm+1mm AC4 Rigid Core', MegaLoc (G5), imported from Germany. AMBIGUOUS CATEGORY: a rigid-core product that also carries an AC (laminate abrasion) rating - it could equally be Laminate. Assigned on plank-vs-tile format; Material type left BLANK because the sheet says only 'Rigid Core' (not SPC/WPC). Thickness 5mm = 4mm core + 1mm assumed attached pad (pad material not named). Confirm construction with Albert/supplier. 50.79 in (1290mm) x 6.81 in (173mm). COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF224" t="inlineStr">
@@ -26418,7 +26418,7 @@
       </c>
       <c r="BC225" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - Elandura Plank 4mm+1mm AC4 - Wood Grain (Gilmour)  | #55024 |". Inhaus Elandura '4mm+1mm AC4 Rigid Core', MegaLoc (G5), imported from Germany. AMBIGUOUS CATEGORY: a rigid-core product that also carries an AC (laminate abrasion) rating - it could equally be Laminate. Assigned on plank-vs-tile format; Material type left BLANK because the sheet says only 'Rigid Core' (not SPC/WPC). Thickness 5mm = 4mm core + 1mm assumed attached pad (pad material not named). Confirm construction with Albert/supplier. 50.79 in (1290mm) x 6.81 in (173mm). COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - Elandura Plank 4mm+1mm AC4 - Wood Grain (Gilmour)  | #55024 |". Inhaus Elandura '4mm+1mm AC4 Rigid Core', MegaLoc (G5), imported from Germany. AMBIGUOUS CATEGORY: a rigid-core product that also carries an AC (laminate abrasion) rating - it could equally be Laminate. Assigned on plank-vs-tile format; Material type left BLANK because the sheet says only 'Rigid Core' (not SPC/WPC). Thickness 5mm = 4mm core + 1mm assumed attached pad (pad material not named). Confirm construction with Albert/supplier. 50.79 in (1290mm) x 6.81 in (173mm). COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF225" t="inlineStr">
@@ -26538,7 +26538,7 @@
       </c>
       <c r="BC226" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - Elandura Plank 4mm+1mm AC4 - Wood Grain (Seaside)  | #55027 |". Inhaus Elandura '4mm+1mm AC4 Rigid Core', MegaLoc (G5), imported from Germany. AMBIGUOUS CATEGORY: a rigid-core product that also carries an AC (laminate abrasion) rating - it could equally be Laminate. Assigned on plank-vs-tile format; Material type left BLANK because the sheet says only 'Rigid Core' (not SPC/WPC). Thickness 5mm = 4mm core + 1mm assumed attached pad (pad material not named). Confirm construction with Albert/supplier. 50.79 in (1290mm) x 6.81 in (173mm). COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - Elandura Plank 4mm+1mm AC4 - Wood Grain (Seaside)  | #55027 |". Inhaus Elandura '4mm+1mm AC4 Rigid Core', MegaLoc (G5), imported from Germany. AMBIGUOUS CATEGORY: a rigid-core product that also carries an AC (laminate abrasion) rating - it could equally be Laminate. Assigned on plank-vs-tile format; Material type left BLANK because the sheet says only 'Rigid Core' (not SPC/WPC). Thickness 5mm = 4mm core + 1mm assumed attached pad (pad material not named). Confirm construction with Albert/supplier. 50.79 in (1290mm) x 6.81 in (173mm). COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF226" t="inlineStr">
@@ -26658,7 +26658,7 @@
       </c>
       <c r="BC227" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - Elandura Plank 4mm+1mm AC4 - Wood Grain (Silver Sand)  | #550". Inhaus Elandura '4mm+1mm AC4 Rigid Core', MegaLoc (G5), imported from Germany. AMBIGUOUS CATEGORY: a rigid-core product that also carries an AC (laminate abrasion) rating - it could equally be Laminate. Assigned on plank-vs-tile format; Material type left BLANK because the sheet says only 'Rigid Core' (not SPC/WPC). Thickness 5mm = 4mm core + 1mm assumed attached pad (pad material not named). Confirm construction with Albert/supplier. 50.79 in (1290mm) x 6.81 in (173mm). COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - Elandura Plank 4mm+1mm AC4 - Wood Grain (Silver Sand)  | #550". Inhaus Elandura '4mm+1mm AC4 Rigid Core', MegaLoc (G5), imported from Germany. AMBIGUOUS CATEGORY: a rigid-core product that also carries an AC (laminate abrasion) rating - it could equally be Laminate. Assigned on plank-vs-tile format; Material type left BLANK because the sheet says only 'Rigid Core' (not SPC/WPC). Thickness 5mm = 4mm core + 1mm assumed attached pad (pad material not named). Confirm construction with Albert/supplier. 50.79 in (1290mm) x 6.81 in (173mm). COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF227" t="inlineStr">
@@ -26778,7 +26778,7 @@
       </c>
       <c r="BC228" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - Elandura Plank 4mm+1mm AC4 - Wood Grain (Sutter)  | #54954 | ". Inhaus Elandura '4mm+1mm AC4 Rigid Core', MegaLoc (G5), imported from Germany. AMBIGUOUS CATEGORY: a rigid-core product that also carries an AC (laminate abrasion) rating - it could equally be Laminate. Assigned on plank-vs-tile format; Material type left BLANK because the sheet says only 'Rigid Core' (not SPC/WPC). Thickness 5mm = 4mm core + 1mm assumed attached pad (pad material not named). Confirm construction with Albert/supplier. 50.79 in (1290mm) x 6.81 in (173mm). COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - Elandura Plank 4mm+1mm AC4 - Wood Grain (Sutter)  | #54954 | ". Inhaus Elandura '4mm+1mm AC4 Rigid Core', MegaLoc (G5), imported from Germany. AMBIGUOUS CATEGORY: a rigid-core product that also carries an AC (laminate abrasion) rating - it could equally be Laminate. Assigned on plank-vs-tile format; Material type left BLANK because the sheet says only 'Rigid Core' (not SPC/WPC). Thickness 5mm = 4mm core + 1mm assumed attached pad (pad material not named). Confirm construction with Albert/supplier. 50.79 in (1290mm) x 6.81 in (173mm). COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF228" t="inlineStr">
@@ -26898,7 +26898,7 @@
       </c>
       <c r="BC229" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - Elandura Plank 4mm+1mm AC4 - Wood Grain (Terra)  | #54955 |  ". Inhaus Elandura '4mm+1mm AC4 Rigid Core', MegaLoc (G5), imported from Germany. AMBIGUOUS CATEGORY: a rigid-core product that also carries an AC (laminate abrasion) rating - it could equally be Laminate. Assigned on plank-vs-tile format; Material type left BLANK because the sheet says only 'Rigid Core' (not SPC/WPC). Thickness 5mm = 4mm core + 1mm assumed attached pad (pad material not named). Confirm construction with Albert/supplier. 50.79 in (1290mm) x 6.81 in (173mm). COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - Elandura Plank 4mm+1mm AC4 - Wood Grain (Terra)  | #54955 |  ". Inhaus Elandura '4mm+1mm AC4 Rigid Core', MegaLoc (G5), imported from Germany. AMBIGUOUS CATEGORY: a rigid-core product that also carries an AC (laminate abrasion) rating - it could equally be Laminate. Assigned on plank-vs-tile format; Material type left BLANK because the sheet says only 'Rigid Core' (not SPC/WPC). Thickness 5mm = 4mm core + 1mm assumed attached pad (pad material not named). Confirm construction with Albert/supplier. 50.79 in (1290mm) x 6.81 in (173mm). COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF229" t="inlineStr">
@@ -27018,7 +27018,7 @@
       </c>
       <c r="BC230" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - Elandura Plank 4mm+1mm AC4 - Wood Grain (Tuscan)  | #55029 | ". Inhaus Elandura '4mm+1mm AC4 Rigid Core', MegaLoc (G5), imported from Germany. AMBIGUOUS CATEGORY: a rigid-core product that also carries an AC (laminate abrasion) rating - it could equally be Laminate. Assigned on plank-vs-tile format; Material type left BLANK because the sheet says only 'Rigid Core' (not SPC/WPC). Thickness 5mm = 4mm core + 1mm assumed attached pad (pad material not named). Confirm construction with Albert/supplier. 50.79 in (1290mm) x 6.81 in (173mm). COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - Elandura Plank 4mm+1mm AC4 - Wood Grain (Tuscan)  | #55029 | ". Inhaus Elandura '4mm+1mm AC4 Rigid Core', MegaLoc (G5), imported from Germany. AMBIGUOUS CATEGORY: a rigid-core product that also carries an AC (laminate abrasion) rating - it could equally be Laminate. Assigned on plank-vs-tile format; Material type left BLANK because the sheet says only 'Rigid Core' (not SPC/WPC). Thickness 5mm = 4mm core + 1mm assumed attached pad (pad material not named). Confirm construction with Albert/supplier. 50.79 in (1290mm) x 6.81 in (173mm). COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF230" t="inlineStr">
@@ -27138,7 +27138,7 @@
       </c>
       <c r="BC231" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - Elandura Plank 4mm+1mm AC4 - Wood Grain (Umber)  | #54957 |  ". Inhaus Elandura '4mm+1mm AC4 Rigid Core', MegaLoc (G5), imported from Germany. AMBIGUOUS CATEGORY: a rigid-core product that also carries an AC (laminate abrasion) rating - it could equally be Laminate. Assigned on plank-vs-tile format; Material type left BLANK because the sheet says only 'Rigid Core' (not SPC/WPC). Thickness 5mm = 4mm core + 1mm assumed attached pad (pad material not named). Confirm construction with Albert/supplier. 50.79 in (1290mm) x 6.81 in (173mm). COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - Elandura Plank 4mm+1mm AC4 - Wood Grain (Umber)  | #54957 |  ". Inhaus Elandura '4mm+1mm AC4 Rigid Core', MegaLoc (G5), imported from Germany. AMBIGUOUS CATEGORY: a rigid-core product that also carries an AC (laminate abrasion) rating - it could equally be Laminate. Assigned on plank-vs-tile format; Material type left BLANK because the sheet says only 'Rigid Core' (not SPC/WPC). Thickness 5mm = 4mm core + 1mm assumed attached pad (pad material not named). Confirm construction with Albert/supplier. 50.79 in (1290mm) x 6.81 in (173mm). COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF231" t="inlineStr">
@@ -27258,7 +27258,7 @@
       </c>
       <c r="BC232" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - Elandura Plank 4mm+1mm AC4 - Wood Grain (Urban)  | #55026 |  ". Inhaus Elandura '4mm+1mm AC4 Rigid Core', MegaLoc (G5), imported from Germany. AMBIGUOUS CATEGORY: a rigid-core product that also carries an AC (laminate abrasion) rating - it could equally be Laminate. Assigned on plank-vs-tile format; Material type left BLANK because the sheet says only 'Rigid Core' (not SPC/WPC). Thickness 5mm = 4mm core + 1mm assumed attached pad (pad material not named). Confirm construction with Albert/supplier. 50.79 in (1290mm) x 6.81 in (173mm). COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - Elandura Plank 4mm+1mm AC4 - Wood Grain (Urban)  | #55026 |  ". Inhaus Elandura '4mm+1mm AC4 Rigid Core', MegaLoc (G5), imported from Germany. AMBIGUOUS CATEGORY: a rigid-core product that also carries an AC (laminate abrasion) rating - it could equally be Laminate. Assigned on plank-vs-tile format; Material type left BLANK because the sheet says only 'Rigid Core' (not SPC/WPC). Thickness 5mm = 4mm core + 1mm assumed attached pad (pad material not named). Confirm construction with Albert/supplier. 50.79 in (1290mm) x 6.81 in (173mm). COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF232" t="inlineStr">
@@ -27378,7 +27378,7 @@
       </c>
       <c r="BC233" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - Elandura Plank 4mm+1mm AC4 - Wood Grain (Woodwind)  | #55028 ". Inhaus Elandura '4mm+1mm AC4 Rigid Core', MegaLoc (G5), imported from Germany. AMBIGUOUS CATEGORY: a rigid-core product that also carries an AC (laminate abrasion) rating - it could equally be Laminate. Assigned on plank-vs-tile format; Material type left BLANK because the sheet says only 'Rigid Core' (not SPC/WPC). Thickness 5mm = 4mm core + 1mm assumed attached pad (pad material not named). Confirm construction with Albert/supplier. 50.79 in (1290mm) x 6.81 in (173mm). COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - Elandura Plank 4mm+1mm AC4 - Wood Grain (Woodwind)  | #55028 ". Inhaus Elandura '4mm+1mm AC4 Rigid Core', MegaLoc (G5), imported from Germany. AMBIGUOUS CATEGORY: a rigid-core product that also carries an AC (laminate abrasion) rating - it could equally be Laminate. Assigned on plank-vs-tile format; Material type left BLANK because the sheet says only 'Rigid Core' (not SPC/WPC). Thickness 5mm = 4mm core + 1mm assumed attached pad (pad material not named). Confirm construction with Albert/supplier. 50.79 in (1290mm) x 6.81 in (173mm). COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF233" t="inlineStr">
@@ -27498,7 +27498,7 @@
       </c>
       <c r="BC234" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - Elandura Tile 4mm+1mm AC4 - Minipearl (Hazelnut)  | #54956 | ". Inhaus Elandura '4mm+1mm AC4 Rigid Core', MegaLoc (G5), imported from Germany. AMBIGUOUS CATEGORY: a rigid-core product that also carries an AC (laminate abrasion) rating - it could equally be Laminate. Assigned on plank-vs-tile format; Material type left BLANK because the sheet says only 'Rigid Core' (not SPC/WPC). Thickness 5mm = 4mm core + 1mm assumed attached pad (pad material not named). Confirm construction with Albert/supplier. 25.12 in (638mm) x 12.2 in (310mm). 'Minipearl' is printed with NO product code - Supplier SKU left blank (never invented). COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - Elandura Tile 4mm+1mm AC4 - Minipearl (Hazelnut)  | #54956 | ". Inhaus Elandura '4mm+1mm AC4 Rigid Core', MegaLoc (G5), imported from Germany. AMBIGUOUS CATEGORY: a rigid-core product that also carries an AC (laminate abrasion) rating - it could equally be Laminate. Assigned on plank-vs-tile format; Material type left BLANK because the sheet says only 'Rigid Core' (not SPC/WPC). Thickness 5mm = 4mm core + 1mm assumed attached pad (pad material not named). Confirm construction with Albert/supplier. 25.12 in (638mm) x 12.2 in (310mm). 'Minipearl' is printed with NO product code - Supplier SKU left blank (never invented). COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF234" t="inlineStr">
@@ -27608,7 +27608,7 @@
       </c>
       <c r="BC235" t="inlineStr">
         <is>
-          <t>Inhaus Elandura '4mm+1mm AC4 Rigid Core', MegaLoc (G5), imported from Germany. AMBIGUOUS CATEGORY: a rigid-core product that also carries an AC (laminate abrasion) rating - it could equally be Laminate. Assigned on plank-vs-tile format; Material type left BLANK because the sheet says only 'Rigid Core' (not SPC/WPC). Thickness 5mm = 4mm core + 1mm assumed attached pad (pad material not named). Confirm construction with Albert/supplier. 25.12 in (638mm) x 12.2 in (310mm). 'Minipearl' is printed with NO product code - Supplier SKU left blank (never invented). COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>Inhaus Elandura '4mm+1mm AC4 Rigid Core', MegaLoc (G5), imported from Germany. AMBIGUOUS CATEGORY: a rigid-core product that also carries an AC (laminate abrasion) rating - it could equally be Laminate. Assigned on plank-vs-tile format; Material type left BLANK because the sheet says only 'Rigid Core' (not SPC/WPC). Thickness 5mm = 4mm core + 1mm assumed attached pad (pad material not named). Confirm construction with Albert/supplier. 25.12 in (638mm) x 12.2 in (310mm). 'Minipearl' is printed with NO product code - Supplier SKU left blank (never invented). COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF235" t="inlineStr">
@@ -27728,7 +27728,7 @@
       </c>
       <c r="BC236" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - Elandura Tile 4mm+1mm AC4 - Minipearl (Mist)  | #54948 |  - 2". Inhaus Elandura '4mm+1mm AC4 Rigid Core', MegaLoc (G5), imported from Germany. AMBIGUOUS CATEGORY: a rigid-core product that also carries an AC (laminate abrasion) rating - it could equally be Laminate. Assigned on plank-vs-tile format; Material type left BLANK because the sheet says only 'Rigid Core' (not SPC/WPC). Thickness 5mm = 4mm core + 1mm assumed attached pad (pad material not named). Confirm construction with Albert/supplier. 25.12 in (638mm) x 12.2 in (310mm). 'Minipearl' is printed with NO product code - Supplier SKU left blank (never invented). COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - Elandura Tile 4mm+1mm AC4 - Minipearl (Mist)  | #54948 |  - 2". Inhaus Elandura '4mm+1mm AC4 Rigid Core', MegaLoc (G5), imported from Germany. AMBIGUOUS CATEGORY: a rigid-core product that also carries an AC (laminate abrasion) rating - it could equally be Laminate. Assigned on plank-vs-tile format; Material type left BLANK because the sheet says only 'Rigid Core' (not SPC/WPC). Thickness 5mm = 4mm core + 1mm assumed attached pad (pad material not named). Confirm construction with Albert/supplier. 25.12 in (638mm) x 12.2 in (310mm). 'Minipearl' is printed with NO product code - Supplier SKU left blank (never invented). COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF236" t="inlineStr">
@@ -27848,7 +27848,7 @@
       </c>
       <c r="BC237" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - Inspiration - Lamdura 8mm AC4 - Wood Collection (Edgewood)  |". Inhaus Inspiration - Lamdura 8mm AC4 'Aqua Protect', MegaLoc, imported from Germany. 50.59" (1285mm) x 7.56 in (192mm) x 8mm. Waterproof left BLANK - 'Aqua Protect' is a water-resistance claim, not a waterproof claim; Material type = Water-Resistant Core on that basis. '(Handscraped EIR)' kept in the colour name as printed and mirrored in Finish type where present. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - Inspiration - Lamdura 8mm AC4 - Wood Collection (Edgewood)  |". Inhaus Inspiration - Lamdura 8mm AC4 'Aqua Protect', MegaLoc, imported from Germany. 50.59" (1285mm) x 7.56 in (192mm) x 8mm. Waterproof left BLANK - 'Aqua Protect' is a water-resistance claim, not a waterproof claim; Material type = Water-Resistant Core on that basis. '(Handscraped EIR)' kept in the colour name as printed and mirrored in Finish type where present. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF237" t="inlineStr">
@@ -27968,7 +27968,7 @@
       </c>
       <c r="BC238" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - Inspiration - Lamdura 8mm AC4 - Wood Collection (Grizzly (Han". Inhaus Inspiration - Lamdura 8mm AC4 'Aqua Protect', MegaLoc, imported from Germany. 50.59" (1285mm) x 7.56 in (192mm) x 8mm. Waterproof left BLANK - 'Aqua Protect' is a water-resistance claim, not a waterproof claim; Material type = Water-Resistant Core on that basis. '(Handscraped EIR)' kept in the colour name as printed and mirrored in Finish type where present. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - Inspiration - Lamdura 8mm AC4 - Wood Collection (Grizzly (Han". Inhaus Inspiration - Lamdura 8mm AC4 'Aqua Protect', MegaLoc, imported from Germany. 50.59" (1285mm) x 7.56 in (192mm) x 8mm. Waterproof left BLANK - 'Aqua Protect' is a water-resistance claim, not a waterproof claim; Material type = Water-Resistant Core on that basis. '(Handscraped EIR)' kept in the colour name as printed and mirrored in Finish type where present. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF238" t="inlineStr">
@@ -28088,7 +28088,7 @@
       </c>
       <c r="BC239" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - Inspiration - Lamdura 8mm AC4 - Wood Collection (Folkstone (H". Inhaus Inspiration - Lamdura 8mm AC4 'Aqua Protect', MegaLoc, imported from Germany. 50.59" (1285mm) x 7.56 in (192mm) x 8mm. Waterproof left BLANK - 'Aqua Protect' is a water-resistance claim, not a waterproof claim; Material type = Water-Resistant Core on that basis. '(Handscraped EIR)' kept in the colour name as printed and mirrored in Finish type where present. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - Inspiration - Lamdura 8mm AC4 - Wood Collection (Folkstone (H". Inhaus Inspiration - Lamdura 8mm AC4 'Aqua Protect', MegaLoc, imported from Germany. 50.59" (1285mm) x 7.56 in (192mm) x 8mm. Waterproof left BLANK - 'Aqua Protect' is a water-resistance claim, not a waterproof claim; Material type = Water-Resistant Core on that basis. '(Handscraped EIR)' kept in the colour name as printed and mirrored in Finish type where present. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF239" t="inlineStr">
@@ -28208,7 +28208,7 @@
       </c>
       <c r="BC240" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - Inspiration - Lamdura 8mm AC4 - Wood Collection (Oak Light Gr". Inhaus Inspiration - Lamdura 8mm AC4 'Aqua Protect', MegaLoc, imported from Germany. 50.59" (1285mm) x 7.56 in (192mm) x 8mm. Waterproof left BLANK - 'Aqua Protect' is a water-resistance claim, not a waterproof claim; Material type = Water-Resistant Core on that basis. '(Handscraped EIR)' kept in the colour name as printed and mirrored in Finish type where present. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - Inspiration - Lamdura 8mm AC4 - Wood Collection (Oak Light Gr". Inhaus Inspiration - Lamdura 8mm AC4 'Aqua Protect', MegaLoc, imported from Germany. 50.59" (1285mm) x 7.56 in (192mm) x 8mm. Waterproof left BLANK - 'Aqua Protect' is a water-resistance claim, not a waterproof claim; Material type = Water-Resistant Core on that basis. '(Handscraped EIR)' kept in the colour name as printed and mirrored in Finish type where present. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF240" t="inlineStr">
@@ -28328,7 +28328,7 @@
       </c>
       <c r="BC241" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - Inspiration - Lamdura 8mm AC4 - Wood Collection (Sedgwick)  |". Inhaus Inspiration - Lamdura 8mm AC4 'Aqua Protect', MegaLoc, imported from Germany. 50.59" (1285mm) x 7.56 in (192mm) x 8mm. Waterproof left BLANK - 'Aqua Protect' is a water-resistance claim, not a waterproof claim; Material type = Water-Resistant Core on that basis. '(Handscraped EIR)' kept in the colour name as printed and mirrored in Finish type where present. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - Inspiration - Lamdura 8mm AC4 - Wood Collection (Sedgwick)  |". Inhaus Inspiration - Lamdura 8mm AC4 'Aqua Protect', MegaLoc, imported from Germany. 50.59" (1285mm) x 7.56 in (192mm) x 8mm. Waterproof left BLANK - 'Aqua Protect' is a water-resistance claim, not a waterproof claim; Material type = Water-Resistant Core on that basis. '(Handscraped EIR)' kept in the colour name as printed and mirrored in Finish type where present. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF241" t="inlineStr">
@@ -28448,7 +28448,7 @@
       </c>
       <c r="BC242" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - Inspiration - Lamdura 8mm AC4 - Wood Collection (Selkirk)  | ". Inhaus Inspiration - Lamdura 8mm AC4 'Aqua Protect', MegaLoc, imported from Germany. 50.59" (1285mm) x 7.56 in (192mm) x 8mm. Waterproof left BLANK - 'Aqua Protect' is a water-resistance claim, not a waterproof claim; Material type = Water-Resistant Core on that basis. '(Handscraped EIR)' kept in the colour name as printed and mirrored in Finish type where present. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - Inspiration - Lamdura 8mm AC4 - Wood Collection (Selkirk)  | ". Inhaus Inspiration - Lamdura 8mm AC4 'Aqua Protect', MegaLoc, imported from Germany. 50.59" (1285mm) x 7.56 in (192mm) x 8mm. Waterproof left BLANK - 'Aqua Protect' is a water-resistance claim, not a waterproof claim; Material type = Water-Resistant Core on that basis. '(Handscraped EIR)' kept in the colour name as printed and mirrored in Finish type where present. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF242" t="inlineStr">
@@ -28568,7 +28568,7 @@
       </c>
       <c r="BC243" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - Inspiration - Lamdura 8mm AC4 - Wood Collection (Tisdale (Han". Inhaus Inspiration - Lamdura 8mm AC4 'Aqua Protect', MegaLoc, imported from Germany. 50.59" (1285mm) x 7.56 in (192mm) x 8mm. Waterproof left BLANK - 'Aqua Protect' is a water-resistance claim, not a waterproof claim; Material type = Water-Resistant Core on that basis. '(Handscraped EIR)' kept in the colour name as printed and mirrored in Finish type where present. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - Inspiration - Lamdura 8mm AC4 - Wood Collection (Tisdale (Han". Inhaus Inspiration - Lamdura 8mm AC4 'Aqua Protect', MegaLoc, imported from Germany. 50.59" (1285mm) x 7.56 in (192mm) x 8mm. Waterproof left BLANK - 'Aqua Protect' is a water-resistance claim, not a waterproof claim; Material type = Water-Resistant Core on that basis. '(Handscraped EIR)' kept in the colour name as printed and mirrored in Finish type where present. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF243" t="inlineStr">
@@ -28688,7 +28688,7 @@
       </c>
       <c r="BC244" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - Inspiration - Lamdura 8mm AC4 - Wood Collection (Woodside)  |". Inhaus Inspiration - Lamdura 8mm AC4 'Aqua Protect', MegaLoc, imported from Germany. 50.59" (1285mm) x 7.56 in (192mm) x 8mm. Waterproof left BLANK - 'Aqua Protect' is a water-resistance claim, not a waterproof claim; Material type = Water-Resistant Core on that basis. '(Handscraped EIR)' kept in the colour name as printed and mirrored in Finish type where present. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANLAM - Inspiration - Lamdura 8mm AC4 - Wood Collection (Woodside)  |". Inhaus Inspiration - Lamdura 8mm AC4 'Aqua Protect', MegaLoc, imported from Germany. 50.59" (1285mm) x 7.56 in (192mm) x 8mm. Waterproof left BLANK - 'Aqua Protect' is a water-resistance claim, not a waterproof claim; Material type = Water-Resistant Core on that basis. '(Handscraped EIR)' kept in the colour name as printed and mirrored in Finish type where present. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF244" t="inlineStr">
@@ -28816,7 +28816,7 @@
       </c>
       <c r="BC245" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANLAM - Inspiration - Lamdura 10mm AC4 - Wood Collection IIC74 Paddin". Inhaus Inspiration - Lamdura 10mm AC4 'Aqua Protect', MegaLoc, imported from Germany. 50.59" (1285mm) x 7.56 in (192mm), '8mm +2mm (Core Plus Pad)' -&gt; Thickness 10mm total, Underpad included = TRUE, Underpad type left blank (material not named). 'IIC74 Padding' -&gt; IIC rating 74; no STC printed. Pieces per box not printed for the 10mm line - 8 assumed from the 8-plank cartons on the sister lines; verify. Waterproof left BLANK ('Aqua Protect'). COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANLAM - Inspiration - Lamdura 10mm AC4 - Wood Collection IIC74 Paddin". Inhaus Inspiration - Lamdura 10mm AC4 'Aqua Protect', MegaLoc, imported from Germany. 50.59" (1285mm) x 7.56 in (192mm), '8mm +2mm (Core Plus Pad)' -&gt; Thickness 10mm total, Underpad included = TRUE, Underpad type left blank (material not named). 'IIC74 Padding' -&gt; IIC rating 74; no STC printed. Pieces per box not printed for the 10mm line - 8 assumed from the 8-plank cartons on the sister lines; verify. Waterproof left BLANK ('Aqua Protect'). COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF245" t="inlineStr">
@@ -28944,7 +28944,7 @@
       </c>
       <c r="BC246" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANLAM - Inspiration - Lamdura 10mm AC4 - Wood Collection IIC74 Paddin". Inhaus Inspiration - Lamdura 10mm AC4 'Aqua Protect', MegaLoc, imported from Germany. 50.59" (1285mm) x 7.56 in (192mm), '8mm +2mm (Core Plus Pad)' -&gt; Thickness 10mm total, Underpad included = TRUE, Underpad type left blank (material not named). 'IIC74 Padding' -&gt; IIC rating 74; no STC printed. Pieces per box not printed for the 10mm line - 8 assumed from the 8-plank cartons on the sister lines; verify. Waterproof left BLANK ('Aqua Protect'). COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANLAM - Inspiration - Lamdura 10mm AC4 - Wood Collection IIC74 Paddin". Inhaus Inspiration - Lamdura 10mm AC4 'Aqua Protect', MegaLoc, imported from Germany. 50.59" (1285mm) x 7.56 in (192mm), '8mm +2mm (Core Plus Pad)' -&gt; Thickness 10mm total, Underpad included = TRUE, Underpad type left blank (material not named). 'IIC74 Padding' -&gt; IIC rating 74; no STC printed. Pieces per box not printed for the 10mm line - 8 assumed from the 8-plank cartons on the sister lines; verify. Waterproof left BLANK ('Aqua Protect'). COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF246" t="inlineStr">
@@ -29072,7 +29072,7 @@
       </c>
       <c r="BC247" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANLAM - Inspiration - Lamdura 10mm AC4 - Wood Collection IIC74 Paddin". Inhaus Inspiration - Lamdura 10mm AC4 'Aqua Protect', MegaLoc, imported from Germany. 50.59" (1285mm) x 7.56 in (192mm), '8mm +2mm (Core Plus Pad)' -&gt; Thickness 10mm total, Underpad included = TRUE, Underpad type left blank (material not named). 'IIC74 Padding' -&gt; IIC rating 74; no STC printed. Pieces per box not printed for the 10mm line - 8 assumed from the 8-plank cartons on the sister lines; verify. Waterproof left BLANK ('Aqua Protect'). COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANLAM - Inspiration - Lamdura 10mm AC4 - Wood Collection IIC74 Paddin". Inhaus Inspiration - Lamdura 10mm AC4 'Aqua Protect', MegaLoc, imported from Germany. 50.59" (1285mm) x 7.56 in (192mm), '8mm +2mm (Core Plus Pad)' -&gt; Thickness 10mm total, Underpad included = TRUE, Underpad type left blank (material not named). 'IIC74 Padding' -&gt; IIC rating 74; no STC printed. Pieces per box not printed for the 10mm line - 8 assumed from the 8-plank cartons on the sister lines; verify. Waterproof left BLANK ('Aqua Protect'). COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF247" t="inlineStr">
@@ -29200,7 +29200,7 @@
       </c>
       <c r="BC248" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANLAM - Inspiration - Lamdura 10mm AC4 - Wood Collection IIC74 Paddin". Inhaus Inspiration - Lamdura 10mm AC4 'Aqua Protect', MegaLoc, imported from Germany. 50.59" (1285mm) x 7.56 in (192mm), '8mm +2mm (Core Plus Pad)' -&gt; Thickness 10mm total, Underpad included = TRUE, Underpad type left blank (material not named). 'IIC74 Padding' -&gt; IIC rating 74; no STC printed. Pieces per box not printed for the 10mm line - 8 assumed from the 8-plank cartons on the sister lines; verify. Waterproof left BLANK ('Aqua Protect'). COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANLAM - Inspiration - Lamdura 10mm AC4 - Wood Collection IIC74 Paddin". Inhaus Inspiration - Lamdura 10mm AC4 'Aqua Protect', MegaLoc, imported from Germany. 50.59" (1285mm) x 7.56 in (192mm), '8mm +2mm (Core Plus Pad)' -&gt; Thickness 10mm total, Underpad included = TRUE, Underpad type left blank (material not named). 'IIC74 Padding' -&gt; IIC rating 74; no STC printed. Pieces per box not printed for the 10mm line - 8 assumed from the 8-plank cartons on the sister lines; verify. Waterproof left BLANK ('Aqua Protect'). COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF248" t="inlineStr">
@@ -29328,7 +29328,7 @@
       </c>
       <c r="BC249" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANLAM - Inspiration - Lamdura 10mm AC4 - Wood Collection IIC74 Paddin". Inhaus Inspiration - Lamdura 10mm AC4 'Aqua Protect', MegaLoc, imported from Germany. 50.59" (1285mm) x 7.56 in (192mm), '8mm +2mm (Core Plus Pad)' -&gt; Thickness 10mm total, Underpad included = TRUE, Underpad type left blank (material not named). 'IIC74 Padding' -&gt; IIC rating 74; no STC printed. Pieces per box not printed for the 10mm line - 8 assumed from the 8-plank cartons on the sister lines; verify. Waterproof left BLANK ('Aqua Protect'). COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANLAM - Inspiration - Lamdura 10mm AC4 - Wood Collection IIC74 Paddin". Inhaus Inspiration - Lamdura 10mm AC4 'Aqua Protect', MegaLoc, imported from Germany. 50.59" (1285mm) x 7.56 in (192mm), '8mm +2mm (Core Plus Pad)' -&gt; Thickness 10mm total, Underpad included = TRUE, Underpad type left blank (material not named). 'IIC74 Padding' -&gt; IIC rating 74; no STC printed. Pieces per box not printed for the 10mm line - 8 assumed from the 8-plank cartons on the sister lines; verify. Waterproof left BLANK ('Aqua Protect'). COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF249" t="inlineStr">
@@ -29456,7 +29456,7 @@
       </c>
       <c r="BC250" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANLAM - Inspiration - Lamdura 10mm AC4 - Wood Collection IIC74 Paddin". Inhaus Inspiration - Lamdura 10mm AC4 'Aqua Protect', MegaLoc, imported from Germany. 50.59" (1285mm) x 7.56 in (192mm), '8mm +2mm (Core Plus Pad)' -&gt; Thickness 10mm total, Underpad included = TRUE, Underpad type left blank (material not named). 'IIC74 Padding' -&gt; IIC rating 74; no STC printed. Pieces per box not printed for the 10mm line - 8 assumed from the 8-plank cartons on the sister lines; verify. Waterproof left BLANK ('Aqua Protect'). COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANLAM - Inspiration - Lamdura 10mm AC4 - Wood Collection IIC74 Paddin". Inhaus Inspiration - Lamdura 10mm AC4 'Aqua Protect', MegaLoc, imported from Germany. 50.59" (1285mm) x 7.56 in (192mm), '8mm +2mm (Core Plus Pad)' -&gt; Thickness 10mm total, Underpad included = TRUE, Underpad type left blank (material not named). 'IIC74 Padding' -&gt; IIC rating 74; no STC printed. Pieces per box not printed for the 10mm line - 8 assumed from the 8-plank cartons on the sister lines; verify. Waterproof left BLANK ('Aqua Protect'). COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF250" t="inlineStr">
@@ -29584,7 +29584,7 @@
       </c>
       <c r="BC251" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANLAM - Inspiration - Lamdura 10mm AC4 - Wood Collection IIC74 Paddin". Inhaus Inspiration - Lamdura 10mm AC4 'Aqua Protect', MegaLoc, imported from Germany. 50.59" (1285mm) x 7.56 in (192mm), '8mm +2mm (Core Plus Pad)' -&gt; Thickness 10mm total, Underpad included = TRUE, Underpad type left blank (material not named). 'IIC74 Padding' -&gt; IIC rating 74; no STC printed. Pieces per box not printed for the 10mm line - 8 assumed from the 8-plank cartons on the sister lines; verify. Waterproof left BLANK ('Aqua Protect'). COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANLAM - Inspiration - Lamdura 10mm AC4 - Wood Collection IIC74 Paddin". Inhaus Inspiration - Lamdura 10mm AC4 'Aqua Protect', MegaLoc, imported from Germany. 50.59" (1285mm) x 7.56 in (192mm), '8mm +2mm (Core Plus Pad)' -&gt; Thickness 10mm total, Underpad included = TRUE, Underpad type left blank (material not named). 'IIC74 Padding' -&gt; IIC rating 74; no STC printed. Pieces per box not printed for the 10mm line - 8 assumed from the 8-plank cartons on the sister lines; verify. Waterproof left BLANK ('Aqua Protect'). COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF251" t="inlineStr">
@@ -29712,7 +29712,7 @@
       </c>
       <c r="BC252" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANLAM - Inspiration - Lamdura 10mm AC4 - Wood Collection IIC74 Paddin". Inhaus Inspiration - Lamdura 10mm AC4 'Aqua Protect', MegaLoc, imported from Germany. 50.59" (1285mm) x 7.56 in (192mm), '8mm +2mm (Core Plus Pad)' -&gt; Thickness 10mm total, Underpad included = TRUE, Underpad type left blank (material not named). 'IIC74 Padding' -&gt; IIC rating 74; no STC printed. Pieces per box not printed for the 10mm line - 8 assumed from the 8-plank cartons on the sister lines; verify. Waterproof left BLANK ('Aqua Protect'). COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANLAM - Inspiration - Lamdura 10mm AC4 - Wood Collection IIC74 Paddin". Inhaus Inspiration - Lamdura 10mm AC4 'Aqua Protect', MegaLoc, imported from Germany. 50.59" (1285mm) x 7.56 in (192mm), '8mm +2mm (Core Plus Pad)' -&gt; Thickness 10mm total, Underpad included = TRUE, Underpad type left blank (material not named). 'IIC74 Padding' -&gt; IIC rating 74; no STC printed. Pieces per box not printed for the 10mm line - 8 assumed from the 8-plank cartons on the sister lines; verify. Waterproof left BLANK ('Aqua Protect'). COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF252" t="inlineStr">
@@ -29785,7 +29785,7 @@
       </c>
       <c r="BC253" t="inlineStr">
         <is>
-          <t>** SPECIAL ORDER **, 8 ft. / piece. Sheet groups 'Reducer / T-Moulding' at $40.00 and 'Stairnose' at $48.50. Cross-supplier accessory markup applied -&gt; Retail $50.00/pc. 'Due to the fragile nature of the product all trims are final sale.' COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>** SPECIAL ORDER **, 8 ft. / piece. Sheet groups 'Reducer / T-Moulding' at $40.00 and 'Stairnose' at $48.50. Cross-supplier accessory markup applied -&gt; Retail $50.00/pc. 'Due to the fragile nature of the product all trims are final sale.' COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF253" t="inlineStr">
@@ -29858,7 +29858,7 @@
       </c>
       <c r="BC254" t="inlineStr">
         <is>
-          <t>** SPECIAL ORDER **, 8 ft. / piece. Sheet groups 'Reducer / T-Moulding' at $40.00 and 'Stairnose' at $48.50. Cross-supplier accessory markup applied -&gt; Retail $50.00/pc. 'Due to the fragile nature of the product all trims are final sale.' COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>** SPECIAL ORDER **, 8 ft. / piece. Sheet groups 'Reducer / T-Moulding' at $40.00 and 'Stairnose' at $48.50. Cross-supplier accessory markup applied -&gt; Retail $50.00/pc. 'Due to the fragile nature of the product all trims are final sale.' COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF254" t="inlineStr">
@@ -29931,7 +29931,7 @@
       </c>
       <c r="BC255" t="inlineStr">
         <is>
-          <t>** SPECIAL ORDER **, 8 ft. / piece. Sheet groups 'Reducer / T-Moulding' at $40.00 and 'Stairnose' at $48.50. Cross-supplier accessory markup applied -&gt; Retail $63.50/pc. 'Due to the fragile nature of the product all trims are final sale.' COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>** SPECIAL ORDER **, 8 ft. / piece. Sheet groups 'Reducer / T-Moulding' at $40.00 and 'Stairnose' at $48.50. Cross-supplier accessory markup applied -&gt; Retail $63.50/pc. 'Due to the fragile nature of the product all trims are final sale.' COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF255" t="inlineStr">
@@ -30030,7 +30030,7 @@
       </c>
       <c r="BC256" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANVIN - SONO - Eclipse - Stone Collection (Centennial Sandstone) 5.5m". AMBIGUOUS CATEGORY/MATERIAL: SONO Eclipse's core construction is not stated anywhere on the sheet (the sister SONO Landscape line says 'Ceramic Composite Core AC5', which matches no canonical Material type value). Category assigned on plank-vs-tile format only; Material type left BLANK and Waterproof left blank. Confirm the construction with Albert/supplier before import. Imported from Germany. DIMENSION AMBIGUITY: the only size printed in the SONO Eclipse block is '50.79" x 7.99"', which sits between the Stone-tile and Wood-plank sub-blocks. 25.37 sf/box / (50.79x7.99/144) = 9.0 planks, so that size was assigned to the Wood plank; the Stone tile's size is therefore NOT printed (25.55 sf/box / 12 tiles = 2.13 sf/tile, consistent with the 25.12" x 12.2" used on SONO Landscape). Width (in) left blank rather than guessed. One price cell ($3.99) spans the whole SONO Eclipse section. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANVIN - SONO - Eclipse - Stone Collection (Centennial Sandstone) 5.5m". AMBIGUOUS CATEGORY/MATERIAL: SONO Eclipse's core construction is not stated anywhere on the sheet (the sister SONO Landscape line says 'Ceramic Composite Core AC5', which matches no canonical Material type value). Category assigned on plank-vs-tile format only; Material type left BLANK and Waterproof left blank. Confirm the construction with Albert/supplier before import. Imported from Germany. DIMENSION AMBIGUITY: the only size printed in the SONO Eclipse block is '50.79" x 7.99"', which sits between the Stone-tile and Wood-plank sub-blocks. 25.37 sf/box / (50.79x7.99/144) = 9.0 planks, so that size was assigned to the Wood plank; the Stone tile's size is therefore NOT printed (25.55 sf/box / 12 tiles = 2.13 sf/tile, consistent with the 25.12" x 12.2" used on SONO Landscape). Width (in) left blank rather than guessed. One price cell ($3.99) spans the whole SONO Eclipse section. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF256" t="inlineStr">
@@ -30129,7 +30129,7 @@
       </c>
       <c r="BC257" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANVIN - SONO - Eclipse - Stone Collection (Pearl Travertine) 5.5mm | ". AMBIGUOUS CATEGORY/MATERIAL: SONO Eclipse's core construction is not stated anywhere on the sheet (the sister SONO Landscape line says 'Ceramic Composite Core AC5', which matches no canonical Material type value). Category assigned on plank-vs-tile format only; Material type left BLANK and Waterproof left blank. Confirm the construction with Albert/supplier before import. Imported from Germany. DIMENSION AMBIGUITY: the only size printed in the SONO Eclipse block is '50.79" x 7.99"', which sits between the Stone-tile and Wood-plank sub-blocks. 25.37 sf/box / (50.79x7.99/144) = 9.0 planks, so that size was assigned to the Wood plank; the Stone tile's size is therefore NOT printed (25.55 sf/box / 12 tiles = 2.13 sf/tile, consistent with the 25.12" x 12.2" used on SONO Landscape). Width (in) left blank rather than guessed. One price cell ($3.99) spans the whole SONO Eclipse section. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANVIN - SONO - Eclipse - Stone Collection (Pearl Travertine) 5.5mm | ". AMBIGUOUS CATEGORY/MATERIAL: SONO Eclipse's core construction is not stated anywhere on the sheet (the sister SONO Landscape line says 'Ceramic Composite Core AC5', which matches no canonical Material type value). Category assigned on plank-vs-tile format only; Material type left BLANK and Waterproof left blank. Confirm the construction with Albert/supplier before import. Imported from Germany. DIMENSION AMBIGUITY: the only size printed in the SONO Eclipse block is '50.79" x 7.99"', which sits between the Stone-tile and Wood-plank sub-blocks. 25.37 sf/box / (50.79x7.99/144) = 9.0 planks, so that size was assigned to the Wood plank; the Stone tile's size is therefore NOT printed (25.55 sf/box / 12 tiles = 2.13 sf/tile, consistent with the 25.12" x 12.2" used on SONO Landscape). Width (in) left blank rather than guessed. One price cell ($3.99) spans the whole SONO Eclipse section. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF257" t="inlineStr">
@@ -30228,7 +30228,7 @@
       </c>
       <c r="BC258" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANVIN - SONO - Eclipse - Stone Collection (Pepper Travertine)  | #534". AMBIGUOUS CATEGORY/MATERIAL: SONO Eclipse's core construction is not stated anywhere on the sheet (the sister SONO Landscape line says 'Ceramic Composite Core AC5', which matches no canonical Material type value). Category assigned on plank-vs-tile format only; Material type left BLANK and Waterproof left blank. Confirm the construction with Albert/supplier before import. Imported from Germany. DIMENSION AMBIGUITY: the only size printed in the SONO Eclipse block is '50.79" x 7.99"', which sits between the Stone-tile and Wood-plank sub-blocks. 25.37 sf/box / (50.79x7.99/144) = 9.0 planks, so that size was assigned to the Wood plank; the Stone tile's size is therefore NOT printed (25.55 sf/box / 12 tiles = 2.13 sf/tile, consistent with the 25.12" x 12.2" used on SONO Landscape). Width (in) left blank rather than guessed. One price cell ($3.99) spans the whole SONO Eclipse section. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANVIN - SONO - Eclipse - Stone Collection (Pepper Travertine)  | #534". AMBIGUOUS CATEGORY/MATERIAL: SONO Eclipse's core construction is not stated anywhere on the sheet (the sister SONO Landscape line says 'Ceramic Composite Core AC5', which matches no canonical Material type value). Category assigned on plank-vs-tile format only; Material type left BLANK and Waterproof left blank. Confirm the construction with Albert/supplier before import. Imported from Germany. DIMENSION AMBIGUITY: the only size printed in the SONO Eclipse block is '50.79" x 7.99"', which sits between the Stone-tile and Wood-plank sub-blocks. 25.37 sf/box / (50.79x7.99/144) = 9.0 planks, so that size was assigned to the Wood plank; the Stone tile's size is therefore NOT printed (25.55 sf/box / 12 tiles = 2.13 sf/tile, consistent with the 25.12" x 12.2" used on SONO Landscape). Width (in) left blank rather than guessed. One price cell ($3.99) spans the whole SONO Eclipse section. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF258" t="inlineStr">
@@ -30327,7 +30327,7 @@
       </c>
       <c r="BC259" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANVIN - SONO - Eclipse - Stone Collection (Reposado Carrara) 5.5mm | ". AMBIGUOUS CATEGORY/MATERIAL: SONO Eclipse's core construction is not stated anywhere on the sheet (the sister SONO Landscape line says 'Ceramic Composite Core AC5', which matches no canonical Material type value). Category assigned on plank-vs-tile format only; Material type left BLANK and Waterproof left blank. Confirm the construction with Albert/supplier before import. Imported from Germany. DIMENSION AMBIGUITY: the only size printed in the SONO Eclipse block is '50.79" x 7.99"', which sits between the Stone-tile and Wood-plank sub-blocks. 25.37 sf/box / (50.79x7.99/144) = 9.0 planks, so that size was assigned to the Wood plank; the Stone tile's size is therefore NOT printed (25.55 sf/box / 12 tiles = 2.13 sf/tile, consistent with the 25.12" x 12.2" used on SONO Landscape). Width (in) left blank rather than guessed. One price cell ($3.99) spans the whole SONO Eclipse section. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANVIN - SONO - Eclipse - Stone Collection (Reposado Carrara) 5.5mm | ". AMBIGUOUS CATEGORY/MATERIAL: SONO Eclipse's core construction is not stated anywhere on the sheet (the sister SONO Landscape line says 'Ceramic Composite Core AC5', which matches no canonical Material type value). Category assigned on plank-vs-tile format only; Material type left BLANK and Waterproof left blank. Confirm the construction with Albert/supplier before import. Imported from Germany. DIMENSION AMBIGUITY: the only size printed in the SONO Eclipse block is '50.79" x 7.99"', which sits between the Stone-tile and Wood-plank sub-blocks. 25.37 sf/box / (50.79x7.99/144) = 9.0 planks, so that size was assigned to the Wood plank; the Stone tile's size is therefore NOT printed (25.55 sf/box / 12 tiles = 2.13 sf/tile, consistent with the 25.12" x 12.2" used on SONO Landscape). Width (in) left blank rather than guessed. One price cell ($3.99) spans the whole SONO Eclipse section. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF259" t="inlineStr">
@@ -30426,7 +30426,7 @@
       </c>
       <c r="BC260" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANVIN - SONO - Eclipse - Stone Collection (Sesame Sandstone) 5.5mm | ". AMBIGUOUS CATEGORY/MATERIAL: SONO Eclipse's core construction is not stated anywhere on the sheet (the sister SONO Landscape line says 'Ceramic Composite Core AC5', which matches no canonical Material type value). Category assigned on plank-vs-tile format only; Material type left BLANK and Waterproof left blank. Confirm the construction with Albert/supplier before import. Imported from Germany. DIMENSION AMBIGUITY: the only size printed in the SONO Eclipse block is '50.79" x 7.99"', which sits between the Stone-tile and Wood-plank sub-blocks. 25.37 sf/box / (50.79x7.99/144) = 9.0 planks, so that size was assigned to the Wood plank; the Stone tile's size is therefore NOT printed (25.55 sf/box / 12 tiles = 2.13 sf/tile, consistent with the 25.12" x 12.2" used on SONO Landscape). Width (in) left blank rather than guessed. One price cell ($3.99) spans the whole SONO Eclipse section. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANVIN - SONO - Eclipse - Stone Collection (Sesame Sandstone) 5.5mm | ". AMBIGUOUS CATEGORY/MATERIAL: SONO Eclipse's core construction is not stated anywhere on the sheet (the sister SONO Landscape line says 'Ceramic Composite Core AC5', which matches no canonical Material type value). Category assigned on plank-vs-tile format only; Material type left BLANK and Waterproof left blank. Confirm the construction with Albert/supplier before import. Imported from Germany. DIMENSION AMBIGUITY: the only size printed in the SONO Eclipse block is '50.79" x 7.99"', which sits between the Stone-tile and Wood-plank sub-blocks. 25.37 sf/box / (50.79x7.99/144) = 9.0 planks, so that size was assigned to the Wood plank; the Stone tile's size is therefore NOT printed (25.55 sf/box / 12 tiles = 2.13 sf/tile, consistent with the 25.12" x 12.2" used on SONO Landscape). Width (in) left blank rather than guessed. One price cell ($3.99) spans the whole SONO Eclipse section. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF260" t="inlineStr">
@@ -30525,7 +30525,7 @@
       </c>
       <c r="BC261" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANVIN - SONO - Eclipse - Stone Collection (Shadow Castle) 5.5mm | #53". AMBIGUOUS CATEGORY/MATERIAL: SONO Eclipse's core construction is not stated anywhere on the sheet (the sister SONO Landscape line says 'Ceramic Composite Core AC5', which matches no canonical Material type value). Category assigned on plank-vs-tile format only; Material type left BLANK and Waterproof left blank. Confirm the construction with Albert/supplier before import. Imported from Germany. DIMENSION AMBIGUITY: the only size printed in the SONO Eclipse block is '50.79" x 7.99"', which sits between the Stone-tile and Wood-plank sub-blocks. 25.37 sf/box / (50.79x7.99/144) = 9.0 planks, so that size was assigned to the Wood plank; the Stone tile's size is therefore NOT printed (25.55 sf/box / 12 tiles = 2.13 sf/tile, consistent with the 25.12" x 12.2" used on SONO Landscape). Width (in) left blank rather than guessed. One price cell ($3.99) spans the whole SONO Eclipse section. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANVIN - SONO - Eclipse - Stone Collection (Shadow Castle) 5.5mm | #53". AMBIGUOUS CATEGORY/MATERIAL: SONO Eclipse's core construction is not stated anywhere on the sheet (the sister SONO Landscape line says 'Ceramic Composite Core AC5', which matches no canonical Material type value). Category assigned on plank-vs-tile format only; Material type left BLANK and Waterproof left blank. Confirm the construction with Albert/supplier before import. Imported from Germany. DIMENSION AMBIGUITY: the only size printed in the SONO Eclipse block is '50.79" x 7.99"', which sits between the Stone-tile and Wood-plank sub-blocks. 25.37 sf/box / (50.79x7.99/144) = 9.0 planks, so that size was assigned to the Wood plank; the Stone tile's size is therefore NOT printed (25.55 sf/box / 12 tiles = 2.13 sf/tile, consistent with the 25.12" x 12.2" used on SONO Landscape). Width (in) left blank rather than guessed. One price cell ($3.99) spans the whole SONO Eclipse section. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF261" t="inlineStr">
@@ -30627,7 +30627,7 @@
       </c>
       <c r="BC262" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANVIN - SONO - Eclipse - Wood Collection (Baywest Oak) 5.5mm | #53452". AMBIGUOUS CATEGORY/MATERIAL: SONO Eclipse's core construction is not stated anywhere on the sheet (the sister SONO Landscape line says 'Ceramic Composite Core AC5', which matches no canonical Material type value). Category assigned on plank-vs-tile format only; Material type left BLANK and Waterproof left blank. Confirm the construction with Albert/supplier before import. Imported from Germany. 50.79" x 7.99"; pieces/box 9 derived from 25.37 sf/box / 2.818 sf per plank (not printed) - verify. One price cell ($3.99) spans the whole SONO Eclipse section. 'Heartlan Walnut' and 'Seawahed Oak' are the supplier's spellings, kept verbatim. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANVIN - SONO - Eclipse - Wood Collection (Baywest Oak) 5.5mm | #53452". AMBIGUOUS CATEGORY/MATERIAL: SONO Eclipse's core construction is not stated anywhere on the sheet (the sister SONO Landscape line says 'Ceramic Composite Core AC5', which matches no canonical Material type value). Category assigned on plank-vs-tile format only; Material type left BLANK and Waterproof left blank. Confirm the construction with Albert/supplier before import. Imported from Germany. 50.79" x 7.99"; pieces/box 9 derived from 25.37 sf/box / 2.818 sf per plank (not printed) - verify. One price cell ($3.99) spans the whole SONO Eclipse section. 'Heartlan Walnut' and 'Seawahed Oak' are the supplier's spellings, kept verbatim. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF262" t="inlineStr">
@@ -30729,7 +30729,7 @@
       </c>
       <c r="BC263" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANVIN - SONO - Eclipse - Wood Collection (Bower Oak) 5.5mm | #53462 |". AMBIGUOUS CATEGORY/MATERIAL: SONO Eclipse's core construction is not stated anywhere on the sheet (the sister SONO Landscape line says 'Ceramic Composite Core AC5', which matches no canonical Material type value). Category assigned on plank-vs-tile format only; Material type left BLANK and Waterproof left blank. Confirm the construction with Albert/supplier before import. Imported from Germany. 50.79" x 7.99"; pieces/box 9 derived from 25.37 sf/box / 2.818 sf per plank (not printed) - verify. One price cell ($3.99) spans the whole SONO Eclipse section. 'Heartlan Walnut' and 'Seawahed Oak' are the supplier's spellings, kept verbatim. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANVIN - SONO - Eclipse - Wood Collection (Bower Oak) 5.5mm | #53462 |". AMBIGUOUS CATEGORY/MATERIAL: SONO Eclipse's core construction is not stated anywhere on the sheet (the sister SONO Landscape line says 'Ceramic Composite Core AC5', which matches no canonical Material type value). Category assigned on plank-vs-tile format only; Material type left BLANK and Waterproof left blank. Confirm the construction with Albert/supplier before import. Imported from Germany. 50.79" x 7.99"; pieces/box 9 derived from 25.37 sf/box / 2.818 sf per plank (not printed) - verify. One price cell ($3.99) spans the whole SONO Eclipse section. 'Heartlan Walnut' and 'Seawahed Oak' are the supplier's spellings, kept verbatim. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF263" t="inlineStr">
@@ -30831,7 +30831,7 @@
       </c>
       <c r="BC264" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANVIN - SONO - Eclipse - Wood Collection (Canim Oak) 5.5mm | #53448 |". AMBIGUOUS CATEGORY/MATERIAL: SONO Eclipse's core construction is not stated anywhere on the sheet (the sister SONO Landscape line says 'Ceramic Composite Core AC5', which matches no canonical Material type value). Category assigned on plank-vs-tile format only; Material type left BLANK and Waterproof left blank. Confirm the construction with Albert/supplier before import. Imported from Germany. 50.79" x 7.99"; pieces/box 9 derived from 25.37 sf/box / 2.818 sf per plank (not printed) - verify. One price cell ($3.99) spans the whole SONO Eclipse section. 'Heartlan Walnut' and 'Seawahed Oak' are the supplier's spellings, kept verbatim. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANVIN - SONO - Eclipse - Wood Collection (Canim Oak) 5.5mm | #53448 |". AMBIGUOUS CATEGORY/MATERIAL: SONO Eclipse's core construction is not stated anywhere on the sheet (the sister SONO Landscape line says 'Ceramic Composite Core AC5', which matches no canonical Material type value). Category assigned on plank-vs-tile format only; Material type left BLANK and Waterproof left blank. Confirm the construction with Albert/supplier before import. Imported from Germany. 50.79" x 7.99"; pieces/box 9 derived from 25.37 sf/box / 2.818 sf per plank (not printed) - verify. One price cell ($3.99) spans the whole SONO Eclipse section. 'Heartlan Walnut' and 'Seawahed Oak' are the supplier's spellings, kept verbatim. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF264" t="inlineStr">
@@ -30933,7 +30933,7 @@
       </c>
       <c r="BC265" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANVIN - SONO - Eclipse - Wood Collection (Coffee Oak) 5.5mm | #53459 ". AMBIGUOUS CATEGORY/MATERIAL: SONO Eclipse's core construction is not stated anywhere on the sheet (the sister SONO Landscape line says 'Ceramic Composite Core AC5', which matches no canonical Material type value). Category assigned on plank-vs-tile format only; Material type left BLANK and Waterproof left blank. Confirm the construction with Albert/supplier before import. Imported from Germany. 50.79" x 7.99"; pieces/box 9 derived from 25.37 sf/box / 2.818 sf per plank (not printed) - verify. One price cell ($3.99) spans the whole SONO Eclipse section. 'Heartlan Walnut' and 'Seawahed Oak' are the supplier's spellings, kept verbatim. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANVIN - SONO - Eclipse - Wood Collection (Coffee Oak) 5.5mm | #53459 ". AMBIGUOUS CATEGORY/MATERIAL: SONO Eclipse's core construction is not stated anywhere on the sheet (the sister SONO Landscape line says 'Ceramic Composite Core AC5', which matches no canonical Material type value). Category assigned on plank-vs-tile format only; Material type left BLANK and Waterproof left blank. Confirm the construction with Albert/supplier before import. Imported from Germany. 50.79" x 7.99"; pieces/box 9 derived from 25.37 sf/box / 2.818 sf per plank (not printed) - verify. One price cell ($3.99) spans the whole SONO Eclipse section. 'Heartlan Walnut' and 'Seawahed Oak' are the supplier's spellings, kept verbatim. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF265" t="inlineStr">
@@ -31035,7 +31035,7 @@
       </c>
       <c r="BC266" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANVIN - SONO - Eclipse - Wood Collection (Forest Grove Oak) 5.5mm | #". AMBIGUOUS CATEGORY/MATERIAL: SONO Eclipse's core construction is not stated anywhere on the sheet (the sister SONO Landscape line says 'Ceramic Composite Core AC5', which matches no canonical Material type value). Category assigned on plank-vs-tile format only; Material type left BLANK and Waterproof left blank. Confirm the construction with Albert/supplier before import. Imported from Germany. 50.79" x 7.99"; pieces/box 9 derived from 25.37 sf/box / 2.818 sf per plank (not printed) - verify. One price cell ($3.99) spans the whole SONO Eclipse section. 'Heartlan Walnut' and 'Seawahed Oak' are the supplier's spellings, kept verbatim. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANVIN - SONO - Eclipse - Wood Collection (Forest Grove Oak) 5.5mm | #". AMBIGUOUS CATEGORY/MATERIAL: SONO Eclipse's core construction is not stated anywhere on the sheet (the sister SONO Landscape line says 'Ceramic Composite Core AC5', which matches no canonical Material type value). Category assigned on plank-vs-tile format only; Material type left BLANK and Waterproof left blank. Confirm the construction with Albert/supplier before import. Imported from Germany. 50.79" x 7.99"; pieces/box 9 derived from 25.37 sf/box / 2.818 sf per plank (not printed) - verify. One price cell ($3.99) spans the whole SONO Eclipse section. 'Heartlan Walnut' and 'Seawahed Oak' are the supplier's spellings, kept verbatim. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF266" t="inlineStr">
@@ -31137,7 +31137,7 @@
       </c>
       <c r="BC267" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANVIN - SONO - Eclipse - Wood Collection (Heartlan Walnut) 5.5mm | #5". AMBIGUOUS CATEGORY/MATERIAL: SONO Eclipse's core construction is not stated anywhere on the sheet (the sister SONO Landscape line says 'Ceramic Composite Core AC5', which matches no canonical Material type value). Category assigned on plank-vs-tile format only; Material type left BLANK and Waterproof left blank. Confirm the construction with Albert/supplier before import. Imported from Germany. 50.79" x 7.99"; pieces/box 9 derived from 25.37 sf/box / 2.818 sf per plank (not printed) - verify. One price cell ($3.99) spans the whole SONO Eclipse section. 'Heartlan Walnut' and 'Seawahed Oak' are the supplier's spellings, kept verbatim. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANVIN - SONO - Eclipse - Wood Collection (Heartlan Walnut) 5.5mm | #5". AMBIGUOUS CATEGORY/MATERIAL: SONO Eclipse's core construction is not stated anywhere on the sheet (the sister SONO Landscape line says 'Ceramic Composite Core AC5', which matches no canonical Material type value). Category assigned on plank-vs-tile format only; Material type left BLANK and Waterproof left blank. Confirm the construction with Albert/supplier before import. Imported from Germany. 50.79" x 7.99"; pieces/box 9 derived from 25.37 sf/box / 2.818 sf per plank (not printed) - verify. One price cell ($3.99) spans the whole SONO Eclipse section. 'Heartlan Walnut' and 'Seawahed Oak' are the supplier's spellings, kept verbatim. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF267" t="inlineStr">
@@ -31239,7 +31239,7 @@
       </c>
       <c r="BC268" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANVIN - SONO - Eclipse - Wood Collection (Jasper Oak) 5.5mm | #53460 ". AMBIGUOUS CATEGORY/MATERIAL: SONO Eclipse's core construction is not stated anywhere on the sheet (the sister SONO Landscape line says 'Ceramic Composite Core AC5', which matches no canonical Material type value). Category assigned on plank-vs-tile format only; Material type left BLANK and Waterproof left blank. Confirm the construction with Albert/supplier before import. Imported from Germany. 50.79" x 7.99"; pieces/box 9 derived from 25.37 sf/box / 2.818 sf per plank (not printed) - verify. One price cell ($3.99) spans the whole SONO Eclipse section. 'Heartlan Walnut' and 'Seawahed Oak' are the supplier's spellings, kept verbatim. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANVIN - SONO - Eclipse - Wood Collection (Jasper Oak) 5.5mm | #53460 ". AMBIGUOUS CATEGORY/MATERIAL: SONO Eclipse's core construction is not stated anywhere on the sheet (the sister SONO Landscape line says 'Ceramic Composite Core AC5', which matches no canonical Material type value). Category assigned on plank-vs-tile format only; Material type left BLANK and Waterproof left blank. Confirm the construction with Albert/supplier before import. Imported from Germany. 50.79" x 7.99"; pieces/box 9 derived from 25.37 sf/box / 2.818 sf per plank (not printed) - verify. One price cell ($3.99) spans the whole SONO Eclipse section. 'Heartlan Walnut' and 'Seawahed Oak' are the supplier's spellings, kept verbatim. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF268" t="inlineStr">
@@ -31341,7 +31341,7 @@
       </c>
       <c r="BC269" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANVIN - SONO - Eclipse - Wood Collection (Liberty Oak) 5.5mm | #53451". AMBIGUOUS CATEGORY/MATERIAL: SONO Eclipse's core construction is not stated anywhere on the sheet (the sister SONO Landscape line says 'Ceramic Composite Core AC5', which matches no canonical Material type value). Category assigned on plank-vs-tile format only; Material type left BLANK and Waterproof left blank. Confirm the construction with Albert/supplier before import. Imported from Germany. 50.79" x 7.99"; pieces/box 9 derived from 25.37 sf/box / 2.818 sf per plank (not printed) - verify. One price cell ($3.99) spans the whole SONO Eclipse section. 'Heartlan Walnut' and 'Seawahed Oak' are the supplier's spellings, kept verbatim. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANVIN - SONO - Eclipse - Wood Collection (Liberty Oak) 5.5mm | #53451". AMBIGUOUS CATEGORY/MATERIAL: SONO Eclipse's core construction is not stated anywhere on the sheet (the sister SONO Landscape line says 'Ceramic Composite Core AC5', which matches no canonical Material type value). Category assigned on plank-vs-tile format only; Material type left BLANK and Waterproof left blank. Confirm the construction with Albert/supplier before import. Imported from Germany. 50.79" x 7.99"; pieces/box 9 derived from 25.37 sf/box / 2.818 sf per plank (not printed) - verify. One price cell ($3.99) spans the whole SONO Eclipse section. 'Heartlan Walnut' and 'Seawahed Oak' are the supplier's spellings, kept verbatim. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF269" t="inlineStr">
@@ -31443,7 +31443,7 @@
       </c>
       <c r="BC270" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANVIN - SONO - Eclipse - Wood Collection (Riverview Oak) 5.5mm | #543". AMBIGUOUS CATEGORY/MATERIAL: SONO Eclipse's core construction is not stated anywhere on the sheet (the sister SONO Landscape line says 'Ceramic Composite Core AC5', which matches no canonical Material type value). Category assigned on plank-vs-tile format only; Material type left BLANK and Waterproof left blank. Confirm the construction with Albert/supplier before import. Imported from Germany. 50.79" x 7.99"; pieces/box 9 derived from 25.37 sf/box / 2.818 sf per plank (not printed) - verify. One price cell ($3.99) spans the whole SONO Eclipse section. 'Heartlan Walnut' and 'Seawahed Oak' are the supplier's spellings, kept verbatim. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANVIN - SONO - Eclipse - Wood Collection (Riverview Oak) 5.5mm | #543". AMBIGUOUS CATEGORY/MATERIAL: SONO Eclipse's core construction is not stated anywhere on the sheet (the sister SONO Landscape line says 'Ceramic Composite Core AC5', which matches no canonical Material type value). Category assigned on plank-vs-tile format only; Material type left BLANK and Waterproof left blank. Confirm the construction with Albert/supplier before import. Imported from Germany. 50.79" x 7.99"; pieces/box 9 derived from 25.37 sf/box / 2.818 sf per plank (not printed) - verify. One price cell ($3.99) spans the whole SONO Eclipse section. 'Heartlan Walnut' and 'Seawahed Oak' are the supplier's spellings, kept verbatim. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF270" t="inlineStr">
@@ -31545,7 +31545,7 @@
       </c>
       <c r="BC271" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANVIN - SONO - Eclipse - Wood Collection (Riviera) 5.5mm | #53449 |  ". AMBIGUOUS CATEGORY/MATERIAL: SONO Eclipse's core construction is not stated anywhere on the sheet (the sister SONO Landscape line says 'Ceramic Composite Core AC5', which matches no canonical Material type value). Category assigned on plank-vs-tile format only; Material type left BLANK and Waterproof left blank. Confirm the construction with Albert/supplier before import. Imported from Germany. 50.79" x 7.99"; pieces/box 9 derived from 25.37 sf/box / 2.818 sf per plank (not printed) - verify. One price cell ($3.99) spans the whole SONO Eclipse section. 'Heartlan Walnut' and 'Seawahed Oak' are the supplier's spellings, kept verbatim. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANVIN - SONO - Eclipse - Wood Collection (Riviera) 5.5mm | #53449 |  ". AMBIGUOUS CATEGORY/MATERIAL: SONO Eclipse's core construction is not stated anywhere on the sheet (the sister SONO Landscape line says 'Ceramic Composite Core AC5', which matches no canonical Material type value). Category assigned on plank-vs-tile format only; Material type left BLANK and Waterproof left blank. Confirm the construction with Albert/supplier before import. Imported from Germany. 50.79" x 7.99"; pieces/box 9 derived from 25.37 sf/box / 2.818 sf per plank (not printed) - verify. One price cell ($3.99) spans the whole SONO Eclipse section. 'Heartlan Walnut' and 'Seawahed Oak' are the supplier's spellings, kept verbatim. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF271" t="inlineStr">
@@ -31647,7 +31647,7 @@
       </c>
       <c r="BC272" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANVIN - SONO - Eclipse - Wood Collection (Saloon (Oak)) 5.5mm | #5344". AMBIGUOUS CATEGORY/MATERIAL: SONO Eclipse's core construction is not stated anywhere on the sheet (the sister SONO Landscape line says 'Ceramic Composite Core AC5', which matches no canonical Material type value). Category assigned on plank-vs-tile format only; Material type left BLANK and Waterproof left blank. Confirm the construction with Albert/supplier before import. Imported from Germany. 50.79" x 7.99"; pieces/box 9 derived from 25.37 sf/box / 2.818 sf per plank (not printed) - verify. One price cell ($3.99) spans the whole SONO Eclipse section. 'Heartlan Walnut' and 'Seawahed Oak' are the supplier's spellings, kept verbatim. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANVIN - SONO - Eclipse - Wood Collection (Saloon (Oak)) 5.5mm | #5344". AMBIGUOUS CATEGORY/MATERIAL: SONO Eclipse's core construction is not stated anywhere on the sheet (the sister SONO Landscape line says 'Ceramic Composite Core AC5', which matches no canonical Material type value). Category assigned on plank-vs-tile format only; Material type left BLANK and Waterproof left blank. Confirm the construction with Albert/supplier before import. Imported from Germany. 50.79" x 7.99"; pieces/box 9 derived from 25.37 sf/box / 2.818 sf per plank (not printed) - verify. One price cell ($3.99) spans the whole SONO Eclipse section. 'Heartlan Walnut' and 'Seawahed Oak' are the supplier's spellings, kept verbatim. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF272" t="inlineStr">
@@ -31749,7 +31749,7 @@
       </c>
       <c r="BC273" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANVIN - SONO - Eclipse - Wood Collection (Sandhill Oak) 5.5mm | #5344". AMBIGUOUS CATEGORY/MATERIAL: SONO Eclipse's core construction is not stated anywhere on the sheet (the sister SONO Landscape line says 'Ceramic Composite Core AC5', which matches no canonical Material type value). Category assigned on plank-vs-tile format only; Material type left BLANK and Waterproof left blank. Confirm the construction with Albert/supplier before import. Imported from Germany. 50.79" x 7.99"; pieces/box 9 derived from 25.37 sf/box / 2.818 sf per plank (not printed) - verify. One price cell ($3.99) spans the whole SONO Eclipse section. 'Heartlan Walnut' and 'Seawahed Oak' are the supplier's spellings, kept verbatim. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANVIN - SONO - Eclipse - Wood Collection (Sandhill Oak) 5.5mm | #5344". AMBIGUOUS CATEGORY/MATERIAL: SONO Eclipse's core construction is not stated anywhere on the sheet (the sister SONO Landscape line says 'Ceramic Composite Core AC5', which matches no canonical Material type value). Category assigned on plank-vs-tile format only; Material type left BLANK and Waterproof left blank. Confirm the construction with Albert/supplier before import. Imported from Germany. 50.79" x 7.99"; pieces/box 9 derived from 25.37 sf/box / 2.818 sf per plank (not printed) - verify. One price cell ($3.99) spans the whole SONO Eclipse section. 'Heartlan Walnut' and 'Seawahed Oak' are the supplier's spellings, kept verbatim. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF273" t="inlineStr">
@@ -31851,7 +31851,7 @@
       </c>
       <c r="BC274" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANVIN - SONO - Eclipse - Wood Collection (Santa Fe (Oak)) 5.5mm | #53". AMBIGUOUS CATEGORY/MATERIAL: SONO Eclipse's core construction is not stated anywhere on the sheet (the sister SONO Landscape line says 'Ceramic Composite Core AC5', which matches no canonical Material type value). Category assigned on plank-vs-tile format only; Material type left BLANK and Waterproof left blank. Confirm the construction with Albert/supplier before import. Imported from Germany. 50.79" x 7.99"; pieces/box 9 derived from 25.37 sf/box / 2.818 sf per plank (not printed) - verify. One price cell ($3.99) spans the whole SONO Eclipse section. 'Heartlan Walnut' and 'Seawahed Oak' are the supplier's spellings, kept verbatim. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANVIN - SONO - Eclipse - Wood Collection (Santa Fe (Oak)) 5.5mm | #53". AMBIGUOUS CATEGORY/MATERIAL: SONO Eclipse's core construction is not stated anywhere on the sheet (the sister SONO Landscape line says 'Ceramic Composite Core AC5', which matches no canonical Material type value). Category assigned on plank-vs-tile format only; Material type left BLANK and Waterproof left blank. Confirm the construction with Albert/supplier before import. Imported from Germany. 50.79" x 7.99"; pieces/box 9 derived from 25.37 sf/box / 2.818 sf per plank (not printed) - verify. One price cell ($3.99) spans the whole SONO Eclipse section. 'Heartlan Walnut' and 'Seawahed Oak' are the supplier's spellings, kept verbatim. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF274" t="inlineStr">
@@ -31953,7 +31953,7 @@
       </c>
       <c r="BC275" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANVIN - SONO - Eclipse - Wood Collection (Sea Washed Oak) 5.5mm | #53". AMBIGUOUS CATEGORY/MATERIAL: SONO Eclipse's core construction is not stated anywhere on the sheet (the sister SONO Landscape line says 'Ceramic Composite Core AC5', which matches no canonical Material type value). Category assigned on plank-vs-tile format only; Material type left BLANK and Waterproof left blank. Confirm the construction with Albert/supplier before import. Imported from Germany. 50.79" x 7.99"; pieces/box 9 derived from 25.37 sf/box / 2.818 sf per plank (not printed) - verify. One price cell ($3.99) spans the whole SONO Eclipse section. 'Heartlan Walnut' and 'Seawahed Oak' are the supplier's spellings, kept verbatim. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANVIN - SONO - Eclipse - Wood Collection (Sea Washed Oak) 5.5mm | #53". AMBIGUOUS CATEGORY/MATERIAL: SONO Eclipse's core construction is not stated anywhere on the sheet (the sister SONO Landscape line says 'Ceramic Composite Core AC5', which matches no canonical Material type value). Category assigned on plank-vs-tile format only; Material type left BLANK and Waterproof left blank. Confirm the construction with Albert/supplier before import. Imported from Germany. 50.79" x 7.99"; pieces/box 9 derived from 25.37 sf/box / 2.818 sf per plank (not printed) - verify. One price cell ($3.99) spans the whole SONO Eclipse section. 'Heartlan Walnut' and 'Seawahed Oak' are the supplier's spellings, kept verbatim. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF275" t="inlineStr">
@@ -32055,7 +32055,7 @@
       </c>
       <c r="BC276" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANVIN - SONO - Eclipse - Wood Collection (Sheridan Bay Oak) 5.5mm | #". AMBIGUOUS CATEGORY/MATERIAL: SONO Eclipse's core construction is not stated anywhere on the sheet (the sister SONO Landscape line says 'Ceramic Composite Core AC5', which matches no canonical Material type value). Category assigned on plank-vs-tile format only; Material type left BLANK and Waterproof left blank. Confirm the construction with Albert/supplier before import. Imported from Germany. 50.79" x 7.99"; pieces/box 9 derived from 25.37 sf/box / 2.818 sf per plank (not printed) - verify. One price cell ($3.99) spans the whole SONO Eclipse section. 'Heartlan Walnut' and 'Seawahed Oak' are the supplier's spellings, kept verbatim. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANVIN - SONO - Eclipse - Wood Collection (Sheridan Bay Oak) 5.5mm | #". AMBIGUOUS CATEGORY/MATERIAL: SONO Eclipse's core construction is not stated anywhere on the sheet (the sister SONO Landscape line says 'Ceramic Composite Core AC5', which matches no canonical Material type value). Category assigned on plank-vs-tile format only; Material type left BLANK and Waterproof left blank. Confirm the construction with Albert/supplier before import. Imported from Germany. 50.79" x 7.99"; pieces/box 9 derived from 25.37 sf/box / 2.818 sf per plank (not printed) - verify. One price cell ($3.99) spans the whole SONO Eclipse section. 'Heartlan Walnut' and 'Seawahed Oak' are the supplier's spellings, kept verbatim. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF276" t="inlineStr">
@@ -32157,7 +32157,7 @@
       </c>
       <c r="BC277" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANVIN - SONO - Eclipse - Wood Collection (Streamwashed Oak) 5.5mm | #". AMBIGUOUS CATEGORY/MATERIAL: SONO Eclipse's core construction is not stated anywhere on the sheet (the sister SONO Landscape line says 'Ceramic Composite Core AC5', which matches no canonical Material type value). Category assigned on plank-vs-tile format only; Material type left BLANK and Waterproof left blank. Confirm the construction with Albert/supplier before import. Imported from Germany. 50.79" x 7.99"; pieces/box 9 derived from 25.37 sf/box / 2.818 sf per plank (not printed) - verify. One price cell ($3.99) spans the whole SONO Eclipse section. 'Heartlan Walnut' and 'Seawahed Oak' are the supplier's spellings, kept verbatim. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANVIN - SONO - Eclipse - Wood Collection (Streamwashed Oak) 5.5mm | #". AMBIGUOUS CATEGORY/MATERIAL: SONO Eclipse's core construction is not stated anywhere on the sheet (the sister SONO Landscape line says 'Ceramic Composite Core AC5', which matches no canonical Material type value). Category assigned on plank-vs-tile format only; Material type left BLANK and Waterproof left blank. Confirm the construction with Albert/supplier before import. Imported from Germany. 50.79" x 7.99"; pieces/box 9 derived from 25.37 sf/box / 2.818 sf per plank (not printed) - verify. One price cell ($3.99) spans the whole SONO Eclipse section. 'Heartlan Walnut' and 'Seawahed Oak' are the supplier's spellings, kept verbatim. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF277" t="inlineStr">
@@ -32259,7 +32259,7 @@
       </c>
       <c r="BC278" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANVIN - SONO - Eclipse - Wood Collection (Sunwashed Oak) 5.5mm | #534". AMBIGUOUS CATEGORY/MATERIAL: SONO Eclipse's core construction is not stated anywhere on the sheet (the sister SONO Landscape line says 'Ceramic Composite Core AC5', which matches no canonical Material type value). Category assigned on plank-vs-tile format only; Material type left BLANK and Waterproof left blank. Confirm the construction with Albert/supplier before import. Imported from Germany. 50.79" x 7.99"; pieces/box 9 derived from 25.37 sf/box / 2.818 sf per plank (not printed) - verify. One price cell ($3.99) spans the whole SONO Eclipse section. 'Heartlan Walnut' and 'Seawahed Oak' are the supplier's spellings, kept verbatim. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANVIN - SONO - Eclipse - Wood Collection (Sunwashed Oak) 5.5mm | #534". AMBIGUOUS CATEGORY/MATERIAL: SONO Eclipse's core construction is not stated anywhere on the sheet (the sister SONO Landscape line says 'Ceramic Composite Core AC5', which matches no canonical Material type value). Category assigned on plank-vs-tile format only; Material type left BLANK and Waterproof left blank. Confirm the construction with Albert/supplier before import. Imported from Germany. 50.79" x 7.99"; pieces/box 9 derived from 25.37 sf/box / 2.818 sf per plank (not printed) - verify. One price cell ($3.99) spans the whole SONO Eclipse section. 'Heartlan Walnut' and 'Seawahed Oak' are the supplier's spellings, kept verbatim. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF278" t="inlineStr">
@@ -32361,7 +32361,7 @@
       </c>
       <c r="BC279" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANVIN - SONO - Eclipse - Wood Collection (Tobacco Oak) 5.5mm | #53454". AMBIGUOUS CATEGORY/MATERIAL: SONO Eclipse's core construction is not stated anywhere on the sheet (the sister SONO Landscape line says 'Ceramic Composite Core AC5', which matches no canonical Material type value). Category assigned on plank-vs-tile format only; Material type left BLANK and Waterproof left blank. Confirm the construction with Albert/supplier before import. Imported from Germany. 50.79" x 7.99"; pieces/box 9 derived from 25.37 sf/box / 2.818 sf per plank (not printed) - verify. One price cell ($3.99) spans the whole SONO Eclipse section. 'Heartlan Walnut' and 'Seawahed Oak' are the supplier's spellings, kept verbatim. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANVIN - SONO - Eclipse - Wood Collection (Tobacco Oak) 5.5mm | #53454". AMBIGUOUS CATEGORY/MATERIAL: SONO Eclipse's core construction is not stated anywhere on the sheet (the sister SONO Landscape line says 'Ceramic Composite Core AC5', which matches no canonical Material type value). Category assigned on plank-vs-tile format only; Material type left BLANK and Waterproof left blank. Confirm the construction with Albert/supplier before import. Imported from Germany. 50.79" x 7.99"; pieces/box 9 derived from 25.37 sf/box / 2.818 sf per plank (not printed) - verify. One price cell ($3.99) spans the whole SONO Eclipse section. 'Heartlan Walnut' and 'Seawahed Oak' are the supplier's spellings, kept verbatim. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF279" t="inlineStr">
@@ -32463,7 +32463,7 @@
       </c>
       <c r="BC280" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANVIN - SONO - Eclipse - Wood Collection (Trimble White Oak) 5.5mm | ". AMBIGUOUS CATEGORY/MATERIAL: SONO Eclipse's core construction is not stated anywhere on the sheet (the sister SONO Landscape line says 'Ceramic Composite Core AC5', which matches no canonical Material type value). Category assigned on plank-vs-tile format only; Material type left BLANK and Waterproof left blank. Confirm the construction with Albert/supplier before import. Imported from Germany. 50.79" x 7.99"; pieces/box 9 derived from 25.37 sf/box / 2.818 sf per plank (not printed) - verify. One price cell ($3.99) spans the whole SONO Eclipse section. 'Heartlan Walnut' and 'Seawahed Oak' are the supplier's spellings, kept verbatim. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANVIN - SONO - Eclipse - Wood Collection (Trimble White Oak) 5.5mm | ". AMBIGUOUS CATEGORY/MATERIAL: SONO Eclipse's core construction is not stated anywhere on the sheet (the sister SONO Landscape line says 'Ceramic Composite Core AC5', which matches no canonical Material type value). Category assigned on plank-vs-tile format only; Material type left BLANK and Waterproof left blank. Confirm the construction with Albert/supplier before import. Imported from Germany. 50.79" x 7.99"; pieces/box 9 derived from 25.37 sf/box / 2.818 sf per plank (not printed) - verify. One price cell ($3.99) spans the whole SONO Eclipse section. 'Heartlan Walnut' and 'Seawahed Oak' are the supplier's spellings, kept verbatim. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF280" t="inlineStr">
@@ -32565,7 +32565,7 @@
       </c>
       <c r="BC281" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANVIN - SONO - Eclipse - Wood Collection (Winter Oak) 5.5mm | #53445 ". AMBIGUOUS CATEGORY/MATERIAL: SONO Eclipse's core construction is not stated anywhere on the sheet (the sister SONO Landscape line says 'Ceramic Composite Core AC5', which matches no canonical Material type value). Category assigned on plank-vs-tile format only; Material type left BLANK and Waterproof left blank. Confirm the construction with Albert/supplier before import. Imported from Germany. 50.79" x 7.99"; pieces/box 9 derived from 25.37 sf/box / 2.818 sf per plank (not printed) - verify. One price cell ($3.99) spans the whole SONO Eclipse section. 'Heartlan Walnut' and 'Seawahed Oak' are the supplier's spellings, kept verbatim. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANVIN - SONO - Eclipse - Wood Collection (Winter Oak) 5.5mm | #53445 ". AMBIGUOUS CATEGORY/MATERIAL: SONO Eclipse's core construction is not stated anywhere on the sheet (the sister SONO Landscape line says 'Ceramic Composite Core AC5', which matches no canonical Material type value). Category assigned on plank-vs-tile format only; Material type left BLANK and Waterproof left blank. Confirm the construction with Albert/supplier before import. Imported from Germany. 50.79" x 7.99"; pieces/box 9 derived from 25.37 sf/box / 2.818 sf per plank (not printed) - verify. One price cell ($3.99) spans the whole SONO Eclipse section. 'Heartlan Walnut' and 'Seawahed Oak' are the supplier's spellings, kept verbatim. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF281" t="inlineStr">
@@ -32643,7 +32643,7 @@
       </c>
       <c r="BC282" t="inlineStr">
         <is>
-          <t>** SPECIAL ORDER **, 94" per piece, printed as 'T-Mold (Slim Trim)'. All three trim types share one $48.50 price cell. Cross-supplier accessory markup applied -&gt; Retail $58.50/pc. 'All SONO Moldings made in the USA', CARB P2 Certified, trims are final sale. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>** SPECIAL ORDER **, 94" per piece, printed as 'T-Mold (Slim Trim)'. All three trim types share one $48.50 price cell. Cross-supplier accessory markup applied -&gt; Retail $58.50/pc. 'All SONO Moldings made in the USA', CARB P2 Certified, trims are final sale. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF282" t="inlineStr">
@@ -32721,7 +32721,7 @@
       </c>
       <c r="BC283" t="inlineStr">
         <is>
-          <t>** SPECIAL ORDER **, 94" per piece, printed as 'Reducer (Slim Cap)'. All three trim types share one $48.50 price cell. Cross-supplier accessory markup applied -&gt; Retail $58.50/pc. 'All SONO Moldings made in the USA', CARB P2 Certified, trims are final sale. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>** SPECIAL ORDER **, 94" per piece, printed as 'Reducer (Slim Cap)'. All three trim types share one $48.50 price cell. Cross-supplier accessory markup applied -&gt; Retail $58.50/pc. 'All SONO Moldings made in the USA', CARB P2 Certified, trims are final sale. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF283" t="inlineStr">
@@ -32799,7 +32799,7 @@
       </c>
       <c r="BC284" t="inlineStr">
         <is>
-          <t>** SPECIAL ORDER **, 94" per piece, printed as 'Stairnose'. All three trim types share one $48.50 price cell. Cross-supplier accessory markup applied -&gt; Retail $63.50/pc. 'All SONO Moldings made in the USA', CARB P2 Certified, trims are final sale. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>** SPECIAL ORDER **, 94" per piece, printed as 'Stairnose'. All three trim types share one $48.50 price cell. Cross-supplier accessory markup applied -&gt; Retail $63.50/pc. 'All SONO Moldings made in the USA', CARB P2 Certified, trims are final sale. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF284" t="inlineStr">
@@ -32900,7 +32900,7 @@
       </c>
       <c r="BC285" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANVIN - SONO - Forest (Plank) -  (Opal Wood (Maple)) 4.5mm | #46100 |". AMBIGUOUS CATEGORY/MATERIAL: SONO Eclipse's core construction is not stated anywhere on the sheet (the sister SONO Landscape line says 'Ceramic Composite Core AC5', which matches no canonical Material type value). Category assigned on plank-vs-tile format only; Material type left BLANK and Waterproof left blank. Confirm the construction with Albert/supplier before import. Imported from Germany. Section header: '**PLEASE CALL TO CHECK AVAILABILITY**' and every colour is marked *DISCONTINUE ITEM*. Plank size not printed for this line (25.37 sf/box matches SONO Eclipse Wood) - Width left blank rather than inferred. Supplier marks this colour *DISCONTINUE ITEM* on the Aug 31 2026 list -&gt; Stock status = Discontinued, Active = FALSE. Confirm remaining stock before import. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANVIN - SONO - Forest (Plank) -  (Opal Wood (Maple)) 4.5mm | #46100 |". AMBIGUOUS CATEGORY/MATERIAL: SONO Eclipse's core construction is not stated anywhere on the sheet (the sister SONO Landscape line says 'Ceramic Composite Core AC5', which matches no canonical Material type value). Category assigned on plank-vs-tile format only; Material type left BLANK and Waterproof left blank. Confirm the construction with Albert/supplier before import. Imported from Germany. Section header: '**PLEASE CALL TO CHECK AVAILABILITY**' and every colour is marked *DISCONTINUE ITEM*. Plank size not printed for this line (25.37 sf/box matches SONO Eclipse Wood) - Width left blank rather than inferred. Supplier marks this colour *DISCONTINUE ITEM* on the Aug 31 2026 list -&gt; Stock status = Discontinued, Active = FALSE. Confirm remaining stock before import. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF285" t="inlineStr">
@@ -33001,7 +33001,7 @@
       </c>
       <c r="BC286" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANVIN - SONO - Forest (Plank) -  (Saddlehorn (Oak)) 4.5mm | #44298 | ". AMBIGUOUS CATEGORY/MATERIAL: SONO Eclipse's core construction is not stated anywhere on the sheet (the sister SONO Landscape line says 'Ceramic Composite Core AC5', which matches no canonical Material type value). Category assigned on plank-vs-tile format only; Material type left BLANK and Waterproof left blank. Confirm the construction with Albert/supplier before import. Imported from Germany. Section header: '**PLEASE CALL TO CHECK AVAILABILITY**' and every colour is marked *DISCONTINUE ITEM*. Plank size not printed for this line (25.37 sf/box matches SONO Eclipse Wood) - Width left blank rather than inferred. Supplier marks this colour *DISCONTINUE ITEM* on the Aug 31 2026 list -&gt; Stock status = Discontinued, Active = FALSE. Confirm remaining stock before import. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANVIN - SONO - Forest (Plank) -  (Saddlehorn (Oak)) 4.5mm | #44298 | ". AMBIGUOUS CATEGORY/MATERIAL: SONO Eclipse's core construction is not stated anywhere on the sheet (the sister SONO Landscape line says 'Ceramic Composite Core AC5', which matches no canonical Material type value). Category assigned on plank-vs-tile format only; Material type left BLANK and Waterproof left blank. Confirm the construction with Albert/supplier before import. Imported from Germany. Section header: '**PLEASE CALL TO CHECK AVAILABILITY**' and every colour is marked *DISCONTINUE ITEM*. Plank size not printed for this line (25.37 sf/box matches SONO Eclipse Wood) - Width left blank rather than inferred. Supplier marks this colour *DISCONTINUE ITEM* on the Aug 31 2026 list -&gt; Stock status = Discontinued, Active = FALSE. Confirm remaining stock before import. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF286" t="inlineStr">
@@ -33102,7 +33102,7 @@
       </c>
       <c r="BC287" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANVIN - SONO - Forest (Plank) -  (Heartland Walnut) 4.5mm | #44308 | ". AMBIGUOUS CATEGORY/MATERIAL: SONO Eclipse's core construction is not stated anywhere on the sheet (the sister SONO Landscape line says 'Ceramic Composite Core AC5', which matches no canonical Material type value). Category assigned on plank-vs-tile format only; Material type left BLANK and Waterproof left blank. Confirm the construction with Albert/supplier before import. Imported from Germany. Section header: '**PLEASE CALL TO CHECK AVAILABILITY**' and every colour is marked *DISCONTINUE ITEM*. Plank size not printed for this line (25.37 sf/box matches SONO Eclipse Wood) - Width left blank rather than inferred. Supplier marks this colour *DISCONTINUE ITEM* on the Aug 31 2026 list -&gt; Stock status = Discontinued, Active = FALSE. Confirm remaining stock before import. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANVIN - SONO - Forest (Plank) -  (Heartland Walnut) 4.5mm | #44308 | ". AMBIGUOUS CATEGORY/MATERIAL: SONO Eclipse's core construction is not stated anywhere on the sheet (the sister SONO Landscape line says 'Ceramic Composite Core AC5', which matches no canonical Material type value). Category assigned on plank-vs-tile format only; Material type left BLANK and Waterproof left blank. Confirm the construction with Albert/supplier before import. Imported from Germany. Section header: '**PLEASE CALL TO CHECK AVAILABILITY**' and every colour is marked *DISCONTINUE ITEM*. Plank size not printed for this line (25.37 sf/box matches SONO Eclipse Wood) - Width left blank rather than inferred. Supplier marks this colour *DISCONTINUE ITEM* on the Aug 31 2026 list -&gt; Stock status = Discontinued, Active = FALSE. Confirm remaining stock before import. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF287" t="inlineStr">
@@ -33209,7 +33209,7 @@
       </c>
       <c r="BC288" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANVIN - SONO - Landscape (Tile) -  (Light Castle)  | #46194 |  - 4.5m". SONO Landscape (Tile), imported from Germany. 4.5mm x 12.2" x 25.12". AMBIGUOUS MATERIAL: the sheet states 'Ceramic Composite Core AC5', which matches no canonical Material type option -&gt; left BLANK and recorded here. Category LVT assigned on tile format. Waterproof left blank. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANVIN - SONO - Landscape (Tile) -  (Light Castle)  | #46194 |  - 4.5m". SONO Landscape (Tile), imported from Germany. 4.5mm x 12.2" x 25.12". AMBIGUOUS MATERIAL: the sheet states 'Ceramic Composite Core AC5', which matches no canonical Material type option -&gt; left BLANK and recorded here. Category LVT assigned on tile format. Waterproof left blank. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF288" t="inlineStr">
@@ -33329,7 +33329,7 @@
       </c>
       <c r="BC289" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANENG - Boen Plank (5" Click Engineered Oak) - Oak (Arizona (10115872". BOEN - PLANK Engineered 'NEW CODES', imported from Norway. 9/16" x 5 7/16" x 86 5/8"; Thickness 14.29mm converted from 9/16". Species printed only as 'Oak'. The sheet prints TWO codes per colour (an alphanumeric article code and a numeric item number) - both stored in Supplier SKU in the combined form, per the Triforest dual-code precedent. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANENG - Boen Plank (5" Click Engineered Oak) - Oak (Arizona (10115872". BOEN - PLANK Engineered 'NEW CODES', imported from Norway. 9/16" x 5 7/16" x 86 5/8"; Thickness 14.29mm converted from 9/16". Species printed only as 'Oak'. The sheet prints TWO codes per colour (an alphanumeric article code and a numeric item number) - both stored in Supplier SKU in the combined form, per the Triforest dual-code precedent. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF289" t="inlineStr">
@@ -33449,7 +33449,7 @@
       </c>
       <c r="BC290" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANENG - Boen Plank (5" Click Engineered Oak) - Oak (California (10116". BOEN - PLANK Engineered 'NEW CODES', imported from Norway. 9/16" x 5 7/16" x 86 5/8"; Thickness 14.29mm converted from 9/16". Species printed only as 'Oak'. The sheet prints TWO codes per colour (an alphanumeric article code and a numeric item number) - both stored in Supplier SKU in the combined form, per the Triforest dual-code precedent. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANENG - Boen Plank (5" Click Engineered Oak) - Oak (California (10116". BOEN - PLANK Engineered 'NEW CODES', imported from Norway. 9/16" x 5 7/16" x 86 5/8"; Thickness 14.29mm converted from 9/16". Species printed only as 'Oak'. The sheet prints TWO codes per colour (an alphanumeric article code and a numeric item number) - both stored in Supplier SKU in the combined form, per the Triforest dual-code precedent. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF290" t="inlineStr">
@@ -33569,7 +33569,7 @@
       </c>
       <c r="BC291" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANENG - Boen Plank (5" Click Engineered Oak) - Oak (Cocoa (10115874))". BOEN - PLANK Engineered 'NEW CODES', imported from Norway. 9/16" x 5 7/16" x 86 5/8"; Thickness 14.29mm converted from 9/16". Species printed only as 'Oak'. The sheet prints TWO codes per colour (an alphanumeric article code and a numeric item number) - both stored in Supplier SKU in the combined form, per the Triforest dual-code precedent. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANENG - Boen Plank (5" Click Engineered Oak) - Oak (Cocoa (10115874))". BOEN - PLANK Engineered 'NEW CODES', imported from Norway. 9/16" x 5 7/16" x 86 5/8"; Thickness 14.29mm converted from 9/16". Species printed only as 'Oak'. The sheet prints TWO codes per colour (an alphanumeric article code and a numeric item number) - both stored in Supplier SKU in the combined form, per the Triforest dual-code precedent. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF291" t="inlineStr">
@@ -33689,7 +33689,7 @@
       </c>
       <c r="BC292" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANENG - Boen Plank (5" Click Engineered Oak) - Oak (Oregon (1016011))". BOEN - PLANK Engineered 'NEW CODES', imported from Norway. 9/16" x 5 7/16" x 86 5/8"; Thickness 14.29mm converted from 9/16". Species printed only as 'Oak'. The sheet prints TWO codes per colour (an alphanumeric article code and a numeric item number) - both stored in Supplier SKU in the combined form, per the Triforest dual-code precedent. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANENG - Boen Plank (5" Click Engineered Oak) - Oak (Oregon (1016011))". BOEN - PLANK Engineered 'NEW CODES', imported from Norway. 9/16" x 5 7/16" x 86 5/8"; Thickness 14.29mm converted from 9/16". Species printed only as 'Oak'. The sheet prints TWO codes per colour (an alphanumeric article code and a numeric item number) - both stored in Supplier SKU in the combined form, per the Triforest dual-code precedent. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF292" t="inlineStr">
@@ -33809,7 +33809,7 @@
       </c>
       <c r="BC293" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANENG - Boen Plank (5" Click Engineered Oak) - Oak (Vivo White (10115". BOEN - PLANK Engineered 'NEW CODES', imported from Norway. 9/16" x 5 7/16" x 86 5/8"; Thickness 14.29mm converted from 9/16". Species printed only as 'Oak'. The sheet prints TWO codes per colour (an alphanumeric article code and a numeric item number) - both stored in Supplier SKU in the combined form, per the Triforest dual-code precedent. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANENG - Boen Plank (5" Click Engineered Oak) - Oak (Vivo White (10115". BOEN - PLANK Engineered 'NEW CODES', imported from Norway. 9/16" x 5 7/16" x 86 5/8"; Thickness 14.29mm converted from 9/16". Species printed only as 'Oak'. The sheet prints TWO codes per colour (an alphanumeric article code and a numeric item number) - both stored in Supplier SKU in the combined form, per the Triforest dual-code precedent. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF293" t="inlineStr">
@@ -33929,7 +33929,7 @@
       </c>
       <c r="BC294" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANENG - Boen Plank (7" Click Engineered Oak) - Oak (California (10116". BOEN - PLANK Engineered 'NEW CODES', imported from Norway. 9/16" x 7 1/8" x 86 5/8", '(2.5 mm Top Layer-14mm Thick)'. Thickness taken from the stated 14mm (9/16" would be 14.29mm) - minor conflict noted. Dual codes stored combined. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANENG - Boen Plank (7" Click Engineered Oak) - Oak (California (10116". BOEN - PLANK Engineered 'NEW CODES', imported from Norway. 9/16" x 7 1/8" x 86 5/8", '(2.5 mm Top Layer-14mm Thick)'. Thickness taken from the stated 14mm (9/16" would be 14.29mm) - minor conflict noted. Dual codes stored combined. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF294" t="inlineStr">
@@ -34049,7 +34049,7 @@
       </c>
       <c r="BC295" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANENG - Boen Plank (7" Click Engineered Oak) - Oak (Oregon (10116853)". BOEN - PLANK Engineered 'NEW CODES', imported from Norway. 9/16" x 7 1/8" x 86 5/8", '(2.5 mm Top Layer-14mm Thick)'. Thickness taken from the stated 14mm (9/16" would be 14.29mm) - minor conflict noted. Dual codes stored combined. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANENG - Boen Plank (7" Click Engineered Oak) - Oak (Oregon (10116853)". BOEN - PLANK Engineered 'NEW CODES', imported from Norway. 9/16" x 7 1/8" x 86 5/8", '(2.5 mm Top Layer-14mm Thick)'. Thickness taken from the stated 14mm (9/16" would be 14.29mm) - minor conflict noted. Dual codes stored combined. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF295" t="inlineStr">
@@ -34169,7 +34169,7 @@
       </c>
       <c r="BC296" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANENG - Boen Live Pure - Oak (Alamo (10124404)) T&amp;G | #EA77VKFD |  - ". BOEN (LIVE PURE) - Engineered, imported from Norway. T&amp;G Engineered Oak, '(2.5 mm Top Layer-13mm Thick)', 9/16" x 5 7/16" x 86 5/8". CONFLICT: the header says 13mm thick but the printed size says 9/16" (14.29mm); the explicit mm figure was used. Dual codes stored combined. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANENG - Boen Live Pure - Oak (Alamo (10124404)) T&amp;G | #EA77VKFD |  - ". BOEN (LIVE PURE) - Engineered, imported from Norway. T&amp;G Engineered Oak, '(2.5 mm Top Layer-13mm Thick)', 9/16" x 5 7/16" x 86 5/8". CONFLICT: the header says 13mm thick but the printed size says 9/16" (14.29mm); the explicit mm figure was used. Dual codes stored combined. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF296" t="inlineStr">
@@ -34289,7 +34289,7 @@
       </c>
       <c r="BC297" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANENG - Boen Live Pure - Oak (Country (10141588)) T&amp;G | #EB4743FD |  ". BOEN (LIVE PURE) - Engineered, imported from Norway. T&amp;G Engineered Oak, '(2.5 mm Top Layer-13mm Thick)', 9/16" x 5 7/16" x 86 5/8". CONFLICT: the header says 13mm thick but the printed size says 9/16" (14.29mm); the explicit mm figure was used. Dual codes stored combined. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANENG - Boen Live Pure - Oak (Country (10141588)) T&amp;G | #EB4743FD |  ". BOEN (LIVE PURE) - Engineered, imported from Norway. T&amp;G Engineered Oak, '(2.5 mm Top Layer-13mm Thick)', 9/16" x 5 7/16" x 86 5/8". CONFLICT: the header says 13mm thick but the printed size says 9/16" (14.29mm); the explicit mm figure was used. Dual codes stored combined. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF297" t="inlineStr">
@@ -34409,7 +34409,7 @@
       </c>
       <c r="BC298" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANENG - Boen Live Pure - Oak (Horizon (10124392)) T&amp;G | #PC77V3FD |  ". BOEN (LIVE PURE) - Engineered, imported from Norway. T&amp;G Engineered Oak, '(2.5 mm Top Layer-13mm Thick)', 9/16" x 5 7/16" x 86 5/8". CONFLICT: the header says 13mm thick but the printed size says 9/16" (14.29mm); the explicit mm figure was used. Dual codes stored combined. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANENG - Boen Live Pure - Oak (Horizon (10124392)) T&amp;G | #PC77V3FD |  ". BOEN (LIVE PURE) - Engineered, imported from Norway. T&amp;G Engineered Oak, '(2.5 mm Top Layer-13mm Thick)', 9/16" x 5 7/16" x 86 5/8". CONFLICT: the header says 13mm thick but the printed size says 9/16" (14.29mm); the explicit mm figure was used. Dual codes stored combined. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF298" t="inlineStr">
@@ -34529,7 +34529,7 @@
       </c>
       <c r="BC299" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANENG - Boen Live Pure - Oak (Mild Grey (10124388)) T&amp;G | #PD77V3FD |". BOEN (LIVE PURE) - Engineered, imported from Norway. T&amp;G Engineered Oak, '(2.5 mm Top Layer-13mm Thick)', 9/16" x 5 7/16" x 86 5/8". CONFLICT: the header says 13mm thick but the printed size says 9/16" (14.29mm); the explicit mm figure was used. Dual codes stored combined. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANENG - Boen Live Pure - Oak (Mild Grey (10124388)) T&amp;G | #PD77V3FD |". BOEN (LIVE PURE) - Engineered, imported from Norway. T&amp;G Engineered Oak, '(2.5 mm Top Layer-13mm Thick)', 9/16" x 5 7/16" x 86 5/8". CONFLICT: the header says 13mm thick but the printed size says 9/16" (14.29mm); the explicit mm figure was used. Dual codes stored combined. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF299" t="inlineStr">
@@ -34649,7 +34649,7 @@
       </c>
       <c r="BC300" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANENG - Boen Live Pure - Oak (Natural (10125076)) T&amp;G | #EB77V3FD |  ". BOEN (LIVE PURE) - Engineered, imported from Norway. T&amp;G Engineered Oak, '(2.5 mm Top Layer-13mm Thick)', 9/16" x 5 7/16" x 86 5/8". CONFLICT: the header says 13mm thick but the printed size says 9/16" (14.29mm); the explicit mm figure was used. Dual codes stored combined. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANENG - Boen Live Pure - Oak (Natural (10125076)) T&amp;G | #EB77V3FD |  ". BOEN (LIVE PURE) - Engineered, imported from Norway. T&amp;G Engineered Oak, '(2.5 mm Top Layer-13mm Thick)', 9/16" x 5 7/16" x 86 5/8". CONFLICT: the header says 13mm thick but the printed size says 9/16" (14.29mm); the explicit mm figure was used. Dual codes stored combined. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF300" t="inlineStr">
@@ -34769,7 +34769,7 @@
       </c>
       <c r="BC301" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANENG - Boen Live Pure - Oak (Pale White (10138295)) T&amp;G | #PI77V6FD ". BOEN (LIVE PURE) - Engineered, imported from Norway. T&amp;G Engineered Oak, '(2.5 mm Top Layer-13mm Thick)', 9/16" x 5 7/16" x 86 5/8". CONFLICT: the header says 13mm thick but the printed size says 9/16" (14.29mm); the explicit mm figure was used. Dual codes stored combined. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANENG - Boen Live Pure - Oak (Pale White (10138295)) T&amp;G | #PI77V6FD ". BOEN (LIVE PURE) - Engineered, imported from Norway. T&amp;G Engineered Oak, '(2.5 mm Top Layer-13mm Thick)', 9/16" x 5 7/16" x 86 5/8". CONFLICT: the header says 13mm thick but the printed size says 9/16" (14.29mm); the explicit mm figure was used. Dual codes stored combined. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF301" t="inlineStr">
@@ -34889,7 +34889,7 @@
       </c>
       <c r="BC302" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANENG - Boen Live Pure - Oak (Warm Cotton (10124384)) T&amp;G | #PE77V3FD". BOEN (LIVE PURE) - Engineered, imported from Norway. T&amp;G Engineered Oak, '(2.5 mm Top Layer-13mm Thick)', 9/16" x 5 7/16" x 86 5/8". CONFLICT: the header says 13mm thick but the printed size says 9/16" (14.29mm); the explicit mm figure was used. Dual codes stored combined. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANENG - Boen Live Pure - Oak (Warm Cotton (10124384)) T&amp;G | #PE77V3FD". BOEN (LIVE PURE) - Engineered, imported from Norway. T&amp;G Engineered Oak, '(2.5 mm Top Layer-13mm Thick)', 9/16" x 5 7/16" x 86 5/8". CONFLICT: the header says 13mm thick but the printed size says 9/16" (14.29mm); the explicit mm figure was used. Dual codes stored combined. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF302" t="inlineStr">
@@ -35009,7 +35009,7 @@
       </c>
       <c r="BC303" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANENG - Boen Live Pure - Oak (White (10124406)) T&amp;G | #EB77V6FD |  - ". BOEN (LIVE PURE) - Engineered, imported from Norway. T&amp;G Engineered Oak, '(2.5 mm Top Layer-13mm Thick)', 9/16" x 5 7/16" x 86 5/8". CONFLICT: the header says 13mm thick but the printed size says 9/16" (14.29mm); the explicit mm figure was used. Dual codes stored combined. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANENG - Boen Live Pure - Oak (White (10124406)) T&amp;G | #EB77V6FD |  - ". BOEN (LIVE PURE) - Engineered, imported from Norway. T&amp;G Engineered Oak, '(2.5 mm Top Layer-13mm Thick)', 9/16" x 5 7/16" x 86 5/8". CONFLICT: the header says 13mm thick but the printed size says 9/16" (14.29mm); the explicit mm figure was used. Dual codes stored combined. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF303" t="inlineStr">
@@ -35134,7 +35134,7 @@
       </c>
       <c r="BC304" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANENG -  Boen Live Pure - Laquer - Oak (Grey Harmony (10144560)) T&amp;G ". BOEN (LIVE PURE-Lacquer) - Engineered, imported from Norway. Section header reads '**Discontinue item** (TBA)' -&gt; whole collection treated as Discontinued / Active FALSE, though a price ($6.99) is still printed; '(TBA)' suggests pricing is to be advised. Two 'Vivo-Natural' rows share a colour name and differ only by article code - the second is suffixed '(V5)' to keep names and handles unique. Confirm with supplier. Supplier marks this colour *DISCONTINUE ITEM* on the Aug 31 2026 list -&gt; Stock status = Discontinued, Active = FALSE. Confirm remaining stock before import. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANENG -  Boen Live Pure - Laquer - Oak (Grey Harmony (10144560)) T&amp;G ". BOEN (LIVE PURE-Lacquer) - Engineered, imported from Norway. Section header reads '**Discontinue item** (TBA)' -&gt; whole collection treated as Discontinued / Active FALSE, though a price ($6.99) is still printed; '(TBA)' suggests pricing is to be advised. Two 'Vivo-Natural' rows share a colour name and differ only by article code - the second is suffixed '(V5)' to keep names and handles unique. Confirm with supplier. Supplier marks this colour *DISCONTINUE ITEM* on the Aug 31 2026 list -&gt; Stock status = Discontinued, Active = FALSE. Confirm remaining stock before import. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF304" t="inlineStr">
@@ -35259,7 +35259,7 @@
       </c>
       <c r="BC305" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANENG -  Boen Live Pure - Laquer - Oak (Vivo-Natural (10143957)) T&amp;G ". BOEN (LIVE PURE-Lacquer) - Engineered, imported from Norway. Section header reads '**Discontinue item** (TBA)' -&gt; whole collection treated as Discontinued / Active FALSE, though a price ($6.99) is still printed; '(TBA)' suggests pricing is to be advised. Two 'Vivo-Natural' rows share a colour name and differ only by article code - the second is suffixed '(V5)' to keep names and handles unique. Confirm with supplier. Supplier marks this colour *DISCONTINUE ITEM* on the Aug 31 2026 list -&gt; Stock status = Discontinued, Active = FALSE. Confirm remaining stock before import. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANENG -  Boen Live Pure - Laquer - Oak (Vivo-Natural (10143957)) T&amp;G ". BOEN (LIVE PURE-Lacquer) - Engineered, imported from Norway. Section header reads '**Discontinue item** (TBA)' -&gt; whole collection treated as Discontinued / Active FALSE, though a price ($6.99) is still printed; '(TBA)' suggests pricing is to be advised. Two 'Vivo-Natural' rows share a colour name and differ only by article code - the second is suffixed '(V5)' to keep names and handles unique. Confirm with supplier. Supplier marks this colour *DISCONTINUE ITEM* on the Aug 31 2026 list -&gt; Stock status = Discontinued, Active = FALSE. Confirm remaining stock before import. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF305" t="inlineStr">
@@ -35384,7 +35384,7 @@
       </c>
       <c r="BC306" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANENG -  Boen Live Pure - Laquer - Oak (Vivo-Natural (Matte) 10037307". BOEN (LIVE PURE-Lacquer) - Engineered, imported from Norway. Section header reads '**Discontinue item** (TBA)' -&gt; whole collection treated as Discontinued / Active FALSE, though a price ($6.99) is still printed; '(TBA)' suggests pricing is to be advised. Two 'Vivo-Natural' rows share a colour name and differ only by article code - the second is suffixed '(V5)' to keep names and handles unique. Confirm with supplier. Supplier marks this colour *DISCONTINUE ITEM* on the Aug 31 2026 list -&gt; Stock status = Discontinued, Active = FALSE. Confirm remaining stock before import. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANENG -  Boen Live Pure - Laquer - Oak (Vivo-Natural (Matte) 10037307". BOEN (LIVE PURE-Lacquer) - Engineered, imported from Norway. Section header reads '**Discontinue item** (TBA)' -&gt; whole collection treated as Discontinued / Active FALSE, though a price ($6.99) is still printed; '(TBA)' suggests pricing is to be advised. Two 'Vivo-Natural' rows share a colour name and differ only by article code - the second is suffixed '(V5)' to keep names and handles unique. Confirm with supplier. Supplier marks this colour *DISCONTINUE ITEM* on the Aug 31 2026 list -&gt; Stock status = Discontinued, Active = FALSE. Confirm remaining stock before import. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF306" t="inlineStr">
@@ -35509,7 +35509,7 @@
       </c>
       <c r="BC307" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANENG -  Boen Live Pure - Laquer - Oak (Vivo White (10144571)) T&amp;G | ". BOEN (LIVE PURE-Lacquer) - Engineered, imported from Norway. Section header reads '**Discontinue item** (TBA)' -&gt; whole collection treated as Discontinued / Active FALSE, though a price ($6.99) is still printed; '(TBA)' suggests pricing is to be advised. Two 'Vivo-Natural' rows share a colour name and differ only by article code - the second is suffixed '(V5)' to keep names and handles unique. Confirm with supplier. Supplier marks this colour *DISCONTINUE ITEM* on the Aug 31 2026 list -&gt; Stock status = Discontinued, Active = FALSE. Confirm remaining stock before import. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by supplier code match to Lightspeed product "CANENG -  Boen Live Pure - Laquer - Oak (Vivo White (10144571)) T&amp;G | ". BOEN (LIVE PURE-Lacquer) - Engineered, imported from Norway. Section header reads '**Discontinue item** (TBA)' -&gt; whole collection treated as Discontinued / Active FALSE, though a price ($6.99) is still printed; '(TBA)' suggests pricing is to be advised. Two 'Vivo-Natural' rows share a colour name and differ only by article code - the second is suffixed '(V5)' to keep names and handles unique. Confirm with supplier. Supplier marks this colour *DISCONTINUE ITEM* on the Aug 31 2026 list -&gt; Stock status = Discontinued, Active = FALSE. Confirm remaining stock before import. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF307" t="inlineStr">
@@ -35626,7 +35626,7 @@
       </c>
       <c r="BC308" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Antikkwood (HS Click) - Oak (Grey Harbour) Click | #CAN.E.M.G". Antikkwood - Engineered Handscraped Click. 5" x 1/2" x RL. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Antikkwood (HS Click) - Oak (Grey Harbour) Click | #CAN.E.M.G". Antikkwood - Engineered Handscraped Click. 5" x 1/2" x RL. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF308" t="inlineStr">
@@ -35748,7 +35748,7 @@
       </c>
       <c r="BC309" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Antikkwood (T&amp;G) - Hickory (Night Owl) T&amp;G | #CAN.E.H.NigOwl.". Antikkwood - Engineered T&amp;G. Supplier marks this colour *DISCONTINUE ITEM* on the Aug 31 2026 list -&gt; Stock status = Discontinued, Active = FALSE. Confirm remaining stock before import. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Antikkwood (T&amp;G) - Hickory (Night Owl) T&amp;G | #CAN.E.H.NigOwl.". Antikkwood - Engineered T&amp;G. Supplier marks this colour *DISCONTINUE ITEM* on the Aug 31 2026 list -&gt; Stock status = Discontinued, Active = FALSE. Confirm remaining stock before import. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF309" t="inlineStr">
@@ -35870,7 +35870,7 @@
       </c>
       <c r="BC310" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Antikkwood (T&amp;G) - Oak (Barnboard) T&amp;G | #CAN.E.O.Bar.6 |  - ". Antikkwood - Engineered T&amp;G. Supplier marks this colour *DISCONTINUE ITEM* on the Aug 31 2026 list -&gt; Stock status = Discontinued, Active = FALSE. Confirm remaining stock before import. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Antikkwood (T&amp;G) - Oak (Barnboard) T&amp;G | #CAN.E.O.Bar.6 |  - ". Antikkwood - Engineered T&amp;G. Supplier marks this colour *DISCONTINUE ITEM* on the Aug 31 2026 list -&gt; Stock status = Discontinued, Active = FALSE. Confirm remaining stock before import. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF310" t="inlineStr">
@@ -35987,7 +35987,7 @@
       </c>
       <c r="BC311" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour variant match to Lightspeed product "CANENG - Antikkwood (T&amp;G) - Acacia (Smokey Brown) T&amp;G | #CAN.E.A.SmoBr". Antikkwood - Engineered T&amp;G. Finish not stated for this row. Supplier marks this colour *DISCONTINUE ITEM* on the Aug 31 2026 list -&gt; Stock status = Discontinued, Active = FALSE. Confirm remaining stock before import. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour variant match to Lightspeed product "CANENG - Antikkwood (T&amp;G) - Acacia (Smokey Brown) T&amp;G | #CAN.E.A.SmoBr". Antikkwood - Engineered T&amp;G. Finish not stated for this row. Supplier marks this colour *DISCONTINUE ITEM* on the Aug 31 2026 list -&gt; Stock status = Discontinued, Active = FALSE. Confirm remaining stock before import. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF311" t="inlineStr">
@@ -36099,7 +36099,7 @@
       </c>
       <c r="BC312" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Antikkwood (T&amp;G) - American Walnut (Natural) T&amp;G | #CAN.E.AW.". Antikkwood - Engineered T&amp;G. Finish not stated. Radiant heat left blank: the global rule names American Black Walnut; the sheet says 'American Walnut' only - confirm species before quoting radiant installs. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Antikkwood (T&amp;G) - American Walnut (Natural) T&amp;G | #CAN.E.AW.". Antikkwood - Engineered T&amp;G. Finish not stated. Radiant heat left blank: the global rule names American Black Walnut; the sheet says 'American Walnut' only - confirm species before quoting radiant installs. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF312" t="inlineStr">
@@ -36221,7 +36221,7 @@
       </c>
       <c r="BC313" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Antikkwood (T&amp;G) - Oak (Belgian Oak) T&amp;G | #CAN.E.O.BelOak.6 ". Antikkwood - Engineered T&amp;G. 6" x 9/16" x RL. 'Handscraped &amp; Distressed' has no word 'Grade' -&gt; finish language, Grade left blank. Box size varies per colour within this one price cell. Supplier marks this colour *DISCONTINUE ITEM* on the Aug 31 2026 list -&gt; Stock status = Discontinued, Active = FALSE. Confirm remaining stock before import. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Antikkwood (T&amp;G) - Oak (Belgian Oak) T&amp;G | #CAN.E.O.BelOak.6 ". Antikkwood - Engineered T&amp;G. 6" x 9/16" x RL. 'Handscraped &amp; Distressed' has no word 'Grade' -&gt; finish language, Grade left blank. Box size varies per colour within this one price cell. Supplier marks this colour *DISCONTINUE ITEM* on the Aug 31 2026 list -&gt; Stock status = Discontinued, Active = FALSE. Confirm remaining stock before import. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF313" t="inlineStr">
@@ -36343,7 +36343,7 @@
       </c>
       <c r="BC314" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Antikkwood (T&amp;G) - Oak (Driftwood) T&amp;G | #CAN.E.O.Dri.6 |  - ". Antikkwood - Engineered T&amp;G. 6" x 9/16" x RL. 'Handscraped &amp; Distressed' has no word 'Grade' -&gt; finish language, Grade left blank. Box size varies per colour within this one price cell. Supplier marks this colour *DISCONTINUE ITEM* on the Aug 31 2026 list -&gt; Stock status = Discontinued, Active = FALSE. Confirm remaining stock before import. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Antikkwood (T&amp;G) - Oak (Driftwood) T&amp;G | #CAN.E.O.Dri.6 |  - ". Antikkwood - Engineered T&amp;G. 6" x 9/16" x RL. 'Handscraped &amp; Distressed' has no word 'Grade' -&gt; finish language, Grade left blank. Box size varies per colour within this one price cell. Supplier marks this colour *DISCONTINUE ITEM* on the Aug 31 2026 list -&gt; Stock status = Discontinued, Active = FALSE. Confirm remaining stock before import. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF314" t="inlineStr">
@@ -36465,7 +36465,7 @@
       </c>
       <c r="BC315" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Antikkwood (T&amp;G) - Oak (Equestrian Grey) T&amp;G | #CAN.E.O.EquGr". Antikkwood - Engineered T&amp;G. 6" x 9/16" x RL. 'Handscraped &amp; Distressed' has no word 'Grade' -&gt; finish language, Grade left blank. Box size varies per colour within this one price cell. Supplier marks this colour *DISCONTINUE ITEM* on the Aug 31 2026 list -&gt; Stock status = Discontinued, Active = FALSE. Confirm remaining stock before import. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Antikkwood (T&amp;G) - Oak (Equestrian Grey) T&amp;G | #CAN.E.O.EquGr". Antikkwood - Engineered T&amp;G. 6" x 9/16" x RL. 'Handscraped &amp; Distressed' has no word 'Grade' -&gt; finish language, Grade left blank. Box size varies per colour within this one price cell. Supplier marks this colour *DISCONTINUE ITEM* on the Aug 31 2026 list -&gt; Stock status = Discontinued, Active = FALSE. Confirm remaining stock before import. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF315" t="inlineStr">
@@ -36587,7 +36587,7 @@
       </c>
       <c r="BC316" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Antikkwood (T&amp;G) - Oak (Stormy Sky) T&amp;G | #CAN.E.O.StoSky.6 |". Antikkwood - Engineered T&amp;G. 6" x 9/16" x RL. 'Handscraped &amp; Distressed' has no word 'Grade' -&gt; finish language, Grade left blank. Box size varies per colour within this one price cell. Supplier marks this colour *DISCONTINUE ITEM* on the Aug 31 2026 list -&gt; Stock status = Discontinued, Active = FALSE. Confirm remaining stock before import. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Antikkwood (T&amp;G) - Oak (Stormy Sky) T&amp;G | #CAN.E.O.StoSky.6 |". Antikkwood - Engineered T&amp;G. 6" x 9/16" x RL. 'Handscraped &amp; Distressed' has no word 'Grade' -&gt; finish language, Grade left blank. Box size varies per colour within this one price cell. Supplier marks this colour *DISCONTINUE ITEM* on the Aug 31 2026 list -&gt; Stock status = Discontinued, Active = FALSE. Confirm remaining stock before import. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF316" t="inlineStr">
@@ -36704,7 +36704,7 @@
       </c>
       <c r="BC317" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Nestwood (T&amp;G) - Oak (Eagle Nest) T&amp;G | #CAN.E.O.EagNes.5 |  ". Nestwood - Engineered T&amp;G, finished in Canada. The whole Nestwood section carries a SINGLE price cell ($3.49) vertically centred over all five sub-groups - read as one price for the section. Confirm; no per-sub-group prices are printed. 5" x 9/16" x RL. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Nestwood (T&amp;G) - Oak (Eagle Nest) T&amp;G | #CAN.E.O.EagNes.5 |  ". Nestwood - Engineered T&amp;G, finished in Canada. The whole Nestwood section carries a SINGLE price cell ($3.49) vertically centred over all five sub-groups - read as one price for the section. Confirm; no per-sub-group prices are printed. 5" x 9/16" x RL. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF317" t="inlineStr">
@@ -36821,7 +36821,7 @@
       </c>
       <c r="BC318" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Nestwood (T&amp;G) - Oak (Inox Oak) T&amp;G | #CAN.E.O.InoOak.5 |  - ". Nestwood - Engineered T&amp;G, finished in Canada. The whole Nestwood section carries a SINGLE price cell ($3.49) vertically centred over all five sub-groups - read as one price for the section. Confirm; no per-sub-group prices are printed. 5" x 9/16" x RL. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Nestwood (T&amp;G) - Oak (Inox Oak) T&amp;G | #CAN.E.O.InoOak.5 |  - ". Nestwood - Engineered T&amp;G, finished in Canada. The whole Nestwood section carries a SINGLE price cell ($3.49) vertically centred over all five sub-groups - read as one price for the section. Confirm; no per-sub-group prices are printed. 5" x 9/16" x RL. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF318" t="inlineStr">
@@ -36938,7 +36938,7 @@
       </c>
       <c r="BC319" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Nestwood (T&amp;G) - Oak (Midnight Oak) T&amp;G | #CAN.E.O.MidOak.6.1". Nestwood - Engineered T&amp;G, finished in Canada. The whole Nestwood section carries a SINGLE price cell ($3.49) vertically centred over all five sub-groups - read as one price for the section. Confirm; no per-sub-group prices are printed. 6" x 3/4" x RL. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Nestwood (T&amp;G) - Oak (Midnight Oak) T&amp;G | #CAN.E.O.MidOak.6.1". Nestwood - Engineered T&amp;G, finished in Canada. The whole Nestwood section carries a SINGLE price cell ($3.49) vertically centred over all five sub-groups - read as one price for the section. Confirm; no per-sub-group prices are printed. 6" x 3/4" x RL. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF319" t="inlineStr">
@@ -37060,7 +37060,7 @@
       </c>
       <c r="BC320" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Nestwood (T&amp;G) - Oak (Grey Cloud) T&amp;G | #CAN.E.O.GreClo.6.1 |". Nestwood - Engineered T&amp;G, finished in Canada. The whole Nestwood section carries a SINGLE price cell ($3.49) vertically centred over all five sub-groups - read as one price for the section. Confirm; no per-sub-group prices are printed. 6" x 9/16" x RL. Supplier marks this colour *DISCONTINUE ITEM* on the Aug 31 2026 list -&gt; Stock status = Discontinued, Active = FALSE. Confirm remaining stock before import. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Nestwood (T&amp;G) - Oak (Grey Cloud) T&amp;G | #CAN.E.O.GreClo.6.1 |". Nestwood - Engineered T&amp;G, finished in Canada. The whole Nestwood section carries a SINGLE price cell ($3.49) vertically centred over all five sub-groups - read as one price for the section. Confirm; no per-sub-group prices are printed. 6" x 9/16" x RL. Supplier marks this colour *DISCONTINUE ITEM* on the Aug 31 2026 list -&gt; Stock status = Discontinued, Active = FALSE. Confirm remaining stock before import. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF320" t="inlineStr">
@@ -37177,7 +37177,7 @@
       </c>
       <c r="BC321" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Nestwood (T&amp;G) - Maple (Cosmopolitan Grey) T&amp;G | #CAN.E.M.Cos". Nestwood - Engineered T&amp;G, finished in Canada. The whole Nestwood section carries a SINGLE price cell ($3.49) vertically centred over all five sub-groups - read as one price for the section. Confirm; no per-sub-group prices are printed. 5" x 9/16" x RL. Finish printed only for Cosmopolitan Grey ('Handscraped'). COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Nestwood (T&amp;G) - Maple (Cosmopolitan Grey) T&amp;G | #CAN.E.M.Cos". Nestwood - Engineered T&amp;G, finished in Canada. The whole Nestwood section carries a SINGLE price cell ($3.49) vertically centred over all five sub-groups - read as one price for the section. Confirm; no per-sub-group prices are printed. 5" x 9/16" x RL. Finish printed only for Cosmopolitan Grey ('Handscraped'). COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF321" t="inlineStr">
@@ -37294,7 +37294,7 @@
       </c>
       <c r="BC322" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Nestwood (T&amp;G) - Maple (Mystic Barrel) T&amp;G | #CAN.E.M.MysBar.". Nestwood - Engineered T&amp;G, finished in Canada. The whole Nestwood section carries a SINGLE price cell ($3.49) vertically centred over all five sub-groups - read as one price for the section. Confirm; no per-sub-group prices are printed. 5" x 9/16" x RL. Finish printed only for Cosmopolitan Grey ('Handscraped'). Supplier marks this colour *DISCONTINUE ITEM* on the Aug 31 2026 list -&gt; Stock status = Discontinued, Active = FALSE. Confirm remaining stock before import. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Nestwood (T&amp;G) - Maple (Mystic Barrel) T&amp;G | #CAN.E.M.MysBar.". Nestwood - Engineered T&amp;G, finished in Canada. The whole Nestwood section carries a SINGLE price cell ($3.49) vertically centred over all five sub-groups - read as one price for the section. Confirm; no per-sub-group prices are printed. 5" x 9/16" x RL. Finish printed only for Cosmopolitan Grey ('Handscraped'). Supplier marks this colour *DISCONTINUE ITEM* on the Aug 31 2026 list -&gt; Stock status = Discontinued, Active = FALSE. Confirm remaining stock before import. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF322" t="inlineStr">
@@ -37411,7 +37411,7 @@
       </c>
       <c r="BC323" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Nestwood (T&amp;G) - Maple (Amsterdam Maple) T&amp;G | #CAN.E.M.AmsMa". Nestwood - Engineered T&amp;G, finished in Canada. The whole Nestwood section carries a SINGLE price cell ($3.49) vertically centred over all five sub-groups - read as one price for the section. Confirm; no per-sub-group prices are printed. 6" x 9/16" x RL. Finish printed only for Amsterdam Maple ('Handscraped'). COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Nestwood (T&amp;G) - Maple (Amsterdam Maple) T&amp;G | #CAN.E.M.AmsMa". Nestwood - Engineered T&amp;G, finished in Canada. The whole Nestwood section carries a SINGLE price cell ($3.49) vertically centred over all five sub-groups - read as one price for the section. Confirm; no per-sub-group prices are printed. 6" x 9/16" x RL. Finish printed only for Amsterdam Maple ('Handscraped'). COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF323" t="inlineStr">
@@ -37523,7 +37523,7 @@
       </c>
       <c r="BC324" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Nestwood (T&amp;G) - Maple (Georgetown Grey) T&amp;G | #CAN.E.M.GeoGr". Nestwood - Engineered T&amp;G, finished in Canada. The whole Nestwood section carries a SINGLE price cell ($3.49) vertically centred over all five sub-groups - read as one price for the section. Confirm; no per-sub-group prices are printed. 6" x 9/16" x RL. Finish printed only for Amsterdam Maple ('Handscraped'). COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Nestwood (T&amp;G) - Maple (Georgetown Grey) T&amp;G | #CAN.E.M.GeoGr". Nestwood - Engineered T&amp;G, finished in Canada. The whole Nestwood section carries a SINGLE price cell ($3.49) vertically centred over all five sub-groups - read as one price for the section. Confirm; no per-sub-group prices are printed. 6" x 9/16" x RL. Finish printed only for Amsterdam Maple ('Handscraped'). COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF324" t="inlineStr">
@@ -37640,7 +37640,7 @@
       </c>
       <c r="BC325" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Unikkwood - Oak (Burnt Rafter) T&amp;G | #CAN.E.O.BurRaf.7 |  - 7". Unikkwood - Engineered - European Wide Plank - T&amp;G. 7" x 3/4" x RL. 'UV Oil' printed in the species column - recorded as a finish. Box size varies per colour. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Unikkwood - Oak (Burnt Rafter) T&amp;G | #CAN.E.O.BurRaf.7 |  - 7". Unikkwood - Engineered - European Wide Plank - T&amp;G. 7" x 3/4" x RL. 'UV Oil' printed in the species column - recorded as a finish. Box size varies per colour. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF325" t="inlineStr">
@@ -37757,7 +37757,7 @@
       </c>
       <c r="BC326" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Unikkwood - Oak (Saratoga Oak) T&amp;G | #CAN.E.O.SarOak.7 |  - 7". Unikkwood - Engineered - European Wide Plank - T&amp;G. 7" x 3/4" x RL. 'UV Oil' printed in the species column - recorded as a finish. Box size varies per colour. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Unikkwood - Oak (Saratoga Oak) T&amp;G | #CAN.E.O.SarOak.7 |  - 7". Unikkwood - Engineered - European Wide Plank - T&amp;G. 7" x 3/4" x RL. 'UV Oil' printed in the species column - recorded as a finish. Box size varies per colour. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF326" t="inlineStr">
@@ -37879,7 +37879,7 @@
       </c>
       <c r="BC327" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Unikkwood - Oak (Symphony Grey) T&amp;G | #CAN.E.O.SymGre.7 |  - ". Unikkwood - Engineered - European Wide Plank - T&amp;G. 7" x 3/4" x RL. 'UV Oil' printed in the species column - recorded as a finish. Box size varies per colour. Supplier marks this colour *DISCONTINUE ITEM* on the Aug 31 2026 list -&gt; Stock status = Discontinued, Active = FALSE. Confirm remaining stock before import. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANENG - Unikkwood - Oak (Symphony Grey) T&amp;G | #CAN.E.O.SymGre.7 |  - ". Unikkwood - Engineered - European Wide Plank - T&amp;G. 7" x 3/4" x RL. 'UV Oil' printed in the species column - recorded as a finish. Box size varies per colour. Supplier marks this colour *DISCONTINUE ITEM* on the Aug 31 2026 list -&gt; Stock status = Discontinued, Active = FALSE. Confirm remaining stock before import. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF327" t="inlineStr">
@@ -37996,7 +37996,7 @@
       </c>
       <c r="BC328" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANHAR - Handcraft - Acacia (Venice Sicily) T&amp;G | #CAN.H.A.VenSic.5.1 ". Handcraft - Solid T&amp;G. 5" x 3/4" x RL. Material type left blank (solid hardwood). Supplier marks *LIMITED STOCK -&gt; mapped to Low stock (the enum has no 'Limited'). COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANHAR - Handcraft - Acacia (Venice Sicily) T&amp;G | #CAN.H.A.VenSic.5.1 ". Handcraft - Solid T&amp;G. 5" x 3/4" x RL. Material type left blank (solid hardwood). Supplier marks *LIMITED STOCK -&gt; mapped to Low stock (the enum has no 'Limited'). COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF328" t="inlineStr">
@@ -38113,7 +38113,7 @@
       </c>
       <c r="BC329" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANHAR - Handcraft - Maple (Desert Husk) T&amp;G | #CAN.H.M.DesHus.5.1 |  ". Handcraft - Solid T&amp;G. 5" x 3/4" x RL. Material type left blank (solid hardwood). Supplier marks *LIMITED STOCK -&gt; mapped to Low stock (the enum has no 'Limited'). COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANHAR - Handcraft - Maple (Desert Husk) T&amp;G | #CAN.H.M.DesHus.5.1 |  ". Handcraft - Solid T&amp;G. 5" x 3/4" x RL. Material type left blank (solid hardwood). Supplier marks *LIMITED STOCK -&gt; mapped to Low stock (the enum has no 'Limited'). COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF329" t="inlineStr">
@@ -38230,7 +38230,7 @@
       </c>
       <c r="BC330" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANHAR - Handcraft - Maple (Toasted Sesame) T&amp;G | #CAN.H.M.ToaSes.5.1 ". Handcraft - Solid T&amp;G. 5" x 3/4" x RL. Material type left blank (solid hardwood). Supplier marks *LIMITED STOCK -&gt; mapped to Low stock (the enum has no 'Limited'). COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANHAR - Handcraft - Maple (Toasted Sesame) T&amp;G | #CAN.H.M.ToaSes.5.1 ". Handcraft - Solid T&amp;G. 5" x 3/4" x RL. Material type left blank (solid hardwood). Supplier marks *LIMITED STOCK -&gt; mapped to Low stock (the enum has no 'Limited'). COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF330" t="inlineStr">
@@ -38332,7 +38332,7 @@
       </c>
       <c r="BC331" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANVIN - LVT (Double Click System) -  (Country Birch)  | #CAN.V.0.CouB". Section header reads 'LVT (Luxury Vinyl Tile) - Double Click System' but both items are printed as 'Plank' at 6" x 48". CONFLICT FLAGGED: Category assigned LVP because the schema defines LVP/LVT by plank-vs-tile FORMAT and these are planks; the supplier's own section calls them LVT. Core construction not stated -&gt; Material type left BLANK, Waterproof left blank. One $1.89 price cell is centred between the two rows and read as covering both. 4.2mm plank. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANVIN - LVT (Double Click System) -  (Country Birch)  | #CAN.V.0.CouB". Section header reads 'LVT (Luxury Vinyl Tile) - Double Click System' but both items are printed as 'Plank' at 6" x 48". CONFLICT FLAGGED: Category assigned LVP because the schema defines LVP/LVT by plank-vs-tile FORMAT and these are planks; the supplier's own section calls them LVT. Core construction not stated -&gt; Material type left BLANK, Waterproof left blank. One $1.89 price cell is centred between the two rows and read as covering both. 4.2mm plank. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF331" t="inlineStr">
@@ -38434,7 +38434,7 @@
       </c>
       <c r="BC332" t="inlineStr">
         <is>
-          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANVIN - LVT (Double Click System) -  (Chestnut Pine)  | #CAN.V.0.CheP". Section header reads 'LVT (Luxury Vinyl Tile) - Double Click System' but both items are printed as 'Plank' at 6" x 48". CONFLICT FLAGGED: Category assigned LVP because the schema defines LVP/LVT by plank-vs-tile FORMAT and these are planks; the supplier's own section calls them LVT. Core construction not stated -&gt; Material type left BLANK, Waterproof left blank. One $1.89 price cell is centred between the two rows and read as covering both. 4mm plank. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>LS ID backfilled 2026-09-03 by colour+spec match to Lightspeed product "CANVIN - LVT (Double Click System) -  (Chestnut Pine)  | #CAN.V.0.CheP". Section header reads 'LVT (Luxury Vinyl Tile) - Double Click System' but both items are printed as 'Plank' at 6" x 48". CONFLICT FLAGGED: Category assigned LVP because the schema defines LVP/LVT by plank-vs-tile FORMAT and these are planks; the supplier's own section calls them LVT. Core construction not stated -&gt; Material type left BLANK, Waterproof left blank. One $1.89 price cell is centred between the two rows and read as covering both. 4mm plank. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF332" t="inlineStr">
@@ -38516,7 +38516,7 @@
       </c>
       <c r="BC333" t="inlineStr">
         <is>
-          <t>Underlayment, 3mm EVA foam, condo-approved, IIC 73 / STC 72, 200 sqft/roll. MARKUP TBD - the cross-supplier underlayment markup is Cost + $20 per piece/roll, but this item is priced per SQUARE FOOT ($0.22/sf; 200 sf/roll = $44.00/roll). Applying +$20 to a per-sf cost is nonsense, so Retail price/unit is left BLANK pending Albert's decision on the unit basis (FAW 'oak stair tread markup TBD' precedent). Box size (sf) holds the 200 sf roll size. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>Underlayment, 3mm EVA foam, condo-approved, IIC 73 / STC 72, 200 sqft/roll. MARKUP TBD - the cross-supplier underlayment markup is Cost + $20 per piece/roll, but this item is priced per SQUARE FOOT ($0.22/sf; 200 sf/roll = $44.00/roll). Applying +$20 to a per-sf cost is nonsense, so Retail price/unit is left BLANK pending Albert's decision on the unit basis (FAW 'oak stair tread markup TBD' precedent). Box size (sf) holds the 200 sf roll size. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF333" t="inlineStr">
@@ -38587,7 +38587,7 @@
       </c>
       <c r="BC334" t="inlineStr">
         <is>
-          <t>Underlayment, 2mm white residential underlay, 200 sqft/roll. MARKUP TBD - the cross-supplier underlayment markup is Cost + $20 per piece/roll, but this item is priced per SQUARE FOOT ($0.12/sf; 200 sf/roll = $24.00/roll). Applying +$20 to a per-sf cost is nonsense, so Retail price/unit is left BLANK pending Albert's decision on the unit basis (FAW 'oak stair tread markup TBD' precedent). Box size (sf) holds the 200 sf roll size. COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>Underlayment, 2mm white residential underlay, 200 sqft/roll. MARKUP TBD - the cross-supplier underlayment markup is Cost + $20 per piece/roll, but this item is priced per SQUARE FOOT ($0.12/sf; 200 sf/roll = $24.00/roll). Applying +$20 to a per-sf cost is nonsense, so Retail price/unit is left BLANK pending Albert's decision on the unit basis (FAW 'oak stair tread markup TBD' precedent). Box size (sf) holds the 200 sf roll size. COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF334" t="inlineStr">
@@ -38665,7 +38665,7 @@
       </c>
       <c r="BC335" t="inlineStr">
         <is>
-          <t>Custom Trims for Engineered Flooring, printed as 'T-moluld / Reducer'. UNIT FLAG: priced PER LINEAR FOOT ($35.00/lin.ft), not per piece; the cross-supplier accessory markup (+$10) is a per-piece rule and has been applied to the per-linear-foot cost as instructed -&gt; Retail $45.00/lin.ft. Confirm the unit basis with Albert. Approx. 15-20 business days, advance payment required, **Final Sale**. Sheet spells it 'T-moluld' (supplier typo). COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>Custom Trims for Engineered Flooring, printed as 'T-moluld / Reducer'. UNIT FLAG: priced PER LINEAR FOOT ($35.00/lin.ft), not per piece; the cross-supplier accessory markup (+$10) is a per-piece rule and has been applied to the per-linear-foot cost as instructed -&gt; Retail $45.00/lin.ft. Confirm the unit basis with Albert. Approx. 15-20 business days, advance payment required, **Final Sale**. Sheet spells it 'T-moluld' (supplier typo). COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF335" t="inlineStr">
@@ -38743,7 +38743,7 @@
       </c>
       <c r="BC336" t="inlineStr">
         <is>
-          <t>Custom Trims for Engineered Flooring, printed as 'T-moluld / Reducer'. UNIT FLAG: priced PER LINEAR FOOT ($35.00/lin.ft), not per piece; the cross-supplier accessory markup (+$10) is a per-piece rule and has been applied to the per-linear-foot cost as instructed -&gt; Retail $45.00/lin.ft. Confirm the unit basis with Albert. Approx. 15-20 business days, advance payment required, **Final Sale**. Sheet spells it 'T-moluld' (supplier typo). COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>Custom Trims for Engineered Flooring, printed as 'T-moluld / Reducer'. UNIT FLAG: priced PER LINEAR FOOT ($35.00/lin.ft), not per piece; the cross-supplier accessory markup (+$10) is a per-piece rule and has been applied to the per-linear-foot cost as instructed -&gt; Retail $45.00/lin.ft. Confirm the unit basis with Albert. Approx. 15-20 business days, advance payment required, **Final Sale**. Sheet spells it 'T-moluld' (supplier typo). COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF336" t="inlineStr">
@@ -38821,7 +38821,7 @@
       </c>
       <c r="BC337" t="inlineStr">
         <is>
-          <t>Custom Trims for Engineered Flooring, printed as 'Stairnose'. UNIT FLAG: priced PER LINEAR FOOT ($40.00/lin.ft), not per piece; the cross-supplier accessory markup (+$15) is a per-piece rule and has been applied to the per-linear-foot cost as instructed -&gt; Retail $55.00/lin.ft. Confirm the unit basis with Albert. Approx. 15-20 business days, advance payment required, **Final Sale**. Sheet spells it 'T-moluld' (supplier typo). COST BASIS UNCONFIRMED: the Aug 31 2026 Product Guide prints a single price with no statement of whether it is Titan's dealer cost or suggested retail. Printed price entered in Cost/unit as-is with no multiplier; Retail = Cost + $1.00. May need a dealer multiplier (cf. CIF x0.60, Olympia x0.564, Biyork MSRP-vs-Your-Price) before import - Albert to settle. NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
+          <t>Custom Trims for Engineered Flooring, printed as 'Stairnose'. UNIT FLAG: priced PER LINEAR FOOT ($40.00/lin.ft), not per piece; the cross-supplier accessory markup (+$15) is a per-piece rule and has been applied to the per-linear-foot cost as instructed -&gt; Retail $55.00/lin.ft. Confirm the unit basis with Albert. Approx. 15-20 business days, advance payment required, **Final Sale**. Sheet spells it 'T-moluld' (supplier typo). COST BASIS CONFIRMED (Albert, 2026-09-03): Canadian Standard prints Titan's cost per unit only - no MSRP, no multiplier. Printed price = Cost/unit as-is; Retail = Cost + $1.00 (schema default). NEW SUPPLIER - Canadian Standard has no subsection in bert-airtable-schema and no records/Supplier option in Airtable. Global rules only; supplier onboarding checklist still owed. SKU suffix 'CANS' and the LS handle scheme are unconfirmed (CANS implied by the skill's HWD-CANS-0001 format example).</t>
         </is>
       </c>
       <c r="BF337" t="inlineStr">

</xml_diff>